<commit_message>
Add Youhosty (Azienda B) data to comparison Excel
</commit_message>
<xml_diff>
--- a/Italianway_Analisi_Comparativa.xlsx
+++ b/Italianway_Analisi_Comparativa.xlsx
@@ -8,8 +8,9 @@
   </bookViews>
   <sheets>
     <sheet name="RIEPILOGO ITALIANWAY" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="CONFRONTO 3 AZIENDE" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="SCORECARD DECISIONALE" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="RIEPILOGO YOUHOSTY" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="CONFRONTO 3 AZIENDE" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="SCORECARD DECISIONALE" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="15">
+  <fonts count="19">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -107,8 +108,30 @@
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="001B3A5C"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001B3A5C"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00000000"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001B3A5C"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="18">
+  <fills count="23">
     <fill>
       <patternFill/>
     </fill>
@@ -195,8 +218,33 @@
         <fgColor rgb="00D5EEF0"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001B3A5C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00AED6F1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002980B9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D6EAF8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EBF5FB"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -218,11 +266,55 @@
         <color rgb="00B8B8B8"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00B8B8B8"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00B8B8B8"/>
+      </right>
+      <top style="thin">
+        <color rgb="00B8B8B8"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00B8B8B8"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00B8B8B8"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00B8B8B8"/>
+      </right>
+      <top style="thin">
+        <color rgb="00B8B8B8"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00B8B8B8"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -292,6 +384,38 @@
     </xf>
     <xf numFmtId="0" fontId="14" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="20" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="20" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="21" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="21" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="22" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="22" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -673,6 +797,9 @@
           <t>ITALIANWAY – ANALISI COMPLETA PER CONFRONTO PROPERTY MANAGER</t>
         </is>
       </c>
+      <c r="B1" s="24" t="n"/>
+      <c r="C1" s="24" t="n"/>
+      <c r="D1" s="25" t="n"/>
     </row>
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -680,6 +807,9 @@
           <t>Fonte: Contratto Mandato v.2025.1501 | Elenco Dotazioni mag-2025 | Polizza Assicurativa | Vademecum Allestimenti</t>
         </is>
       </c>
+      <c r="B2" s="24" t="n"/>
+      <c r="C2" s="24" t="n"/>
+      <c r="D2" s="25" t="n"/>
     </row>
     <row r="3" ht="24" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
@@ -709,6 +839,9 @@
           <t>💰 COMMISSIONI E COSTI</t>
         </is>
       </c>
+      <c r="B4" s="24" t="n"/>
+      <c r="C4" s="24" t="n"/>
+      <c r="D4" s="25" t="n"/>
     </row>
     <row r="5" ht="40" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
@@ -870,6 +1003,9 @@
           <t>📄 CONTRATTO E VINCOLI</t>
         </is>
       </c>
+      <c r="B12" s="24" t="n"/>
+      <c r="C12" s="24" t="n"/>
+      <c r="D12" s="25" t="n"/>
     </row>
     <row r="13" ht="40" customHeight="1">
       <c r="A13" s="5" t="inlineStr">
@@ -1031,6 +1167,9 @@
           <t>🛎️ SERVIZI INCLUSI NEL SISTEMA</t>
         </is>
       </c>
+      <c r="B20" s="24" t="n"/>
+      <c r="C20" s="24" t="n"/>
+      <c r="D20" s="25" t="n"/>
     </row>
     <row r="21" ht="40" customHeight="1">
       <c r="A21" s="5" t="inlineStr">
@@ -1236,6 +1375,9 @@
           <t>🛡️ COPERTURA ASSICURATIVA</t>
         </is>
       </c>
+      <c r="B30" s="24" t="n"/>
+      <c r="C30" s="24" t="n"/>
+      <c r="D30" s="25" t="n"/>
     </row>
     <row r="31" ht="40" customHeight="1">
       <c r="A31" s="5" t="inlineStr">
@@ -1433,6 +1575,9 @@
           <t>🏠 REQUISITI E DOTAZIONI OBBLIGATORIE</t>
         </is>
       </c>
+      <c r="B40" s="24" t="n"/>
+      <c r="C40" s="24" t="n"/>
+      <c r="D40" s="25" t="n"/>
     </row>
     <row r="41" ht="40" customHeight="1">
       <c r="A41" s="5" t="inlineStr">
@@ -1722,6 +1867,9 @@
           <t>🏢 STRUTTURA AZIENDALE</t>
         </is>
       </c>
+      <c r="B54" s="24" t="n"/>
+      <c r="C54" s="24" t="n"/>
+      <c r="D54" s="25" t="n"/>
     </row>
     <row r="55" ht="40" customHeight="1">
       <c r="A55" s="5" t="inlineStr">
@@ -1828,6 +1976,1836 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:D99"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="52" customWidth="1" min="2" max="2"/>
+    <col width="46" customWidth="1" min="3" max="3"/>
+    <col width="46" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="36" customHeight="1">
+      <c r="A1" s="26" t="inlineStr">
+        <is>
+          <t>YOUHOSTY (A.P.P.A. Srl) – ANALISI COMPLETA</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="27" t="inlineStr">
+        <is>
+          <t>Fonte: Contratto di Servizi v.2026 (A.P.P.A. Srl, Milano, P.IVA 09454690968) | Allegato 1 Scheda Comparazione</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="24" customHeight="1">
+      <c r="A3" s="28" t="inlineStr">
+        <is>
+          <t>CATEGORIA / VOCE</t>
+        </is>
+      </c>
+      <c r="B3" s="28" t="inlineStr">
+        <is>
+          <t>DETTAGLIO / VALORE</t>
+        </is>
+      </c>
+      <c r="C3" s="28" t="inlineStr">
+        <is>
+          <t>PRO (+)</t>
+        </is>
+      </c>
+      <c r="D3" s="28" t="inlineStr">
+        <is>
+          <t>CONTRO (–)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="29" t="inlineStr">
+        <is>
+          <t>🏢 STRUTTURA AZIENDALE</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="40" customHeight="1">
+      <c r="A5" s="30" t="inlineStr">
+        <is>
+          <t>Società</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>A.P.P.A. Srl – Milano, via G. Pezzi 2 | P.IVA 09454690968 | Cap. soc. €35.000 i.v.</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>Società operativa con sede a Milano</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>Capitale sociale basso (€35.000) rispetto a strutture più grandi</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="40" customHeight="1">
+      <c r="A6" s="31" t="inlineStr">
+        <is>
+          <t>Marchio</t>
+        </is>
+      </c>
+      <c r="B6" s="32" t="inlineStr">
+        <is>
+          <t>Youhosty (licenza d'uso su A.P.P.A. Srl)</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>Brand riconoscibile nel settore</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>Non è un brand di proprietà: cambio licenziatario possibile</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="40" customHeight="1">
+      <c r="A7" s="30" t="inlineStr">
+        <is>
+          <t>Modello operativo</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>Gestione diretta (non franchising)</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>Controllo qualità più uniforme rispetto a network di affiliati</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>Minore capillarità territoriale rispetto a reti franchise nazionali</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="40" customHeight="1">
+      <c r="A8" s="31" t="inlineStr">
+        <is>
+          <t>Cessione contratto</t>
+        </is>
+      </c>
+      <c r="B8" s="32" t="inlineStr">
+        <is>
+          <t>Youhosty può cedere il contratto a terzi analoghi senza consenso del cliente</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>Continuità del servizio garantita</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>Il cliente non ha potere di veto sul cambio di gestore</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="29" t="inlineStr">
+        <is>
+          <t>📦 STRUTTURA DEI PACCHETTI</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="40" customHeight="1">
+      <c r="A10" s="30" t="inlineStr">
+        <is>
+          <t>Tipi di pacchetto</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>4 opzioni: Online | All-Inclusive | Flexible | Superflex</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>Flessibilità di scelta in base alle esigenze del proprietario</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>Complessità nella comparazione: ogni pacchetto ha costi e vincoli molto diversi</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="40" customHeight="1">
+      <c r="A11" s="31" t="inlineStr">
+        <is>
+          <t>Pacchetto Online</t>
+        </is>
+      </c>
+      <c r="B11" s="32" t="inlineStr">
+        <is>
+          <t>Solo gestione digitale prenotazioni (no operatività offline)</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>Costo ridotto (10% breve termine)</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>Nessun supporto fisico; check-in e pulizie a carico del proprietario</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="40" customHeight="1">
+      <c r="A12" s="30" t="inlineStr">
+        <is>
+          <t>Pacchetto All-Inclusive</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>Gestione completa: foto, pratiche, check-in auto, pulizie, burocrazia</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>Servizio turnkey paragonabile a Italianway</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>Durata 24 mesi; recesso solo per forza maggiore: massima rigidità</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="40" customHeight="1">
+      <c r="A13" s="31" t="inlineStr">
+        <is>
+          <t>Pacchetto Flexible</t>
+        </is>
+      </c>
+      <c r="B13" s="32" t="inlineStr">
+        <is>
+          <t>Via di mezzo tra Online e All-Inclusive</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>Periodo di prova 8 mesi; maggiore flessibilità rispetto ad All-Inclusive</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>Commissioni più alte (18,5%); pratiche chiusura costose (€320)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="40" customHeight="1">
+      <c r="A14" s="30" t="inlineStr">
+        <is>
+          <t>Pacchetto Superflex</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>Per proprietari con requisito minimo notti garantite</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>Commissioni negoziabili per grandi volumi</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>Nessuna opzione di recesso standard; minimo notti obbligatorio</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="29" t="inlineStr">
+        <is>
+          <t>💶 SETUP FEE (una tantum, IVA esclusa – valori All-Inclusive con pagamento anticipato)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="40" customHeight="1">
+      <c r="A16" s="30" t="inlineStr">
+        <is>
+          <t>Servizio fotografico</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>€99 (standard) / €69* (pagamento anticipato 7gg)</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>Incluso nel pacchetto; prezzo contenuto rispetto al mercato</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>Costo esplicito a parte; in Italianway è incluso nel corrispettivo unico €600</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="40" customHeight="1">
+      <c r="A17" s="31" t="inlineStr">
+        <is>
+          <t>Pratiche casa vacanza (CAV)</t>
+        </is>
+      </c>
+      <c r="B17" s="32" t="inlineStr">
+        <is>
+          <t>€199 (standard) / €149* (ant.) – bolli inclusi</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>Bolli inclusi; prezzo competitivo</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>Obbligatorio solo per locazioni brevi; costo a carico del proprietario</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="40" customHeight="1">
+      <c r="A18" s="30" t="inlineStr">
+        <is>
+          <t>Check-up iniziale</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>€0 (All-Inclusive) | €49/€39* (Flexible) | €39* (Superflex)</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>Check-up gratuito con All-Inclusive</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>Costo esplicito negli altri pacchetti</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="40" customHeight="1">
+      <c r="A19" s="31" t="inlineStr">
+        <is>
+          <t>Installazione self check-in automatizzato</t>
+        </is>
+      </c>
+      <c r="B19" s="32" t="inlineStr">
+        <is>
+          <t>€0 (All-Inclusive) | €49/€39* (Flexible) | €39* (Superflex)</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>Incluso gratuitamente con All-Inclusive</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>Costo €250 per disinstallazione/voltura al recesso (tutti i pacchetti)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="40" customHeight="1">
+      <c r="A20" s="30" t="inlineStr">
+        <is>
+          <t>Adempimenti sicurezza (estintore+CO+kit PS)</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>€259 (standard) / €219* (ant.) – All-Inclusive</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>Gestione sicurezza delegata in noleggio+manutenzione</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>Importo non trascurabile; noleggio → non di proprietà del cliente</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="40" customHeight="1">
+      <c r="A21" s="31" t="inlineStr">
+        <is>
+          <t>Pulizie iniziali (facoltativo)</t>
+        </is>
+      </c>
+      <c r="B21" s="32" t="inlineStr">
+        <is>
+          <t>Mono €70 | Bilocale €100 | Trilocale €150 | Quadrilocale €200 | &gt;Plurilocale &gt;€250</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>Servizio opzionale; prezzi chiari e proporzionali</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>Facoltativo ma raccomandato per buone recensioni iniziali</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="40" customHeight="1">
+      <c r="A22" s="30" t="inlineStr">
+        <is>
+          <t>Aspirapolvere (facoltativo)</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>€69 standard / €49* (ant.)</t>
+        </is>
+      </c>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>Diventa proprietà del cliente dopo pagamento integrale</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="inlineStr">
+        <is>
+          <t>Solo 1 incluso; sostituzione successiva €60+IVA</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="40" customHeight="1">
+      <c r="A23" s="31" t="inlineStr">
+        <is>
+          <t>Alternativa setup fee</t>
+        </is>
+      </c>
+      <c r="B23" s="32" t="inlineStr">
+        <is>
+          <t>Nessuna setup fee + 2,5% aggiuntivo sulle commissioni di gestione</t>
+        </is>
+      </c>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>Opzione per chi non vuole anticipare costi</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>Il 2,5% extra si accumula nel tempo e può superare il costo della setup fee</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="20" customHeight="1">
+      <c r="A24" s="29" t="inlineStr">
+        <is>
+          <t>💰 COMMISSIONI – LOCAZIONI BREVI (% sul corrispettivo pagato dall'ospite, IVA esclusa)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="40" customHeight="1">
+      <c r="A25" s="30" t="inlineStr">
+        <is>
+          <t>Commissione All-Inclusive (1 immobile)</t>
+        </is>
+      </c>
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t>16,5% del corrispettivo ospite</t>
+        </is>
+      </c>
+      <c r="C25" s="7" t="inlineStr">
+        <is>
+          <t>Più bassa del 25% di Italianway (ma basi di calcolo diverse – vedi CONTRO)</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>Commissioni OTA vengono ANCHE addebitate separatamente al cliente → il netto è inferiore</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="40" customHeight="1">
+      <c r="A26" s="31" t="inlineStr">
+        <is>
+          <t>Commissione All-Inclusive (2-5 immobili)</t>
+        </is>
+      </c>
+      <c r="B26" s="32" t="inlineStr">
+        <is>
+          <t>13,9%</t>
+        </is>
+      </c>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>Economie di scala significative</t>
+        </is>
+      </c>
+      <c r="D26" s="32" t="inlineStr"/>
+    </row>
+    <row r="27" ht="40" customHeight="1">
+      <c r="A27" s="30" t="inlineStr">
+        <is>
+          <t>Commissione All-Inclusive (6-10 immobili)</t>
+        </is>
+      </c>
+      <c r="B27" s="6" t="inlineStr">
+        <is>
+          <t>12,9%</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr"/>
+      <c r="D27" s="6" t="inlineStr"/>
+    </row>
+    <row r="28" ht="40" customHeight="1">
+      <c r="A28" s="31" t="inlineStr">
+        <is>
+          <t>Commissione All-Inclusive (+11 immobili)</t>
+        </is>
+      </c>
+      <c r="B28" s="32" t="inlineStr">
+        <is>
+          <t>11,9%</t>
+        </is>
+      </c>
+      <c r="C28" s="7" t="inlineStr">
+        <is>
+          <t>Molto competitivo per portfolio grandi</t>
+        </is>
+      </c>
+      <c r="D28" s="32" t="inlineStr"/>
+    </row>
+    <row r="29" ht="40" customHeight="1">
+      <c r="A29" s="30" t="inlineStr">
+        <is>
+          <t>Commissione Online (1 immobile)</t>
+        </is>
+      </c>
+      <c r="B29" s="6" t="inlineStr">
+        <is>
+          <t>10%</t>
+        </is>
+      </c>
+      <c r="C29" s="7" t="inlineStr">
+        <is>
+          <t>La più bassa del mercato per chi gestisce operatività in proprio</t>
+        </is>
+      </c>
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>No servizi offline: check-in, pulizie, burocrazia a carico del proprietario</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="40" customHeight="1">
+      <c r="A30" s="31" t="inlineStr">
+        <is>
+          <t>Commissione Flexible (1 immobile)</t>
+        </is>
+      </c>
+      <c r="B30" s="32" t="inlineStr">
+        <is>
+          <t>18,5%</t>
+        </is>
+      </c>
+      <c r="C30" s="7" t="inlineStr">
+        <is>
+          <t>Periodo di prova 8 mesi</t>
+        </is>
+      </c>
+      <c r="D30" s="8" t="inlineStr">
+        <is>
+          <t>Commissione alta; pratiche chiusura €320</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="40" customHeight="1">
+      <c r="A31" s="30" t="inlineStr">
+        <is>
+          <t>Commissione Superflex (1 immobile)</t>
+        </is>
+      </c>
+      <c r="B31" s="6" t="inlineStr">
+        <is>
+          <t>24,5%</t>
+        </is>
+      </c>
+      <c r="C31" s="6" t="inlineStr"/>
+      <c r="D31" s="8" t="inlineStr">
+        <is>
+          <t>La più costosa; senso solo per altissimi volumi garantiti</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="40" customHeight="1">
+      <c r="A32" s="31" t="inlineStr">
+        <is>
+          <t>Commissione OTA (Airbnb, Booking, ecc.)</t>
+        </is>
+      </c>
+      <c r="B32" s="32" t="inlineStr">
+        <is>
+          <t>Anticipata da Youhosty e ADDEBITATA al cliente al netto IVA</t>
+        </is>
+      </c>
+      <c r="C32" s="7" t="inlineStr">
+        <is>
+          <t>Il cliente non anticipa le OTA</t>
+        </is>
+      </c>
+      <c r="D32" s="8" t="inlineStr">
+        <is>
+          <t>Si somma alla commissione Youhosty: costo totale effettivo più alto del dichiarato</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="20" customHeight="1">
+      <c r="A33" s="29" t="inlineStr">
+        <is>
+          <t>💰 COMMISSIONI – LOCAZIONI MEDIO/LUNGO TERMINE</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="40" customHeight="1">
+      <c r="A34" s="30" t="inlineStr">
+        <is>
+          <t>A canone libero – All-Inclusive</t>
+        </is>
+      </c>
+      <c r="B34" s="6" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="C34" s="7" t="inlineStr">
+        <is>
+          <t>Nessuna commissione per il gestore se non richiesta garanzia</t>
+        </is>
+      </c>
+      <c r="D34" s="8" t="inlineStr">
+        <is>
+          <t>Solo se scelto All-Inclusive o Online</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="40" customHeight="1">
+      <c r="A35" s="31" t="inlineStr">
+        <is>
+          <t>A canone concordato – All-Inclusive</t>
+        </is>
+      </c>
+      <c r="B35" s="32" t="inlineStr">
+        <is>
+          <t>4% del corrispettivo ospite</t>
+        </is>
+      </c>
+      <c r="C35" s="32" t="inlineStr"/>
+      <c r="D35" s="32" t="inlineStr"/>
+    </row>
+    <row r="36" ht="40" customHeight="1">
+      <c r="A36" s="30" t="inlineStr">
+        <is>
+          <t>A canone garantito – All-Inclusive</t>
+        </is>
+      </c>
+      <c r="B36" s="6" t="inlineStr">
+        <is>
+          <t>5% del corrispettivo ospite</t>
+        </is>
+      </c>
+      <c r="C36" s="7" t="inlineStr">
+        <is>
+          <t>Canone garantito disponibile (Allegato 3)</t>
+        </is>
+      </c>
+      <c r="D36" s="8" t="inlineStr">
+        <is>
+          <t>Il canone garantito ha costo aggiuntivo ed è regolato da allegato separato</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="40" customHeight="1">
+      <c r="A37" s="31" t="inlineStr">
+        <is>
+          <t>Variazione canone medio-lungo termine</t>
+        </is>
+      </c>
+      <c r="B37" s="32" t="inlineStr">
+        <is>
+          <t>Youhosty può variare il canone fino a +10% senza consenso cliente</t>
+        </is>
+      </c>
+      <c r="C37" s="7" t="inlineStr">
+        <is>
+          <t>Flessibilità commerciale per massimizzare l'affittabilità</t>
+        </is>
+      </c>
+      <c r="D37" s="8" t="inlineStr">
+        <is>
+          <t>Il proprietario non controlla il prezzo di listino del proprio immobile</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="40" customHeight="1">
+      <c r="A38" s="30" t="inlineStr">
+        <is>
+          <t>Segnalazione ospite da proprietario</t>
+        </is>
+      </c>
+      <c r="B38" s="6" t="inlineStr">
+        <is>
+          <t>+2% sul totale mensile cliente</t>
+        </is>
+      </c>
+      <c r="C38" s="7" t="inlineStr">
+        <is>
+          <t>Incentivo per auto-portare ospiti</t>
+        </is>
+      </c>
+      <c r="D38" s="8" t="inlineStr">
+        <is>
+          <t>Il proprietario viene penalizzato economicamente per i propri contatti</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="40" customHeight="1">
+      <c r="A39" s="31" t="inlineStr">
+        <is>
+          <t>+3 unità in gestione Youhosty</t>
+        </is>
+      </c>
+      <c r="B39" s="32" t="inlineStr">
+        <is>
+          <t>+2% ulteriore sul totale mensile</t>
+        </is>
+      </c>
+      <c r="C39" s="32" t="inlineStr"/>
+      <c r="D39" s="8" t="inlineStr">
+        <is>
+          <t>Aumento progressivo dei costi con più immobili</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="20" customHeight="1">
+      <c r="A40" s="29" t="inlineStr">
+        <is>
+          <t>📅 ABBONAMENTO MENSILE MANUTENZIONE (IVA esclusa)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="40" customHeight="1">
+      <c r="A41" s="30" t="inlineStr">
+        <is>
+          <t>Costo All-Inclusive</t>
+        </is>
+      </c>
+      <c r="B41" s="6" t="inlineStr">
+        <is>
+          <t>€19,90/mese mono/bilocale | €26,90/mese trilo/quadrilocale</t>
+        </is>
+      </c>
+      <c r="C41" s="7" t="inlineStr">
+        <is>
+          <t>Manutenzione continuativa inclusa; check-up periodico; rinnovo attrezzatura pulizie</t>
+        </is>
+      </c>
+      <c r="D41" s="8" t="inlineStr">
+        <is>
+          <t>Dovuto anche con appartamento sfitto e anche per locazioni &gt;30 giorni (nessun break)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="40" customHeight="1">
+      <c r="A42" s="31" t="inlineStr">
+        <is>
+          <t>Costo Flexible</t>
+        </is>
+      </c>
+      <c r="B42" s="32" t="inlineStr">
+        <is>
+          <t>€22,90/mese mono/bilocale | €29,90/mese trilo/quadrilocale</t>
+        </is>
+      </c>
+      <c r="C42" s="32" t="inlineStr"/>
+      <c r="D42" s="32" t="inlineStr"/>
+    </row>
+    <row r="43" ht="40" customHeight="1">
+      <c r="A43" s="30" t="inlineStr">
+        <is>
+          <t>Massimale incluso nel mensile</t>
+        </is>
+      </c>
+      <c r="B43" s="6" t="inlineStr">
+        <is>
+          <t>€50 IVA inclusa/mese di interventi</t>
+        </is>
+      </c>
+      <c r="C43" s="7" t="inlineStr">
+        <is>
+          <t>Piccole manutenzioni coperte senza costi extra</t>
+        </is>
+      </c>
+      <c r="D43" s="8" t="inlineStr">
+        <is>
+          <t>Massimale molto basso: qualsiasi intervento oltre €50 genera costo aggiuntivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="40" customHeight="1">
+      <c r="A44" s="31" t="inlineStr">
+        <is>
+          <t>Interventi oltre €100 IVA inclusa</t>
+        </is>
+      </c>
+      <c r="B44" s="32" t="inlineStr">
+        <is>
+          <t>Previo consenso del cliente (6h di tempo per risposta in urgenza)</t>
+        </is>
+      </c>
+      <c r="C44" s="7" t="inlineStr">
+        <is>
+          <t>Maggior tutela rispetto a Italianway (soglia €200 senza consenso)</t>
+        </is>
+      </c>
+      <c r="D44" s="8" t="inlineStr">
+        <is>
+          <t>Se proprietario non risponde entro 6h, Youhosty agisce autonomamente</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="40" customHeight="1">
+      <c r="A45" s="30" t="inlineStr">
+        <is>
+          <t>Manutenzione straordinaria</t>
+        </is>
+      </c>
+      <c r="B45" s="6" t="inlineStr">
+        <is>
+          <t>Se proprietario non interviene entro 24h: Youhosty agisce in nome e per conto</t>
+        </is>
+      </c>
+      <c r="C45" s="7" t="inlineStr">
+        <is>
+          <t>Gestione rapida di emergenze</t>
+        </is>
+      </c>
+      <c r="D45" s="8" t="inlineStr">
+        <is>
+          <t>Costo ribaltato sul cliente; Youhosty può sospendere la pubblicizzazione se non si interviene</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="20" customHeight="1">
+      <c r="A46" s="29" t="inlineStr">
+        <is>
+          <t>📄 CONTRATTO, DURATA E RECESSO</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="40" customHeight="1">
+      <c r="A47" s="30" t="inlineStr">
+        <is>
+          <t>Durata All-Inclusive</t>
+        </is>
+      </c>
+      <c r="B47" s="6" t="inlineStr">
+        <is>
+          <t>24 mesi con rinnovo automatico (disdetta 3 mesi prima scadenza)</t>
+        </is>
+      </c>
+      <c r="C47" s="7" t="inlineStr">
+        <is>
+          <t>Stabilità per il gestore</t>
+        </is>
+      </c>
+      <c r="D47" s="8" t="inlineStr">
+        <is>
+          <t>Doppia la durata di Italianway (12 mesi); molto più vincolante</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="40" customHeight="1">
+      <c r="A48" s="31" t="inlineStr">
+        <is>
+          <t>Durata Online/Flexible</t>
+        </is>
+      </c>
+      <c r="B48" s="32" t="inlineStr">
+        <is>
+          <t>10/8 mesi periodo di prova + rinnovo 12 mesi</t>
+        </is>
+      </c>
+      <c r="C48" s="7" t="inlineStr">
+        <is>
+          <t>Periodo di prova prima dell'impegno lungo</t>
+        </is>
+      </c>
+      <c r="D48" s="8" t="inlineStr">
+        <is>
+          <t>Rinnovo automatico: rischio dimenticarsi di disdire</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="40" customHeight="1">
+      <c r="A49" s="30" t="inlineStr">
+        <is>
+          <t>Recesso All-Inclusive</t>
+        </is>
+      </c>
+      <c r="B49" s="6" t="inlineStr">
+        <is>
+          <t>Solo per forza maggiore verificata OPPURE immediato con €50/gg</t>
+        </is>
+      </c>
+      <c r="C49" s="7" t="inlineStr">
+        <is>
+          <t>Uscita di emergenza possibile</t>
+        </is>
+      </c>
+      <c r="D49" s="8" t="inlineStr">
+        <is>
+          <t>Il recesso ordinario non esiste: è di fatto un contratto a termine 24 mesi</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="40" customHeight="1">
+      <c r="A50" s="31" t="inlineStr">
+        <is>
+          <t>Recesso Online/Flexible</t>
+        </is>
+      </c>
+      <c r="B50" s="32" t="inlineStr">
+        <is>
+          <t>120 giorni preavviso OPPURE immediato con €50-100/gg</t>
+        </is>
+      </c>
+      <c r="C50" s="32" t="inlineStr"/>
+      <c r="D50" s="8" t="inlineStr">
+        <is>
+          <t>4 mesi è un vincolo significativo; penale giornaliera elevata</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="40" customHeight="1">
+      <c r="A51" s="30" t="inlineStr">
+        <is>
+          <t>Pratiche chiusura rapporto</t>
+        </is>
+      </c>
+      <c r="B51" s="6" t="inlineStr">
+        <is>
+          <t>Online €150 | All-Inclusive €220 | Flexible/Superflex €320</t>
+        </is>
+      </c>
+      <c r="C51" s="7" t="inlineStr">
+        <is>
+          <t>Costo esplicitato chiaramente</t>
+        </is>
+      </c>
+      <c r="D51" s="8" t="inlineStr">
+        <is>
+          <t>Costo obbligatorio al termine del contratto; in Italianway non è previsto</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="40" customHeight="1">
+      <c r="A52" s="31" t="inlineStr">
+        <is>
+          <t>Disinstallazione self check-in</t>
+        </is>
+      </c>
+      <c r="B52" s="32" t="inlineStr">
+        <is>
+          <t>€250 (Online/All-Inclusive) | €350 (Flexible/Superflex) – oppure voltura al cliente</t>
+        </is>
+      </c>
+      <c r="C52" s="32" t="inlineStr"/>
+      <c r="D52" s="8" t="inlineStr">
+        <is>
+          <t>Costo uscita significativo, da sommare alle pratiche chiusura</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="40" customHeight="1">
+      <c r="A53" s="30" t="inlineStr">
+        <is>
+          <t>Costo totale uscita (All-Inclusive)</t>
+        </is>
+      </c>
+      <c r="B53" s="6" t="inlineStr">
+        <is>
+          <t>€220 pratiche + €250 disinstallazione = €470 IVA esclusa</t>
+        </is>
+      </c>
+      <c r="C53" s="6" t="inlineStr"/>
+      <c r="D53" s="8" t="inlineStr">
+        <is>
+          <t>Barriera economica all'uscita elevata</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="40" customHeight="1">
+      <c r="A54" s="31" t="inlineStr">
+        <is>
+          <t>Prenotazioni post-recesso</t>
+        </is>
+      </c>
+      <c r="B54" s="32" t="inlineStr">
+        <is>
+          <t>Se prenotazioni terminano dopo data recesso: Youhosty incassa tutto</t>
+        </is>
+      </c>
+      <c r="C54" s="32" t="inlineStr"/>
+      <c r="D54" s="8" t="inlineStr">
+        <is>
+          <t>Il proprietario perde tutti gli incassi delle prenotazioni a scavalco</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="40" customHeight="1">
+      <c r="A55" s="30" t="inlineStr">
+        <is>
+          <t>Esclusiva</t>
+        </is>
+      </c>
+      <c r="B55" s="6" t="inlineStr">
+        <is>
+          <t>Sì – il cliente non può locare con terzi per tutta la durata</t>
+        </is>
+      </c>
+      <c r="C55" s="6" t="inlineStr"/>
+      <c r="D55" s="8" t="inlineStr">
+        <is>
+          <t>Penale: pari agli oneri accessori maturati sui contratti paralleli</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="40" customHeight="1">
+      <c r="A56" s="31" t="inlineStr">
+        <is>
+          <t>Penale accesso non autorizzato</t>
+        </is>
+      </c>
+      <c r="B56" s="32" t="inlineStr">
+        <is>
+          <t>€50 se il proprietario entra senza bloccare il calendario</t>
+        </is>
+      </c>
+      <c r="C56" s="32" t="inlineStr"/>
+      <c r="D56" s="8" t="inlineStr">
+        <is>
+          <t>Clausola penalizzante anche per usi d'emergenza</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="40" customHeight="1">
+      <c r="A57" s="30" t="inlineStr">
+        <is>
+          <t>Penale condivisione contratto</t>
+        </is>
+      </c>
+      <c r="B57" s="6" t="inlineStr">
+        <is>
+          <t>€1.000 per aver condiviso il contratto con terzi non autorizzati</t>
+        </is>
+      </c>
+      <c r="C57" s="6" t="inlineStr"/>
+      <c r="D57" s="8" t="inlineStr">
+        <is>
+          <t>Clausola limitante la libertà di consultare professionisti</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="20" customHeight="1">
+      <c r="A58" s="29" t="inlineStr">
+        <is>
+          <t>🏠 USO PERSONALE DELL'IMMOBILE</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="40" customHeight="1">
+      <c r="A59" s="30" t="inlineStr">
+        <is>
+          <t>Giorni uso personale All-Inclusive</t>
+        </is>
+      </c>
+      <c r="B59" s="6" t="inlineStr">
+        <is>
+          <t>45 giorni/anno (fuori Salone del Mobile e altri eventi primari)</t>
+        </is>
+      </c>
+      <c r="C59" s="7" t="inlineStr">
+        <is>
+          <t>Più giorni rispetto a Italianway (non specificato, ma con costi di ripristino)</t>
+        </is>
+      </c>
+      <c r="D59" s="8" t="inlineStr">
+        <is>
+          <t>Bloccati specifici periodi di alto afflusso: impossibile usare l'immobile nei momenti più redditizi</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="40" customHeight="1">
+      <c r="A60" s="31" t="inlineStr">
+        <is>
+          <t>Giorni uso personale Online/Flexible</t>
+        </is>
+      </c>
+      <c r="B60" s="32" t="inlineStr">
+        <is>
+          <t>20 gg periodo prova | 24 gg/anno successivi</t>
+        </is>
+      </c>
+      <c r="C60" s="32" t="inlineStr"/>
+      <c r="D60" s="8" t="inlineStr">
+        <is>
+          <t>Limitazione ridotta rispetto ad All-Inclusive</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="40" customHeight="1">
+      <c r="A61" s="30" t="inlineStr">
+        <is>
+          <t>Costo giorni aggiuntivi All-Inclusive/Flexible</t>
+        </is>
+      </c>
+      <c r="B61" s="6" t="inlineStr">
+        <is>
+          <t>€15 +IVA/giorno aggiuntivo + obbligo pulizia a carico proprietario</t>
+        </is>
+      </c>
+      <c r="C61" s="7" t="inlineStr">
+        <is>
+          <t>Costo contenuto per giorni extra</t>
+        </is>
+      </c>
+      <c r="D61" s="6" t="inlineStr"/>
+    </row>
+    <row r="62" ht="20" customHeight="1">
+      <c r="A62" s="29" t="inlineStr">
+        <is>
+          <t>🛎️ SERVIZI INCLUSI (pacchetto All-Inclusive)</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="40" customHeight="1">
+      <c r="A63" s="30" t="inlineStr">
+        <is>
+          <t>Piattaforma monitoraggio</t>
+        </is>
+      </c>
+      <c r="B63" s="6" t="inlineStr">
+        <is>
+          <t>App/sito internet per verificare andamento in tempo reale</t>
+        </is>
+      </c>
+      <c r="C63" s="7" t="inlineStr">
+        <is>
+          <t>Strumento digitale proprietario</t>
+        </is>
+      </c>
+      <c r="D63" s="8" t="inlineStr">
+        <is>
+          <t>Non si conosce il nome della piattaforma; non paragonabile a KALISI di Italianway per funzionalità descritte</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="40" customHeight="1">
+      <c r="A64" s="31" t="inlineStr">
+        <is>
+          <t>Revenue management</t>
+        </is>
+      </c>
+      <c r="B64" s="32" t="inlineStr">
+        <is>
+          <t>Software di ottimizzazione prezzi in outsourcing</t>
+        </is>
+      </c>
+      <c r="C64" s="7" t="inlineStr">
+        <is>
+          <t>Prezzi ottimizzati dinamicamente</t>
+        </is>
+      </c>
+      <c r="D64" s="8" t="inlineStr">
+        <is>
+          <t>Software in outsourcing = Youhosty non controlla direttamente l'algoritmo</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="40" customHeight="1">
+      <c r="A65" s="30" t="inlineStr">
+        <is>
+          <t>Pubblicazione OTA</t>
+        </is>
+      </c>
+      <c r="B65" s="6" t="inlineStr">
+        <is>
+          <t>Creazione e gestione profilo su più piattaforme (OTA non nominate esplicitamente)</t>
+        </is>
+      </c>
+      <c r="C65" s="7" t="inlineStr">
+        <is>
+          <t>Visibilità multicanale</t>
+        </is>
+      </c>
+      <c r="D65" s="8" t="inlineStr">
+        <is>
+          <t>Costo OTA addebitato al cliente (non nominale nel contratto)</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="40" customHeight="1">
+      <c r="A66" s="31" t="inlineStr">
+        <is>
+          <t>Self check-in automatizzato</t>
+        </is>
+      </c>
+      <c r="B66" s="32" t="inlineStr">
+        <is>
+          <t>Installato e gestito da Youhosty (meccanismi fisici)</t>
+        </is>
+      </c>
+      <c r="C66" s="7" t="inlineStr">
+        <is>
+          <t>Autonomia ospite; nessun intervento fisico per accoglienza</t>
+        </is>
+      </c>
+      <c r="D66" s="8" t="inlineStr">
+        <is>
+          <t>Costo disinstallazione €250-350 al termine</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="40" customHeight="1">
+      <c r="A67" s="30" t="inlineStr">
+        <is>
+          <t>Gestione prenotazioni e ospiti</t>
+        </is>
+      </c>
+      <c r="B67" s="6" t="inlineStr">
+        <is>
+          <t>Interazioni e recensioni in multilingua</t>
+        </is>
+      </c>
+      <c r="C67" s="7" t="inlineStr">
+        <is>
+          <t>Esperienza ospiti migliorata</t>
+        </is>
+      </c>
+      <c r="D67" s="6" t="inlineStr"/>
+    </row>
+    <row r="68" ht="40" customHeight="1">
+      <c r="A68" s="31" t="inlineStr">
+        <is>
+          <t>Burocrazia (Questura, CAV, cedolare)</t>
+        </is>
+      </c>
+      <c r="B68" s="32" t="inlineStr">
+        <is>
+          <t>Inclusa – cedolare secca solo per &lt;4 immobili e &lt;30gg</t>
+        </is>
+      </c>
+      <c r="C68" s="7" t="inlineStr">
+        <is>
+          <t>Gestione burocrazia delegata</t>
+        </is>
+      </c>
+      <c r="D68" s="8" t="inlineStr">
+        <is>
+          <t>Cedolare secca non gestita per &gt;4 immobili o locazioni &gt;30gg: obbligo torna al cliente</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="40" customHeight="1">
+      <c r="A69" s="30" t="inlineStr">
+        <is>
+          <t>Pagamento saldo cliente</t>
+        </is>
+      </c>
+      <c r="B69" s="6" t="inlineStr">
+        <is>
+          <t>Entro il 30° giorno del mese successivo all'incasso dalla piattaforma</t>
+        </is>
+      </c>
+      <c r="C69" s="7" t="inlineStr">
+        <is>
+          <t>Cadenza mensile</t>
+        </is>
+      </c>
+      <c r="D69" s="8" t="inlineStr">
+        <is>
+          <t>Può tardare fino a ~60 gg per incassi di inizio mese; nessun interesse sulle somme trattenute</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="40" customHeight="1">
+      <c r="A70" s="31" t="inlineStr">
+        <is>
+          <t>Più immobili</t>
+        </is>
+      </c>
+      <c r="B70" s="32" t="inlineStr">
+        <is>
+          <t>Bonifico cumulativo con reportistica per singolo immobile</t>
+        </is>
+      </c>
+      <c r="C70" s="7" t="inlineStr">
+        <is>
+          <t>Semplificazione per portafoglio multi-immobile</t>
+        </is>
+      </c>
+      <c r="D70" s="32" t="inlineStr"/>
+    </row>
+    <row r="71" ht="40" customHeight="1">
+      <c r="A71" s="30" t="inlineStr">
+        <is>
+          <t>Rinnovo attrezzatura pulizie</t>
+        </is>
+      </c>
+      <c r="B71" s="6" t="inlineStr">
+        <is>
+          <t>Incluso nell'abbonamento mensile (dopo usura)</t>
+        </is>
+      </c>
+      <c r="C71" s="7" t="inlineStr">
+        <is>
+          <t>Manutenzione dotazioni coperta</t>
+        </is>
+      </c>
+      <c r="D71" s="8" t="inlineStr">
+        <is>
+          <t>La prima fornitura deve essere presente in appartamento a carico proprietario</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="20" customHeight="1">
+      <c r="A72" s="29" t="inlineStr">
+        <is>
+          <t>🛡️ GARANZIA DANNI E ASSICURAZIONE</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="40" customHeight="1">
+      <c r="A73" s="30" t="inlineStr">
+        <is>
+          <t>Cauzione ospite</t>
+        </is>
+      </c>
+      <c r="B73" s="6" t="inlineStr">
+        <is>
+          <t>Applicata ove possibile dalla piattaforma (es. AirCover di Airbnb)</t>
+        </is>
+      </c>
+      <c r="C73" s="7" t="inlineStr">
+        <is>
+          <t>Protezione base inclusa dalla piattaforma</t>
+        </is>
+      </c>
+      <c r="D73" s="8" t="inlineStr">
+        <is>
+          <t>Non garantita su tutte le piattaforme; importo variabile e non definito contrattualmente</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="40" customHeight="1">
+      <c r="A74" s="31" t="inlineStr">
+        <is>
+          <t>Responsabilità di Youhosty per danni</t>
+        </is>
+      </c>
+      <c r="B74" s="32" t="inlineStr">
+        <is>
+          <t>Nessuna – Youhosty esplicitamente non responsabile</t>
+        </is>
+      </c>
+      <c r="C74" s="32" t="inlineStr"/>
+      <c r="D74" s="8" t="inlineStr">
+        <is>
+          <t>Il proprietario si assume tutto il rischio di danni all'immobile</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="40" customHeight="1">
+      <c r="A75" s="30" t="inlineStr">
+        <is>
+          <t>Assicurazione RC obbligatoria</t>
+        </is>
+      </c>
+      <c r="B75" s="6" t="inlineStr">
+        <is>
+          <t>A carico del cliente (obbligatoria per legge)</t>
+        </is>
+      </c>
+      <c r="C75" s="6" t="inlineStr"/>
+      <c r="D75" s="8" t="inlineStr">
+        <is>
+          <t>Youhosty non fornisce né gestisce polizze assicurative</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="40" customHeight="1">
+      <c r="A76" s="31" t="inlineStr">
+        <is>
+          <t>Assicurazione beni di pregio</t>
+        </is>
+      </c>
+      <c r="B76" s="32" t="inlineStr">
+        <is>
+          <t>Consigliata ma a carico e gestione del cliente</t>
+        </is>
+      </c>
+      <c r="C76" s="32" t="inlineStr"/>
+      <c r="D76" s="8" t="inlineStr">
+        <is>
+          <t>Nessuna polizza collettiva come quella di Italianway (RC €1M, incendio, furto)</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="40" customHeight="1">
+      <c r="A77" s="30" t="inlineStr">
+        <is>
+          <t>Canone garantito</t>
+        </is>
+      </c>
+      <c r="B77" s="6" t="inlineStr">
+        <is>
+          <t>Disponibile (Allegato 3 – non allegato nel documento ricevuto)</t>
+        </is>
+      </c>
+      <c r="C77" s="7" t="inlineStr">
+        <is>
+          <t>Opzione di protezione dal rischio vacancy</t>
+        </is>
+      </c>
+      <c r="D77" s="8" t="inlineStr">
+        <is>
+          <t>Costo aggiuntivo; allegato non disponibile per valutazione</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="40" customHeight="1">
+      <c r="A78" s="31" t="inlineStr">
+        <is>
+          <t>Recupero danni &gt; cauzione</t>
+        </is>
+      </c>
+      <c r="B78" s="32" t="inlineStr">
+        <is>
+          <t>Youhosty si attiva senza obbligo di risultato</t>
+        </is>
+      </c>
+      <c r="C78" s="7" t="inlineStr">
+        <is>
+          <t>Supporto nella gestione del sinistro</t>
+        </is>
+      </c>
+      <c r="D78" s="8" t="inlineStr">
+        <is>
+          <t>Nessuna garanzia di recupero; azioni legali a carico del cliente</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="40" customHeight="1">
+      <c r="A79" s="30" t="inlineStr">
+        <is>
+          <t>Oggetti di valore</t>
+        </is>
+      </c>
+      <c r="B79" s="6" t="inlineStr">
+        <is>
+          <t>Non devono essere presenti in appartamento</t>
+        </is>
+      </c>
+      <c r="C79" s="6" t="inlineStr"/>
+      <c r="D79" s="8" t="inlineStr">
+        <is>
+          <t>Nessuna copertura per oggetti non nell'inventario Youhosty</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="20" customHeight="1">
+      <c r="A80" s="29" t="inlineStr">
+        <is>
+          <t>📋 OBBLIGHI E ONERI DEL CLIENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="40" customHeight="1">
+      <c r="A81" s="30" t="inlineStr">
+        <is>
+          <t>Chiavi da consegnare</t>
+        </is>
+      </c>
+      <c r="B81" s="6" t="inlineStr">
+        <is>
+          <t>5 mazzi (o 1 con self check-in installato)</t>
+        </is>
+      </c>
+      <c r="C81" s="7" t="inlineStr">
+        <is>
+          <t>Risparmio rispetto a Italianway (6 mazzi)</t>
+        </is>
+      </c>
+      <c r="D81" s="6" t="inlineStr"/>
+    </row>
+    <row r="82" ht="40" customHeight="1">
+      <c r="A82" s="31" t="inlineStr">
+        <is>
+          <t>Piumoni</t>
+        </is>
+      </c>
+      <c r="B82" s="32" t="inlineStr">
+        <is>
+          <t>Almeno 1 per letto</t>
+        </is>
+      </c>
+      <c r="C82" s="32" t="inlineStr"/>
+      <c r="D82" s="8" t="inlineStr">
+        <is>
+          <t>Non specifica ulteriori dotazioni obbligatorie (meno prescrittivo di Italianway)</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="40" customHeight="1">
+      <c r="A83" s="30" t="inlineStr">
+        <is>
+          <t>APE e certificazione impianti</t>
+        </is>
+      </c>
+      <c r="B83" s="6" t="inlineStr">
+        <is>
+          <t>Obbligatoria per locazioni &gt;30 giorni</t>
+        </is>
+      </c>
+      <c r="C83" s="7" t="inlineStr">
+        <is>
+          <t>Youhosty può acquistarla per conto del cliente</t>
+        </is>
+      </c>
+      <c r="D83" s="8" t="inlineStr">
+        <is>
+          <t>Costo APE €180 e estratti catastali €100 a carico cliente</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="40" customHeight="1">
+      <c r="A84" s="31" t="inlineStr">
+        <is>
+          <t>TARI, canone RAI, utenze</t>
+        </is>
+      </c>
+      <c r="B84" s="32" t="inlineStr">
+        <is>
+          <t>A carico del cliente</t>
+        </is>
+      </c>
+      <c r="C84" s="32" t="inlineStr"/>
+      <c r="D84" s="8" t="inlineStr">
+        <is>
+          <t>A differenza di Italianway dove queste voci sono incluse nel canone</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="40" customHeight="1">
+      <c r="A85" s="30" t="inlineStr">
+        <is>
+          <t>Prima dotazione pulizie</t>
+        </is>
+      </c>
+      <c r="B85" s="6" t="inlineStr">
+        <is>
+          <t>Presente in appartamento a carico proprietario (prima della messa online)</t>
+        </is>
+      </c>
+      <c r="C85" s="6" t="inlineStr"/>
+      <c r="D85" s="6" t="inlineStr"/>
+    </row>
+    <row r="86" ht="40" customHeight="1">
+      <c r="A86" s="31" t="inlineStr">
+        <is>
+          <t>Verifica regolamento condominiale</t>
+        </is>
+      </c>
+      <c r="B86" s="32" t="inlineStr">
+        <is>
+          <t>Obbligo del cliente verificare che il condominio permetta affitti brevi</t>
+        </is>
+      </c>
+      <c r="C86" s="32" t="inlineStr"/>
+      <c r="D86" s="8" t="inlineStr">
+        <is>
+          <t>Se il condominio lo vieta e l'attività parte, la responsabilità è del cliente</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="40" customHeight="1">
+      <c r="A87" s="30" t="inlineStr">
+        <is>
+          <t>Stato dell'immobile</t>
+        </is>
+      </c>
+      <c r="B87" s="6" t="inlineStr">
+        <is>
+          <t>Deve essere a norma e in perfetto stato; criticità check-up iniziale da ripristinare prima dell'avvio</t>
+        </is>
+      </c>
+      <c r="C87" s="6" t="inlineStr"/>
+      <c r="D87" s="8" t="inlineStr">
+        <is>
+          <t>Il cliente sostiene i costi di eventuale messa a norma</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="40" customHeight="1">
+      <c r="A88" s="31" t="inlineStr">
+        <is>
+          <t>Vendita immobile</t>
+        </is>
+      </c>
+      <c r="B88" s="32" t="inlineStr">
+        <is>
+          <t>Mandato automatico a Youhosty per pubblicazione annuncio tramite partner</t>
+        </is>
+      </c>
+      <c r="C88" s="7" t="inlineStr">
+        <is>
+          <t>Supporto alla vendita senza costi aggiuntivi dichiarati</t>
+        </is>
+      </c>
+      <c r="D88" s="8" t="inlineStr">
+        <is>
+          <t>Il proprietario perde il controllo sulla scelta dell'agente immobiliare</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" ht="20" customHeight="1">
+      <c r="A89" s="29" t="inlineStr">
+        <is>
+          <t>🔧 SERVIZI A RICHIESTA (IVA esclusa)</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="40" customHeight="1">
+      <c r="A90" s="30" t="inlineStr">
+        <is>
+          <t>Property Finding</t>
+        </is>
+      </c>
+      <c r="B90" s="6" t="inlineStr">
+        <is>
+          <t>€1.000 + 3,5% sul valore di acquisto</t>
+        </is>
+      </c>
+      <c r="C90" s="7" t="inlineStr">
+        <is>
+          <t>Servizio di ricerca immobili per investimento</t>
+        </is>
+      </c>
+      <c r="D90" s="8" t="inlineStr">
+        <is>
+          <t>Costo fisso alto + percentuale sull'acquisto</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" ht="40" customHeight="1">
+      <c r="A91" s="31" t="inlineStr">
+        <is>
+          <t>Pulizie approfondite mensili</t>
+        </is>
+      </c>
+      <c r="B91" s="32" t="inlineStr">
+        <is>
+          <t>€30/mese (mono/bi) | €50/mese (tri/quadri) | €100/mese (plurilocale)</t>
+        </is>
+      </c>
+      <c r="C91" s="7" t="inlineStr">
+        <is>
+          <t>Prezzi competitivi e chiari</t>
+        </is>
+      </c>
+      <c r="D91" s="8" t="inlineStr">
+        <is>
+          <t>Servizio a parte rispetto all'abbonamento</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" ht="40" customHeight="1">
+      <c r="A92" s="30" t="inlineStr">
+        <is>
+          <t>Estratti catastali</t>
+        </is>
+      </c>
+      <c r="B92" s="6" t="inlineStr">
+        <is>
+          <t>€100</t>
+        </is>
+      </c>
+      <c r="C92" s="6" t="inlineStr"/>
+      <c r="D92" s="6" t="inlineStr"/>
+    </row>
+    <row r="93" ht="40" customHeight="1">
+      <c r="A93" s="31" t="inlineStr">
+        <is>
+          <t>APE</t>
+        </is>
+      </c>
+      <c r="B93" s="32" t="inlineStr">
+        <is>
+          <t>€180</t>
+        </is>
+      </c>
+      <c r="C93" s="32" t="inlineStr"/>
+      <c r="D93" s="32" t="inlineStr"/>
+    </row>
+    <row r="94" ht="40" customHeight="1">
+      <c r="A94" s="30" t="inlineStr">
+        <is>
+          <t>Gestione corrispondenza</t>
+        </is>
+      </c>
+      <c r="B94" s="6" t="inlineStr">
+        <is>
+          <t>€5,99/mese</t>
+        </is>
+      </c>
+      <c r="C94" s="6" t="inlineStr"/>
+      <c r="D94" s="8" t="inlineStr">
+        <is>
+          <t>Costo ricorrente per servizio base</t>
+        </is>
+      </c>
+    </row>
+    <row r="95" ht="40" customHeight="1">
+      <c r="A95" s="31" t="inlineStr">
+        <is>
+          <t>Sostituzione aspirapolvere</t>
+        </is>
+      </c>
+      <c r="B95" s="32" t="inlineStr">
+        <is>
+          <t>€60 +IVA</t>
+        </is>
+      </c>
+      <c r="C95" s="32" t="inlineStr"/>
+      <c r="D95" s="32" t="inlineStr"/>
+    </row>
+    <row r="96" ht="40" customHeight="1">
+      <c r="A96" s="30" t="inlineStr">
+        <is>
+          <t>Consulenza legale/finanziaria</t>
+        </is>
+      </c>
+      <c r="B96" s="6" t="inlineStr">
+        <is>
+          <t>Da definire</t>
+        </is>
+      </c>
+      <c r="C96" s="7" t="inlineStr">
+        <is>
+          <t>Accesso a professionisti nazionali/internazionali</t>
+        </is>
+      </c>
+      <c r="D96" s="8" t="inlineStr">
+        <is>
+          <t>Costi non trasparenti; regolati da contratto separato</t>
+        </is>
+      </c>
+    </row>
+    <row r="97" ht="20" customHeight="1">
+      <c r="A97" s="29" t="inlineStr">
+        <is>
+          <t>🏡 COMMISSIONE COMPRAVENDITA</t>
+        </is>
+      </c>
+    </row>
+    <row r="98" ht="40" customHeight="1">
+      <c r="A98" s="30" t="inlineStr">
+        <is>
+          <t>Con esclusiva vendita (6 mesi)</t>
+        </is>
+      </c>
+      <c r="B98" s="6" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="C98" s="7" t="inlineStr">
+        <is>
+          <t>Nessuna commissione se si dà l'esclusiva a Youhosty</t>
+        </is>
+      </c>
+      <c r="D98" s="8" t="inlineStr">
+        <is>
+          <t>Il proprietario non può affidarsi ad altri agenti per 6 mesi</t>
+        </is>
+      </c>
+    </row>
+    <row r="99" ht="40" customHeight="1">
+      <c r="A99" s="31" t="inlineStr">
+        <is>
+          <t>Senza esclusiva vendita</t>
+        </is>
+      </c>
+      <c r="B99" s="32" t="inlineStr">
+        <is>
+          <t>3% (All-Inclusive) / 3,5% (altri pacchetti)</t>
+        </is>
+      </c>
+      <c r="C99" s="32" t="inlineStr"/>
+      <c r="D99" s="8" t="inlineStr">
+        <is>
+          <t>Commissione elevata senza esclusiva</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="15">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A40:D40"/>
+    <mergeCell ref="A9:D9"/>
+    <mergeCell ref="A80:D80"/>
+    <mergeCell ref="A89:D89"/>
+    <mergeCell ref="A58:D58"/>
+    <mergeCell ref="A97:D97"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="A62:D62"/>
+    <mergeCell ref="A72:D72"/>
+    <mergeCell ref="A15:D15"/>
+    <mergeCell ref="A24:D24"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A33:D33"/>
+    <mergeCell ref="A46:D46"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:D55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1843,6 +3821,9 @@
           <t>CONFRONTO PROPERTY MANAGER – ITALIANWAY vs AZIENDA B vs AZIENDA C</t>
         </is>
       </c>
+      <c r="B1" s="24" t="n"/>
+      <c r="C1" s="24" t="n"/>
+      <c r="D1" s="25" t="n"/>
     </row>
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="11" t="inlineStr">
@@ -1850,6 +3831,9 @@
           <t>Inserire i dati delle altre due aziende nelle colonne gialle per confronto automatico</t>
         </is>
       </c>
+      <c r="B2" s="24" t="n"/>
+      <c r="C2" s="24" t="n"/>
+      <c r="D2" s="25" t="n"/>
     </row>
     <row r="3" ht="28" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
@@ -1862,10 +3846,10 @@
           <t>ITALIANWAY</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>AZIENDA B
-(da compilare)</t>
+      <c r="C3" s="33" t="inlineStr">
+        <is>
+          <t>YOUHOSTY
+(A.P.P.A. Srl)</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
@@ -1881,6 +3865,9 @@
           <t>▶  COMMISSIONI</t>
         </is>
       </c>
+      <c r="B4" s="24" t="n"/>
+      <c r="C4" s="24" t="n"/>
+      <c r="D4" s="25" t="n"/>
     </row>
     <row r="5" ht="38" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
@@ -1893,7 +3880,13 @@
           <t>25% + 2% (a carico ospite) + 2% (provvigione mediatore)</t>
         </is>
       </c>
-      <c r="C5" s="14" t="inlineStr"/>
+      <c r="C5" s="34" t="inlineStr">
+        <is>
+          <t>All-Inclusive 1 imm: 16,5% Youhosty + costo OTA addebitato
+Online 1 imm: 10% + OTA
+NB: basi diverse da Italianway</t>
+        </is>
+      </c>
       <c r="D5" s="14" t="inlineStr"/>
     </row>
     <row r="6" ht="38" customHeight="1">
@@ -1907,7 +3900,12 @@
           <t>€ 600 + IVA</t>
         </is>
       </c>
-      <c r="C6" s="14" t="inlineStr"/>
+      <c r="C6" s="34" t="inlineStr">
+        <is>
+          <t>All-Inclusive (ant.): foto €69 + CAV €149 + sicurezza €219 ≈ €437 IVA escl.
+Alternativa: 0 setup + 2,5% extra su commissioni</t>
+        </is>
+      </c>
       <c r="D6" s="14" t="inlineStr"/>
     </row>
     <row r="7" ht="38" customHeight="1">
@@ -1921,7 +3919,11 @@
           <t>2% (solo breve termine)</t>
         </is>
       </c>
-      <c r="C7" s="14" t="inlineStr"/>
+      <c r="C7" s="34" t="inlineStr">
+        <is>
+          <t>Non applicabile (nessun mediatore separato)</t>
+        </is>
+      </c>
       <c r="D7" s="14" t="inlineStr"/>
     </row>
     <row r="8" ht="38" customHeight="1">
@@ -1935,7 +3937,11 @@
           <t>25% del costo soggiorno</t>
         </is>
       </c>
-      <c r="C8" s="14" t="inlineStr"/>
+      <c r="C8" s="34" t="inlineStr">
+        <is>
+          <t>Non separata: le commissioni Youhosty sono a carico del proprietario (trattenute dal ricavo), non dell'ospite</t>
+        </is>
+      </c>
       <c r="D8" s="14" t="inlineStr"/>
     </row>
     <row r="9" ht="38" customHeight="1">
@@ -1949,7 +3955,11 @@
           <t>2% del costo soggiorno (incluso nel 25%)</t>
         </is>
       </c>
-      <c r="C9" s="14" t="inlineStr"/>
+      <c r="C9" s="34" t="inlineStr">
+        <is>
+          <t>Non esplicitamente menzionate</t>
+        </is>
+      </c>
       <c r="D9" s="14" t="inlineStr"/>
     </row>
     <row r="10" ht="38" customHeight="1">
@@ -1963,7 +3973,11 @@
           <t>Max 10% del preventivo (opzionale)</t>
         </is>
       </c>
-      <c r="C10" s="14" t="inlineStr"/>
+      <c r="C10" s="34" t="inlineStr">
+        <is>
+          <t>Servizio arredo 'da definire'; non incluso in alcun pacchetto standard</t>
+        </is>
+      </c>
       <c r="D10" s="14" t="inlineStr"/>
     </row>
     <row r="11" ht="20" customHeight="1">
@@ -1972,6 +3986,9 @@
           <t>▶  CONTRATTO</t>
         </is>
       </c>
+      <c r="B11" s="24" t="n"/>
+      <c r="C11" s="24" t="n"/>
+      <c r="D11" s="25" t="n"/>
     </row>
     <row r="12" ht="38" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
@@ -1984,7 +4001,12 @@
           <t>12 mesi</t>
         </is>
       </c>
-      <c r="C12" s="14" t="inlineStr"/>
+      <c r="C12" s="34" t="inlineStr">
+        <is>
+          <t>All-Inclusive: 24 mesi
+Online/Flexible: 8-10 mesi di prova</t>
+        </is>
+      </c>
       <c r="D12" s="14" t="inlineStr"/>
     </row>
     <row r="13" ht="38" customHeight="1">
@@ -1998,7 +4020,11 @@
           <t>Tacito annuale</t>
         </is>
       </c>
-      <c r="C13" s="14" t="inlineStr"/>
+      <c r="C13" s="34" t="inlineStr">
+        <is>
+          <t>Automatico (disdetta 3 mesi prima scadenza per All-Inclusive)</t>
+        </is>
+      </c>
       <c r="D13" s="14" t="inlineStr"/>
     </row>
     <row r="14" ht="38" customHeight="1">
@@ -2012,7 +4038,12 @@
           <t>3 mesi (raccomandata)</t>
         </is>
       </c>
-      <c r="C14" s="14" t="inlineStr"/>
+      <c r="C14" s="34" t="inlineStr">
+        <is>
+          <t>All-Inclusive: solo forza maggiore o immediato €50/gg
+Online/Flexible: 120 giorni</t>
+        </is>
+      </c>
       <c r="D14" s="14" t="inlineStr"/>
     </row>
     <row r="15" ht="38" customHeight="1">
@@ -2026,7 +4057,12 @@
           <t>€ 20 / giorno</t>
         </is>
       </c>
-      <c r="C15" s="14" t="inlineStr"/>
+      <c r="C15" s="34" t="inlineStr">
+        <is>
+          <t>Recesso immediato: €50/gg (Online/All-Incl.) o €100/gg (Flexible)
+Più pratiche chiusura €220-320 + disinstallazione €250-350</t>
+        </is>
+      </c>
       <c r="D15" s="14" t="inlineStr"/>
     </row>
     <row r="16" ht="38" customHeight="1">
@@ -2040,7 +4076,11 @@
           <t>Sì – assoluta per tutta la durata</t>
         </is>
       </c>
-      <c r="C16" s="14" t="inlineStr"/>
+      <c r="C16" s="34" t="inlineStr">
+        <is>
+          <t>Sì – assoluta (penale = oneri maturati sui contratti paralleli)</t>
+        </is>
+      </c>
       <c r="D16" s="14" t="inlineStr"/>
     </row>
     <row r="17" ht="38" customHeight="1">
@@ -2054,7 +4094,13 @@
           <t>Consentito (con costi di ripristino)</t>
         </is>
       </c>
-      <c r="C17" s="14" t="inlineStr"/>
+      <c r="C17" s="34" t="inlineStr">
+        <is>
+          <t>All-Inclusive: 45 gg/anno (fuori Salone Mobile)
+Online/Flexible: 24 gg/anno
+Extra: €15+IVA/gg</t>
+        </is>
+      </c>
       <c r="D17" s="14" t="inlineStr"/>
     </row>
     <row r="18" ht="38" customHeight="1">
@@ -2068,7 +4114,11 @@
           <t>14 giorni dalla firma</t>
         </is>
       </c>
-      <c r="C18" s="14" t="inlineStr"/>
+      <c r="C18" s="34" t="inlineStr">
+        <is>
+          <t>Non menzionato esplicitamente nel contratto</t>
+        </is>
+      </c>
       <c r="D18" s="14" t="inlineStr"/>
     </row>
     <row r="19" ht="20" customHeight="1">
@@ -2077,6 +4127,9 @@
           <t>▶  SERVIZI</t>
         </is>
       </c>
+      <c r="B19" s="24" t="n"/>
+      <c r="C19" s="24" t="n"/>
+      <c r="D19" s="25" t="n"/>
     </row>
     <row r="20" ht="38" customHeight="1">
       <c r="A20" s="5" t="inlineStr">
@@ -2089,7 +4142,11 @@
           <t>KALISI (proprietaria Italianway)</t>
         </is>
       </c>
-      <c r="C20" s="14" t="inlineStr"/>
+      <c r="C20" s="34" t="inlineStr">
+        <is>
+          <t>App/sito internet Youhosty (nome non specificato)</t>
+        </is>
+      </c>
       <c r="D20" s="14" t="inlineStr"/>
     </row>
     <row r="21" ht="38" customHeight="1">
@@ -2103,7 +4160,11 @@
           <t>Sì – algoritmo + ufficio RM</t>
         </is>
       </c>
-      <c r="C21" s="14" t="inlineStr"/>
+      <c r="C21" s="34" t="inlineStr">
+        <is>
+          <t>Sì – software in outsourcing (provider non nominato)</t>
+        </is>
+      </c>
       <c r="D21" s="14" t="inlineStr"/>
     </row>
     <row r="22" ht="38" customHeight="1">
@@ -2117,7 +4178,12 @@
           <t>Portale Italianway + OTA terze</t>
         </is>
       </c>
-      <c r="C22" s="14" t="inlineStr"/>
+      <c r="C22" s="34" t="inlineStr">
+        <is>
+          <t>Sì – OTA multiple (non nominate)
+Costo OTA addebitato al cliente</t>
+        </is>
+      </c>
       <c r="D22" s="14" t="inlineStr"/>
     </row>
     <row r="23" ht="38" customHeight="1">
@@ -2131,7 +4197,11 @@
           <t>Sì – incluso</t>
         </is>
       </c>
-      <c r="C23" s="14" t="inlineStr"/>
+      <c r="C23" s="34" t="inlineStr">
+        <is>
+          <t>Sì – self check-in automatizzato incluso (All-Inclusive)</t>
+        </is>
+      </c>
       <c r="D23" s="14" t="inlineStr"/>
     </row>
     <row r="24" ht="38" customHeight="1">
@@ -2145,7 +4215,11 @@
           <t>Sì – a carico ospite</t>
         </is>
       </c>
-      <c r="C24" s="14" t="inlineStr"/>
+      <c r="C24" s="34" t="inlineStr">
+        <is>
+          <t>Sì – costo ribaltato sull'ospite (ove possibile sulla piattaforma)</t>
+        </is>
+      </c>
       <c r="D24" s="14" t="inlineStr"/>
     </row>
     <row r="25" ht="38" customHeight="1">
@@ -2159,7 +4233,11 @@
           <t>Sì – incluso</t>
         </is>
       </c>
-      <c r="C25" s="14" t="inlineStr"/>
+      <c r="C25" s="34" t="inlineStr">
+        <is>
+          <t>Sì – incluso in All-Inclusive</t>
+        </is>
+      </c>
       <c r="D25" s="14" t="inlineStr"/>
     </row>
     <row r="26" ht="38" customHeight="1">
@@ -2173,7 +4251,11 @@
           <t>Sì – incluso</t>
         </is>
       </c>
-      <c r="C26" s="14" t="inlineStr"/>
+      <c r="C26" s="34" t="inlineStr">
+        <is>
+          <t>Non menzionato esplicitamente</t>
+        </is>
+      </c>
       <c r="D26" s="14" t="inlineStr"/>
     </row>
     <row r="27" ht="38" customHeight="1">
@@ -2187,7 +4269,11 @@
           <t>Sì – incluso</t>
         </is>
       </c>
-      <c r="C27" s="14" t="inlineStr"/>
+      <c r="C27" s="34" t="inlineStr">
+        <is>
+          <t>Sì – €99 (o €69 con pagamento anticipato), obbligatoria</t>
+        </is>
+      </c>
       <c r="D27" s="14" t="inlineStr"/>
     </row>
     <row r="28" ht="38" customHeight="1">
@@ -2201,7 +4287,11 @@
           <t>Sì – incluso</t>
         </is>
       </c>
-      <c r="C28" s="14" t="inlineStr"/>
+      <c r="C28" s="34" t="inlineStr">
+        <is>
+          <t>Sì – gestione profilo multilingua inclusa</t>
+        </is>
+      </c>
       <c r="D28" s="14" t="inlineStr"/>
     </row>
     <row r="29" ht="38" customHeight="1">
@@ -2215,7 +4305,11 @@
           <t>Sì – frequenza non specificata</t>
         </is>
       </c>
-      <c r="C29" s="14" t="inlineStr"/>
+      <c r="C29" s="34" t="inlineStr">
+        <is>
+          <t>Sì – check-up periodico nell'abbonamento mensile</t>
+        </is>
+      </c>
       <c r="D29" s="14" t="inlineStr"/>
     </row>
     <row r="30" ht="38" customHeight="1">
@@ -2229,7 +4323,11 @@
           <t>Entro il 28° del mese successivo</t>
         </is>
       </c>
-      <c r="C30" s="14" t="inlineStr"/>
+      <c r="C30" s="34" t="inlineStr">
+        <is>
+          <t>Entro il 30° giorno del mese successivo all'incasso dalla piattaforma</t>
+        </is>
+      </c>
       <c r="D30" s="14" t="inlineStr"/>
     </row>
     <row r="31" ht="20" customHeight="1">
@@ -2238,6 +4336,9 @@
           <t>▶  ASSICURAZIONE</t>
         </is>
       </c>
+      <c r="B31" s="24" t="n"/>
+      <c r="C31" s="24" t="n"/>
+      <c r="D31" s="25" t="n"/>
     </row>
     <row r="32" ht="38" customHeight="1">
       <c r="A32" s="5" t="inlineStr">
@@ -2250,7 +4351,11 @@
           <t>€ 1.000.000</t>
         </is>
       </c>
-      <c r="C32" s="14" t="inlineStr"/>
+      <c r="C32" s="34" t="inlineStr">
+        <is>
+          <t>Non fornita da Youhosty – obbligatoria per legge a carico cliente</t>
+        </is>
+      </c>
       <c r="D32" s="14" t="inlineStr"/>
     </row>
     <row r="33" ht="38" customHeight="1">
@@ -2264,7 +4369,11 @@
           <t>€ 75.000 PRA</t>
         </is>
       </c>
-      <c r="C33" s="14" t="inlineStr"/>
+      <c r="C33" s="34" t="inlineStr">
+        <is>
+          <t>Non fornita – a carico cliente</t>
+        </is>
+      </c>
       <c r="D33" s="14" t="inlineStr"/>
     </row>
     <row r="34" ht="38" customHeight="1">
@@ -2278,7 +4387,11 @@
           <t>€ 10.000 PRA</t>
         </is>
       </c>
-      <c r="C34" s="14" t="inlineStr"/>
+      <c r="C34" s="34" t="inlineStr">
+        <is>
+          <t>Non fornita – a carico cliente</t>
+        </is>
+      </c>
       <c r="D34" s="14" t="inlineStr"/>
     </row>
     <row r="35" ht="38" customHeight="1">
@@ -2292,7 +4405,11 @@
           <t>€ 2.500 PRA</t>
         </is>
       </c>
-      <c r="C35" s="14" t="inlineStr"/>
+      <c r="C35" s="34" t="inlineStr">
+        <is>
+          <t>Non fornita – a carico cliente</t>
+        </is>
+      </c>
       <c r="D35" s="14" t="inlineStr"/>
     </row>
     <row r="36" ht="38" customHeight="1">
@@ -2306,7 +4423,11 @@
           <t>€ 2.000 PRA</t>
         </is>
       </c>
-      <c r="C36" s="14" t="inlineStr"/>
+      <c r="C36" s="34" t="inlineStr">
+        <is>
+          <t>Non fornita – a carico cliente</t>
+        </is>
+      </c>
       <c r="D36" s="14" t="inlineStr"/>
     </row>
     <row r="37" ht="38" customHeight="1">
@@ -2320,7 +4441,11 @@
           <t>Sì</t>
         </is>
       </c>
-      <c r="C37" s="14" t="inlineStr"/>
+      <c r="C37" s="34" t="inlineStr">
+        <is>
+          <t>Non fornita – a carico cliente</t>
+        </is>
+      </c>
       <c r="D37" s="14" t="inlineStr"/>
     </row>
     <row r="38" ht="38" customHeight="1">
@@ -2334,7 +4459,11 @@
           <t>€ 100 / sinistro</t>
         </is>
       </c>
-      <c r="C38" s="14" t="inlineStr"/>
+      <c r="C38" s="34" t="inlineStr">
+        <is>
+          <t>Cauzione ospite (ove possibile sulla piattaforma); importo variabile</t>
+        </is>
+      </c>
       <c r="D38" s="14" t="inlineStr"/>
     </row>
     <row r="39" ht="38" customHeight="1">
@@ -2348,7 +4477,11 @@
           <t>1 anno</t>
         </is>
       </c>
-      <c r="C39" s="14" t="inlineStr"/>
+      <c r="C39" s="34" t="inlineStr">
+        <is>
+          <t>Non applicabile (nessuna polizza Youhosty)</t>
+        </is>
+      </c>
       <c r="D39" s="14" t="inlineStr"/>
     </row>
     <row r="40" ht="38" customHeight="1">
@@ -2362,7 +4495,11 @@
           <t>TODESCO SAS Insurance Brokers</t>
         </is>
       </c>
-      <c r="C40" s="14" t="inlineStr"/>
+      <c r="C40" s="34" t="inlineStr">
+        <is>
+          <t>Nessuno – cliente autonomo</t>
+        </is>
+      </c>
       <c r="D40" s="14" t="inlineStr"/>
     </row>
     <row r="41" ht="20" customHeight="1">
@@ -2371,6 +4508,9 @@
           <t>▶  DOTAZIONI (oneri proprietario)</t>
         </is>
       </c>
+      <c r="B41" s="24" t="n"/>
+      <c r="C41" s="24" t="n"/>
+      <c r="D41" s="25" t="n"/>
     </row>
     <row r="42" ht="38" customHeight="1">
       <c r="A42" s="5" t="inlineStr">
@@ -2383,7 +4523,12 @@
           <t>Frigorifero, lavatrice, TV smart≥32", microonde, bollitore, tostapane</t>
         </is>
       </c>
-      <c r="C42" s="14" t="inlineStr"/>
+      <c r="C42" s="34" t="inlineStr">
+        <is>
+          <t>Non specificati in lista (meno prescrittivo)
+Aspirapolv. incluso nella Setup Fee (facoltativo)</t>
+        </is>
+      </c>
       <c r="D42" s="14" t="inlineStr"/>
     </row>
     <row r="43" ht="38" customHeight="1">
@@ -2397,7 +4542,11 @@
           <t>Sì</t>
         </is>
       </c>
-      <c r="C43" s="14" t="inlineStr"/>
+      <c r="C43" s="34" t="inlineStr">
+        <is>
+          <t>Non menzionato esplicitamente</t>
+        </is>
+      </c>
       <c r="D43" s="14" t="inlineStr"/>
     </row>
     <row r="44" ht="38" customHeight="1">
@@ -2411,7 +4560,11 @@
           <t>Obbligatoria medio termine; raccomandata breve</t>
         </is>
       </c>
-      <c r="C44" s="14" t="inlineStr"/>
+      <c r="C44" s="34" t="inlineStr">
+        <is>
+          <t>Non menzionata</t>
+        </is>
+      </c>
       <c r="D44" s="14" t="inlineStr"/>
     </row>
     <row r="45" ht="38" customHeight="1">
@@ -2425,7 +4578,12 @@
           <t>Sì – a carico proprietà</t>
         </is>
       </c>
-      <c r="C45" s="14" t="inlineStr"/>
+      <c r="C45" s="34" t="inlineStr">
+        <is>
+          <t>Sì – in noleggio gestito da Youhosty (€219-259 con All-Inclusive)
+Rinnovo incluso nell'abbonamento mensile</t>
+        </is>
+      </c>
       <c r="D45" s="14" t="inlineStr"/>
     </row>
     <row r="46" ht="38" customHeight="1">
@@ -2439,7 +4597,11 @@
           <t>6 mazzi completi</t>
         </is>
       </c>
-      <c r="C46" s="14" t="inlineStr"/>
+      <c r="C46" s="34" t="inlineStr">
+        <is>
+          <t>5 mazzi (o 1 con self check-in installato)</t>
+        </is>
+      </c>
       <c r="D46" s="14" t="inlineStr"/>
     </row>
     <row r="47" ht="38" customHeight="1">
@@ -2453,7 +4615,11 @@
           <t>A carico proprietario</t>
         </is>
       </c>
-      <c r="C47" s="14" t="inlineStr"/>
+      <c r="C47" s="34" t="inlineStr">
+        <is>
+          <t>Facoltativa: mono €70 / bilocale €100 / trilocale €150</t>
+        </is>
+      </c>
       <c r="D47" s="14" t="inlineStr"/>
     </row>
     <row r="48" ht="38" customHeight="1">
@@ -2467,7 +4633,11 @@
           <t>A carico proprietario</t>
         </is>
       </c>
-      <c r="C48" s="14" t="inlineStr"/>
+      <c r="C48" s="34" t="inlineStr">
+        <is>
+          <t>Non menzionato</t>
+        </is>
+      </c>
       <c r="D48" s="14" t="inlineStr"/>
     </row>
     <row r="49" ht="38" customHeight="1">
@@ -2481,7 +4651,11 @@
           <t>No – vietati</t>
         </is>
       </c>
-      <c r="C49" s="14" t="inlineStr"/>
+      <c r="C49" s="34" t="inlineStr">
+        <is>
+          <t>Non specificato (nessun divieto esplicito)</t>
+        </is>
+      </c>
       <c r="D49" s="14" t="inlineStr"/>
     </row>
     <row r="50" ht="38" customHeight="1">
@@ -2495,7 +4669,11 @@
           <t>Prodotti brand Italianway a carico PM</t>
         </is>
       </c>
-      <c r="C50" s="14" t="inlineStr"/>
+      <c r="C50" s="34" t="inlineStr">
+        <is>
+          <t>Nessun branding Youhosty in appartamento (non menzionato)</t>
+        </is>
+      </c>
       <c r="D50" s="14" t="inlineStr"/>
     </row>
     <row r="51" ht="20" customHeight="1">
@@ -2504,6 +4682,9 @@
           <t>▶  STRUTTURA AZIENDALE</t>
         </is>
       </c>
+      <c r="B51" s="24" t="n"/>
+      <c r="C51" s="24" t="n"/>
+      <c r="D51" s="25" t="n"/>
     </row>
     <row r="52" ht="38" customHeight="1">
       <c r="A52" s="5" t="inlineStr">
@@ -2516,7 +4697,12 @@
           <t>Franchising (Italianway SpA + affiliati locali)</t>
         </is>
       </c>
-      <c r="C52" s="14" t="inlineStr"/>
+      <c r="C52" s="34" t="inlineStr">
+        <is>
+          <t>Gestione diretta (non franchising)
+A.P.P.A. Srl Milano</t>
+        </is>
+      </c>
       <c r="D52" s="14" t="inlineStr"/>
     </row>
     <row r="53" ht="38" customHeight="1">
@@ -2530,7 +4716,11 @@
           <t>Milano, via Battistotti Sassi 11</t>
         </is>
       </c>
-      <c r="C53" s="14" t="inlineStr"/>
+      <c r="C53" s="34" t="inlineStr">
+        <is>
+          <t>Milano, via G. Pezzi 2 (cap 20135)</t>
+        </is>
+      </c>
       <c r="D53" s="14" t="inlineStr"/>
     </row>
     <row r="54" ht="38" customHeight="1">
@@ -2544,7 +4734,12 @@
           <t>Italianway SpA in mandato per il proprietario</t>
         </is>
       </c>
-      <c r="C54" s="14" t="inlineStr"/>
+      <c r="C54" s="34" t="inlineStr">
+        <is>
+          <t>Youhosty incassa per conto del cliente
+Oneri dovuti anche in caso di mancato incasso</t>
+        </is>
+      </c>
       <c r="D54" s="14" t="inlineStr"/>
     </row>
     <row r="55" ht="38" customHeight="1">
@@ -2558,17 +4753,22 @@
           <t>Versata da Italianway SpA in nome del proprietario</t>
         </is>
       </c>
-      <c r="C55" s="14" t="inlineStr"/>
+      <c r="C55" s="34" t="inlineStr">
+        <is>
+          <t>Solo per &lt;4 immobili e locazioni &lt;30 giorni
+Altrimenti obbligo torna al cliente</t>
+        </is>
+      </c>
       <c r="D55" s="14" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="8">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A31:D31"/>
-    <mergeCell ref="A11:D11"/>
     <mergeCell ref="A4:D4"/>
     <mergeCell ref="A41:D41"/>
     <mergeCell ref="A19:D19"/>
+    <mergeCell ref="A11:D11"/>
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="A51:D51"/>
   </mergeCells>
@@ -2576,7 +4776,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2598,6 +4798,10 @@
           <t>SCORECARD DECISIONALE – Punteggi comparativi (da compilare)</t>
         </is>
       </c>
+      <c r="B1" s="24" t="n"/>
+      <c r="C1" s="24" t="n"/>
+      <c r="D1" s="24" t="n"/>
+      <c r="E1" s="25" t="n"/>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="20" t="inlineStr">
@@ -2605,6 +4809,10 @@
           <t>Punteggio da 1 (pessimo) a 5 (ottimo) per ogni criterio. Peso in %. Totale ponderato calcolato automaticamente.</t>
         </is>
       </c>
+      <c r="B2" s="24" t="n"/>
+      <c r="C2" s="24" t="n"/>
+      <c r="D2" s="24" t="n"/>
+      <c r="E2" s="25" t="n"/>
     </row>
     <row r="3" ht="24" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
@@ -2617,9 +4825,9 @@
           <t>ITALIANWAY</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>AZIENDA B</t>
+      <c r="C3" s="33" t="inlineStr">
+        <is>
+          <t>YOUHOSTY</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
@@ -2644,11 +4852,16 @@
           <t>3</t>
         </is>
       </c>
-      <c r="C4" s="22" t="inlineStr"/>
+      <c r="C4" s="35" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="D4" s="22" t="inlineStr"/>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>Italianway: 25% ospite + 2% provv. – verificare vs mercato</t>
+          <t>Italianway: 25% ospite + 2% provv. – verificare vs mercato
+Youhosty: 16,5% + OTA (addebitata) + abbonamento mensile €19,90-26,90 + pratiche chiusura €470 → più costoso di quanto appare</t>
         </is>
       </c>
     </row>
@@ -2663,11 +4876,16 @@
           <t>4</t>
         </is>
       </c>
-      <c r="C5" s="22" t="inlineStr"/>
+      <c r="C5" s="35" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="D5" s="22" t="inlineStr"/>
       <c r="E5" s="10" t="inlineStr">
         <is>
-          <t>Costi abbastanza espliciti nel contratto</t>
+          <t>Costi abbastanza espliciti nel contratto
+Youhosty: prezzi espliciti ma molti componenti separati (OTA, mensile, chiusura) rendono difficile il calcolo del costo totale</t>
         </is>
       </c>
     </row>
@@ -2682,11 +4900,16 @@
           <t>2</t>
         </is>
       </c>
-      <c r="C6" s="22" t="inlineStr"/>
+      <c r="C6" s="35" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D6" s="22" t="inlineStr"/>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>Esclusiva + 3 mesi preavviso + rinnovo tacito = poco flessibile</t>
+          <t>Esclusiva + 3 mesi preavviso + rinnovo tacito = poco flessibile
+All-Inclusive 24 mesi, recesso solo forza maggiore, pratiche chiusura €470, penale accesso €50 → il meno flessibile</t>
         </is>
       </c>
     </row>
@@ -2701,11 +4924,16 @@
           <t>4</t>
         </is>
       </c>
-      <c r="C7" s="22" t="inlineStr"/>
+      <c r="C7" s="35" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
       <c r="D7" s="22" t="inlineStr"/>
       <c r="E7" s="10" t="inlineStr">
         <is>
-          <t>Check-in, pulizie, burocrazia gestiti; qualità PM locale da verificare</t>
+          <t>Check-in, pulizie, burocrazia gestiti; qualità PM locale da verificare
+Self check-in automatizzato, gestione completa, multilingual; gestione diretta (non franchising) → qualità più uniforme</t>
         </is>
       </c>
     </row>
@@ -2720,11 +4948,16 @@
           <t>4</t>
         </is>
       </c>
-      <c r="C8" s="22" t="inlineStr"/>
+      <c r="C8" s="35" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="D8" s="22" t="inlineStr"/>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>KALISI: real-time, algoritmo Revenue Management</t>
+          <t>KALISI: real-time, algoritmo Revenue Management
+App/sito proprietario con revenue management in outsourcing; meno descritto di KALISI ma funzionale</t>
         </is>
       </c>
     </row>
@@ -2739,11 +4972,16 @@
           <t>4</t>
         </is>
       </c>
-      <c r="C9" s="22" t="inlineStr"/>
+      <c r="C9" s="35" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="D9" s="22" t="inlineStr"/>
       <c r="E9" s="10" t="inlineStr">
         <is>
-          <t>Accesso KALISI; pagamento il 28 del mese</t>
+          <t>Accesso KALISI; pagamento il 28 del mese
+Reportistica per immobile disponibile; pagamento entro 30° mese; OTA addebitata separatamente aumenta complessità</t>
         </is>
       </c>
     </row>
@@ -2758,11 +4996,16 @@
           <t>3</t>
         </is>
       </c>
-      <c r="C10" s="22" t="inlineStr"/>
+      <c r="C10" s="35" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D10" s="22" t="inlineStr"/>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>RC €1M ottima; massimali incendio/furto nella media</t>
+          <t>RC €1M ottima; massimali incendio/furto nella media
+Nessuna polizza collettiva: solo cauzione piattaforma e consiglio di stipulare RC propria → rischio massimo per il proprietario</t>
         </is>
       </c>
     </row>
@@ -2777,11 +5020,16 @@
           <t>2</t>
         </is>
       </c>
-      <c r="C11" s="22" t="inlineStr"/>
+      <c r="C11" s="35" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
       <c r="D11" s="22" t="inlineStr"/>
       <c r="E11" s="10" t="inlineStr">
         <is>
-          <t>Lista dotazioni lunga; sicurezza e pulizia pre-shooting a carico proprietario</t>
+          <t>Lista dotazioni lunga; sicurezza e pulizia pre-shooting a carico proprietario
+Lista dotazioni non prescrittiva; meno obblighi iniziali; sicurezza in noleggio gestito da Youhosty</t>
         </is>
       </c>
     </row>
@@ -2796,11 +5044,16 @@
           <t>4</t>
         </is>
       </c>
-      <c r="C12" s="22" t="inlineStr"/>
+      <c r="C12" s="35" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="D12" s="22" t="inlineStr"/>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>Brand nazionale; franchising diffuso; dal 2014</t>
+          <t>Brand nazionale; franchising diffuso; dal 2014
+Brand riconoscibile a Milano; meno capillare di Italianway a livello nazionale</t>
         </is>
       </c>
     </row>
@@ -2815,11 +5068,16 @@
           <t>3</t>
         </is>
       </c>
-      <c r="C13" s="22" t="inlineStr"/>
+      <c r="C13" s="35" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="D13" s="22" t="inlineStr"/>
       <c r="E13" s="10" t="inlineStr">
         <is>
-          <t>Italianway SpA intermedia: dipendenza da solidità aziendale</t>
+          <t>Italianway SpA intermedia: dipendenza da solidità aziendale
+Oneri dovuti anche senza incasso; canone garantito disponibile (Allegato 3) ma non allegato</t>
         </is>
       </c>
     </row>
@@ -2834,11 +5092,16 @@
           <t>3</t>
         </is>
       </c>
-      <c r="C14" s="22" t="inlineStr"/>
+      <c r="C14" s="35" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="D14" s="22" t="inlineStr"/>
       <c r="E14" s="6" t="inlineStr">
         <is>
-          <t>Possibile ma con costi di ripristino non quantificati</t>
+          <t>Possibile ma con costi di ripristino non quantificati
+45 gg/anno All-Inclusive, fuori eventi principali; €15/gg extra; più gg rispetto a Italianway ma con limitazioni sui periodi</t>
         </is>
       </c>
     </row>
@@ -2853,11 +5116,16 @@
           <t>3</t>
         </is>
       </c>
-      <c r="C15" s="22" t="inlineStr"/>
+      <c r="C15" s="35" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
       <c r="D15" s="22" t="inlineStr"/>
       <c r="E15" s="10" t="inlineStr">
         <is>
-          <t>PM locale affiliato; qualità variabile per zona</t>
+          <t>PM locale affiliato; qualità variabile per zona
+Gestione diretta non franchise → interlocutore unico e stabile; abbonamento mensile con check-up periodico</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Easylife S.p.A. (Azienda C) data to comparison Excel
</commit_message>
<xml_diff>
--- a/Italianway_Analisi_Comparativa.xlsx
+++ b/Italianway_Analisi_Comparativa.xlsx
@@ -9,8 +9,9 @@
   <sheets>
     <sheet name="RIEPILOGO ITALIANWAY" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="RIEPILOGO YOUHOSTY" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="CONFRONTO 3 AZIENDE" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="SCORECARD DECISIONALE" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="RIEPILOGO EASYLIFE" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="CONFRONTO 3 AZIENDE" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="SCORECARD DECISIONALE" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -131,7 +132,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="23">
+  <fills count="24">
     <fill>
       <patternFill/>
     </fill>
@@ -243,6 +244,11 @@
         <fgColor rgb="00EBF5FB"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F0F7EE"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="6">
     <border>
@@ -314,7 +320,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -415,6 +421,12 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="22" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="23" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="23" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1991,6 +2003,9 @@
           <t>YOUHOSTY (A.P.P.A. Srl) – ANALISI COMPLETA</t>
         </is>
       </c>
+      <c r="B1" s="24" t="n"/>
+      <c r="C1" s="24" t="n"/>
+      <c r="D1" s="25" t="n"/>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="27" t="inlineStr">
@@ -1998,6 +2013,9 @@
           <t>Fonte: Contratto di Servizi v.2026 (A.P.P.A. Srl, Milano, P.IVA 09454690968) | Allegato 1 Scheda Comparazione</t>
         </is>
       </c>
+      <c r="B2" s="24" t="n"/>
+      <c r="C2" s="24" t="n"/>
+      <c r="D2" s="25" t="n"/>
     </row>
     <row r="3" ht="24" customHeight="1">
       <c r="A3" s="28" t="inlineStr">
@@ -2027,6 +2045,9 @@
           <t>🏢 STRUTTURA AZIENDALE</t>
         </is>
       </c>
+      <c r="B4" s="24" t="n"/>
+      <c r="C4" s="24" t="n"/>
+      <c r="D4" s="25" t="n"/>
     </row>
     <row r="5" ht="40" customHeight="1">
       <c r="A5" s="30" t="inlineStr">
@@ -2122,6 +2143,9 @@
           <t>📦 STRUTTURA DEI PACCHETTI</t>
         </is>
       </c>
+      <c r="B9" s="24" t="n"/>
+      <c r="C9" s="24" t="n"/>
+      <c r="D9" s="25" t="n"/>
     </row>
     <row r="10" ht="40" customHeight="1">
       <c r="A10" s="30" t="inlineStr">
@@ -2239,6 +2263,9 @@
           <t>💶 SETUP FEE (una tantum, IVA esclusa – valori All-Inclusive con pagamento anticipato)</t>
         </is>
       </c>
+      <c r="B15" s="24" t="n"/>
+      <c r="C15" s="24" t="n"/>
+      <c r="D15" s="25" t="n"/>
     </row>
     <row r="16" ht="40" customHeight="1">
       <c r="A16" s="30" t="inlineStr">
@@ -2422,6 +2449,9 @@
           <t>💰 COMMISSIONI – LOCAZIONI BREVI (% sul corrispettivo pagato dall'ospite, IVA esclusa)</t>
         </is>
       </c>
+      <c r="B24" s="24" t="n"/>
+      <c r="C24" s="24" t="n"/>
+      <c r="D24" s="25" t="n"/>
     </row>
     <row r="25" ht="40" customHeight="1">
       <c r="A25" s="30" t="inlineStr">
@@ -2585,6 +2615,9 @@
           <t>💰 COMMISSIONI – LOCAZIONI MEDIO/LUNGO TERMINE</t>
         </is>
       </c>
+      <c r="B33" s="24" t="n"/>
+      <c r="C33" s="24" t="n"/>
+      <c r="D33" s="25" t="n"/>
     </row>
     <row r="34" ht="40" customHeight="1">
       <c r="A34" s="30" t="inlineStr">
@@ -2712,6 +2745,9 @@
           <t>📅 ABBONAMENTO MENSILE MANUTENZIONE (IVA esclusa)</t>
         </is>
       </c>
+      <c r="B40" s="24" t="n"/>
+      <c r="C40" s="24" t="n"/>
+      <c r="D40" s="25" t="n"/>
     </row>
     <row r="41" ht="40" customHeight="1">
       <c r="A41" s="30" t="inlineStr">
@@ -2821,6 +2857,9 @@
           <t>📄 CONTRATTO, DURATA E RECESSO</t>
         </is>
       </c>
+      <c r="B46" s="24" t="n"/>
+      <c r="C46" s="24" t="n"/>
+      <c r="D46" s="25" t="n"/>
     </row>
     <row r="47" ht="40" customHeight="1">
       <c r="A47" s="30" t="inlineStr">
@@ -3042,6 +3081,9 @@
           <t>🏠 USO PERSONALE DELL'IMMOBILE</t>
         </is>
       </c>
+      <c r="B58" s="24" t="n"/>
+      <c r="C58" s="24" t="n"/>
+      <c r="D58" s="25" t="n"/>
     </row>
     <row r="59" ht="40" customHeight="1">
       <c r="A59" s="30" t="inlineStr">
@@ -3107,6 +3149,9 @@
           <t>🛎️ SERVIZI INCLUSI (pacchetto All-Inclusive)</t>
         </is>
       </c>
+      <c r="B62" s="24" t="n"/>
+      <c r="C62" s="24" t="n"/>
+      <c r="D62" s="25" t="n"/>
     </row>
     <row r="63" ht="40" customHeight="1">
       <c r="A63" s="30" t="inlineStr">
@@ -3304,6 +3349,9 @@
           <t>🛡️ GARANZIA DANNI E ASSICURAZIONE</t>
         </is>
       </c>
+      <c r="B72" s="24" t="n"/>
+      <c r="C72" s="24" t="n"/>
+      <c r="D72" s="25" t="n"/>
     </row>
     <row r="73" ht="40" customHeight="1">
       <c r="A73" s="30" t="inlineStr">
@@ -3449,6 +3497,9 @@
           <t>📋 OBBLIGHI E ONERI DEL CLIENTE</t>
         </is>
       </c>
+      <c r="B80" s="24" t="n"/>
+      <c r="C80" s="24" t="n"/>
+      <c r="D80" s="25" t="n"/>
     </row>
     <row r="81" ht="40" customHeight="1">
       <c r="A81" s="30" t="inlineStr">
@@ -3604,6 +3655,9 @@
           <t>🔧 SERVIZI A RICHIESTA (IVA esclusa)</t>
         </is>
       </c>
+      <c r="B89" s="24" t="n"/>
+      <c r="C89" s="24" t="n"/>
+      <c r="D89" s="25" t="n"/>
     </row>
     <row r="90" ht="40" customHeight="1">
       <c r="A90" s="30" t="inlineStr">
@@ -3737,6 +3791,9 @@
           <t>🏡 COMMISSIONE COMPRAVENDITA</t>
         </is>
       </c>
+      <c r="B97" s="24" t="n"/>
+      <c r="C97" s="24" t="n"/>
+      <c r="D97" s="25" t="n"/>
     </row>
     <row r="98" ht="40" customHeight="1">
       <c r="A98" s="30" t="inlineStr">
@@ -3806,6 +3863,1189 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:D64"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="52" customWidth="1" min="2" max="2"/>
+    <col width="46" customWidth="1" min="3" max="3"/>
+    <col width="46" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="36" customHeight="1">
+      <c r="A1" s="26" t="inlineStr">
+        <is>
+          <t>EASYLIFE S.p.A. – ANALISI COMPLETA</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="27" t="inlineStr">
+        <is>
+          <t>Fonte: Mandato di Gestione per Affitti Brevi (Easylife S.p.A., Via G.B. Pergolesi 26, 20124 Milano, P.IVA 09640480969)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="24" customHeight="1">
+      <c r="A3" s="28" t="inlineStr">
+        <is>
+          <t>CATEGORIA / VOCE</t>
+        </is>
+      </c>
+      <c r="B3" s="28" t="inlineStr">
+        <is>
+          <t>DETTAGLIO / VALORE</t>
+        </is>
+      </c>
+      <c r="C3" s="28" t="inlineStr">
+        <is>
+          <t>PRO (+)</t>
+        </is>
+      </c>
+      <c r="D3" s="28" t="inlineStr">
+        <is>
+          <t>CONTRO (–)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="29" t="inlineStr">
+        <is>
+          <t>🏢 STRUTTURA AZIENDALE</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="40" customHeight="1">
+      <c r="A5" s="30" t="inlineStr">
+        <is>
+          <t>Società</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>Easylife S.p.A. – Via G.B. Pergolesi 26, 20124 Milano | P.IVA 09640480969 | REA MI-2103718</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>Società per Azioni (maggiore stabilità patrimoniale rispetto a Srl/startup)</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>Meno informazioni pubbliche disponibili sul track record operativo</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="40" customHeight="1">
+      <c r="A6" s="31" t="inlineStr">
+        <is>
+          <t>Rappresentante legale</t>
+        </is>
+      </c>
+      <c r="B6" s="32" t="inlineStr">
+        <is>
+          <t>Donato Cella (nato Potenza 15/07/1981 – CF: CLLDNT81L15G942G)</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>Responsabilità e interlocutore identificati nel contratto</t>
+        </is>
+      </c>
+      <c r="D6" s="32" t="inlineStr"/>
+    </row>
+    <row r="7" ht="40" customHeight="1">
+      <c r="A7" s="30" t="inlineStr">
+        <is>
+          <t>Marchio</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>Easylife House (portale OTA proprietario incluso)</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>Portale proprietario aggiuntivo rispetto a soli OTA terzi</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr"/>
+    </row>
+    <row r="8" ht="40" customHeight="1">
+      <c r="A8" s="31" t="inlineStr">
+        <is>
+          <t>Modello operativo</t>
+        </is>
+      </c>
+      <c r="B8" s="32" t="inlineStr">
+        <is>
+          <t>Gestione diretta con partner/collaboratori</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>Flessibilità nell'esecuzione con partner specializzati</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>Il PM può avvalersi di terzi per l'esecuzione: qualità dipendente dai partner</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="29" t="inlineStr">
+        <is>
+          <t>💰 COMMISSIONI E CORRISPETTIVO</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="40" customHeight="1">
+      <c r="A10" s="30" t="inlineStr">
+        <is>
+          <t>Commissione base</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>25% + IVA sul netto prenotazione (netto OTA, netto pulizie, netto biancheria)
+Opzione 'Senza Pensieri': 27,5% + IVA</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>Calcolo sulla prenotazione netta: OTA e pulizie già scorporate prima della commissione</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>La commissione base è simile a Italianway (25%) ma con basi diverse – verificare il netto effettivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="40" customHeight="1">
+      <c r="A11" s="31" t="inlineStr">
+        <is>
+          <t>Commissione OTA</t>
+        </is>
+      </c>
+      <c r="B11" s="32" t="inlineStr">
+        <is>
+          <t>OTA (Airbnb, Booking, ecc.) addebitate all'OSPITE separatamente</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>Il proprietario non anticipa le commissioni OTA</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>Le OTA vengono comunque sostenute dall'ospite: impatto sul prezzo totale del soggiorno</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="40" customHeight="1">
+      <c r="A12" s="30" t="inlineStr">
+        <is>
+          <t>Pulizie e biancheria</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>Addebitate all'ospite separatamente (escluse dalla base commissionale)</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>Costo pulizie non a carico del proprietario</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>Il prezzo totale per l'ospite è più alto → potenziale impatto sulla competitività</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="40" customHeight="1">
+      <c r="A13" s="31" t="inlineStr">
+        <is>
+          <t>Formula 'Senza Pensieri'</t>
+        </is>
+      </c>
+      <c r="B13" s="32" t="inlineStr">
+        <is>
+          <t>Opzionale: +2,5% sulla commissione → 27,5% totale
+Copre piccole manutenzioni e sostituzione accessori (lista dettagliata in Allegato C)</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>Trasparenza sul costo della copertura manutenzioni
+Evita costi inaspettati per piccoli interventi e sostituzione oggetti comuni</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>Costo aggiuntivo ricorrente su ogni prenotazione anche se non servono interventi in quel mese</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="40" customHeight="1">
+      <c r="A14" s="30" t="inlineStr">
+        <is>
+          <t>Commissione per compravendita</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>2% del prezzo di vendita (tramite agenzia partner obbligatoria)</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>Nessuna richiesta aggiuntiva rispetto al mercato per la mediazione</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>Il proprietario è obbligato a usare l'agenzia partner: perde libertà nella scelta del mediatore</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="29" t="inlineStr">
+        <is>
+          <t>💶 COSTI DI AVVIO (UNA TANTUM, IVA esclusa salvo indicazione)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="40" customHeight="1">
+      <c r="A16" s="30" t="inlineStr">
+        <is>
+          <t>Pratiche amministrative / setup iniziale</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>€300 (trattenuto dal primo bonifico del primo mese)</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>Nessun pagamento anticipato: trattenuto dai primi incassi</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>Costo presente ma non disaggregato (pratiche CAV, SUAP, adempimenti vari inclusi)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="40" customHeight="1">
+      <c r="A17" s="31" t="inlineStr">
+        <is>
+          <t>Fotografia professionale</t>
+        </is>
+      </c>
+      <c r="B17" s="32" t="inlineStr">
+        <is>
+          <t>€140 + IVA</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>Obbligatoria prima dell'avvio; prezzo nella media di mercato</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>Costo separato; in Italianway incluso nel corrispettivo unico €600+IVA</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="40" customHeight="1">
+      <c r="A18" s="30" t="inlineStr">
+        <is>
+          <t>Sostituzione cilindro serratura</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>€195,57 IVA inclusa (inclusa reinstallazione originale al termine)</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>Al termine del contratto il cilindro originale viene ripristinato senza costi aggiuntivi</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>Costo iniziale non trascurabile; la serratura viene sostituita anche solo temporaneamente</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="40" customHeight="1">
+      <c r="A19" s="31" t="inlineStr">
+        <is>
+          <t>Installazione key box (videocitofono + cassettina)</t>
+        </is>
+      </c>
+      <c r="B19" s="32" t="inlineStr">
+        <is>
+          <t>€185 + IVA (+ €150 IVA se necessario sostituire anche il citofono)</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>Gestione accesso autonomo ospiti senza intervento fisico</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>Costo a carico del proprietario; dipende dalla struttura dell'immobile</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="40" customHeight="1">
+      <c r="A20" s="30" t="inlineStr">
+        <is>
+          <t>Costo totale avvio indicativo</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>~€300 + €140+IVA + €195,57 + €185+IVA ≈ €820+ IVA escl.</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>Costi ben documentati nel contratto</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>Costo totale avvio più alto rispetto a Youhosty All-Inclusive (~€437) ma in linea con Italianway (~€600)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="29" t="inlineStr">
+        <is>
+          <t>📄 CONTRATTO, DURATA E RECESSO</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="40" customHeight="1">
+      <c r="A22" s="30" t="inlineStr">
+        <is>
+          <t>Durata contratto</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>18 mesi dalla prima prenotazione ricevuta, rinnovabile automaticamente per ulteriori 18 mesi</t>
+        </is>
+      </c>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>Durata intermedia: meno vincolante di Youhosty (24 mesi), più di Italianway (12 mesi)</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="inlineStr">
+        <is>
+          <t>Rinnovo automatico: rischio di restare vincolati se non si disdice per tempo</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="40" customHeight="1">
+      <c r="A23" s="31" t="inlineStr">
+        <is>
+          <t>Preavviso disdetta</t>
+        </is>
+      </c>
+      <c r="B23" s="32" t="inlineStr">
+        <is>
+          <t>90 giorni prima di ciascuna scadenza (raccomandata a/r o PEC)</t>
+        </is>
+      </c>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>Preavviso chiaro e documentato</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>90 giorni = 3 mesi: obbligo di pianificazione anticipata</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="40" customHeight="1">
+      <c r="A24" s="30" t="inlineStr">
+        <is>
+          <t>Recesso anticipato PM</t>
+        </is>
+      </c>
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>Il PM può recedere con 30 giorni di preavviso (raccomandata o PEC)</t>
+        </is>
+      </c>
+      <c r="C24" s="7" t="inlineStr">
+        <is>
+          <t>PM può uscire rapidamente in caso di problemi</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="inlineStr">
+        <is>
+          <t>Asimmetria: il PM ha grande flessibilità di uscita, il cliente no</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="40" customHeight="1">
+      <c r="A25" s="31" t="inlineStr">
+        <is>
+          <t>Recesso anticipato cliente</t>
+        </is>
+      </c>
+      <c r="B25" s="32" t="inlineStr">
+        <is>
+          <t>Non previsto esplicitamente nel contratto ricevuto</t>
+        </is>
+      </c>
+      <c r="C25" s="32" t="inlineStr"/>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>Nessuna clausola di recesso anticipato per il cliente → vincolato per tutta la durata</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="40" customHeight="1">
+      <c r="A26" s="30" t="inlineStr">
+        <is>
+          <t>Costo uscita contratto</t>
+        </is>
+      </c>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>Non previste penali esplicite di uscita (a differenza di Youhosty €470)</t>
+        </is>
+      </c>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>Nessuna exit fee dichiarata → vantaggio significativo rispetto a Youhosty</t>
+        </is>
+      </c>
+      <c r="D26" s="8" t="inlineStr">
+        <is>
+          <t>Le prenotazioni a scavalco devono essere onorate da entrambe le parti</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="40" customHeight="1">
+      <c r="A27" s="31" t="inlineStr">
+        <is>
+          <t>Prenotazioni post-recesso</t>
+        </is>
+      </c>
+      <c r="B27" s="32" t="inlineStr">
+        <is>
+          <t>Entrambe le parti obbligate a onorare prenotazioni concluse prima del recesso</t>
+        </is>
+      </c>
+      <c r="C27" s="7" t="inlineStr">
+        <is>
+          <t>Tutela reciproca e trasparenza</t>
+        </is>
+      </c>
+      <c r="D27" s="32" t="inlineStr"/>
+    </row>
+    <row r="28" ht="40" customHeight="1">
+      <c r="A28" s="30" t="inlineStr">
+        <is>
+          <t>Esclusiva</t>
+        </is>
+      </c>
+      <c r="B28" s="6" t="inlineStr">
+        <is>
+          <t>Mandato irrevocabile con esclusiva (Art. 2.1)</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="inlineStr"/>
+      <c r="D28" s="8" t="inlineStr">
+        <is>
+          <t>Il proprietario non può gestire l'immobile in proprio o con altri gestori per tutta la durata</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="40" customHeight="1">
+      <c r="A29" s="31" t="inlineStr">
+        <is>
+          <t>Penale accesso non autorizzato</t>
+        </is>
+      </c>
+      <c r="B29" s="32" t="inlineStr">
+        <is>
+          <t>Trattenuta INTEGRALE degli incassi del mese successivo + risoluzione immediata + risarcimento danni</t>
+        </is>
+      </c>
+      <c r="C29" s="32" t="inlineStr"/>
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>Penale estremamente severa: anche un accesso emergenziale non notificato comporta perdita di tutti gli incassi mensili</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="20" customHeight="1">
+      <c r="A30" s="29" t="inlineStr">
+        <is>
+          <t>🏠 USO PERSONALE DELL'IMMOBILE</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="40" customHeight="1">
+      <c r="A31" s="30" t="inlineStr">
+        <is>
+          <t>Giorni uso personale</t>
+        </is>
+      </c>
+      <c r="B31" s="6" t="inlineStr">
+        <is>
+          <t>Max 30 giorni/anno totali (previa richiesta scritta 15 gg prima via email)</t>
+        </is>
+      </c>
+      <c r="C31" s="7" t="inlineStr">
+        <is>
+          <t>30 giorni in linea con Italianway; flessibile (non limitato a periodi specifici)</t>
+        </is>
+      </c>
+      <c r="D31" s="8" t="inlineStr">
+        <is>
+          <t>Se le date prescelte sono già prenotate, il PM propone alternative → nessuna garanzia sulle date preferite</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="40" customHeight="1">
+      <c r="A32" s="31" t="inlineStr">
+        <is>
+          <t>Procedura uso personale</t>
+        </is>
+      </c>
+      <c r="B32" s="32" t="inlineStr">
+        <is>
+          <t>Email a booking@easylife.house e amministrazione@easylife.house con check-in/out esatti</t>
+        </is>
+      </c>
+      <c r="C32" s="7" t="inlineStr">
+        <is>
+          <t>Procedura chiara e documentata via email</t>
+        </is>
+      </c>
+      <c r="D32" s="8" t="inlineStr">
+        <is>
+          <t>Obbligo di preavviso scritto di 15 giorni: non adatto a usi spontanei</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="40" customHeight="1">
+      <c r="A33" s="30" t="inlineStr">
+        <is>
+          <t>Costo uso personale</t>
+        </is>
+      </c>
+      <c r="B33" s="6" t="inlineStr">
+        <is>
+          <t>Solo spese di pulizia addebitate al cliente</t>
+        </is>
+      </c>
+      <c r="C33" s="7" t="inlineStr">
+        <is>
+          <t>Nessun costo giornaliero aggiuntivo (a differenza di Youhosty €15/gg)</t>
+        </is>
+      </c>
+      <c r="D33" s="8" t="inlineStr">
+        <is>
+          <t>Le pulizie rimangono a carico</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="20" customHeight="1">
+      <c r="A34" s="29" t="inlineStr">
+        <is>
+          <t>🛎️ SERVIZI INCLUSI NEL MANDATO</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="40" customHeight="1">
+      <c r="A35" s="30" t="inlineStr">
+        <is>
+          <t>Piattaforma monitoraggio</t>
+        </is>
+      </c>
+      <c r="B35" s="6" t="inlineStr">
+        <is>
+          <t>Portale web per controllo andamento, spettanze cliente e PM</t>
+        </is>
+      </c>
+      <c r="C35" s="7" t="inlineStr">
+        <is>
+          <t>Strumento di controllo in tempo reale</t>
+        </is>
+      </c>
+      <c r="D35" s="8" t="inlineStr">
+        <is>
+          <t>Caratteristiche non descritte in dettaglio; da verificare le funzionalità rispetto a KALISI</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="40" customHeight="1">
+      <c r="A36" s="31" t="inlineStr">
+        <is>
+          <t>Revenue management / pricing</t>
+        </is>
+      </c>
+      <c r="B36" s="32" t="inlineStr">
+        <is>
+          <t>Il PM determina liberamente i prezzi in base al mercato (art. 2.2)</t>
+        </is>
+      </c>
+      <c r="C36" s="7" t="inlineStr">
+        <is>
+          <t>Gestione professionale della tariffazione dinamica</t>
+        </is>
+      </c>
+      <c r="D36" s="8" t="inlineStr">
+        <is>
+          <t>Il cliente non può interferire nella scelta dei prezzi: zero controllo sul pricing</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="40" customHeight="1">
+      <c r="A37" s="30" t="inlineStr">
+        <is>
+          <t>Pubblicazione OTA</t>
+        </is>
+      </c>
+      <c r="B37" s="6" t="inlineStr">
+        <is>
+          <t>Gestione su OTA multiple incluso il portale proprietario Easylife House</t>
+        </is>
+      </c>
+      <c r="C37" s="7" t="inlineStr">
+        <is>
+          <t>Canale aggiuntivo proprietario rispetto a sole OTA terze</t>
+        </is>
+      </c>
+      <c r="D37" s="8" t="inlineStr">
+        <is>
+          <t>OTA non nominate esplicitamente nel contratto</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="40" customHeight="1">
+      <c r="A38" s="31" t="inlineStr">
+        <is>
+          <t>Check-in / check-out</t>
+        </is>
+      </c>
+      <c r="B38" s="32" t="inlineStr">
+        <is>
+          <t>Remoto/automatizzato (key box) o su richiesta con staff</t>
+        </is>
+      </c>
+      <c r="C38" s="7" t="inlineStr">
+        <is>
+          <t>Gestione autonoma ospiti senza personale fisico</t>
+        </is>
+      </c>
+      <c r="D38" s="32" t="inlineStr"/>
+    </row>
+    <row r="39" ht="40" customHeight="1">
+      <c r="A39" s="30" t="inlineStr">
+        <is>
+          <t>Comunicazioni autorità (Questura, ecc.)</t>
+        </is>
+      </c>
+      <c r="B39" s="6" t="inlineStr">
+        <is>
+          <t>Incluse nel mandato (art. 2.1 e procura speciale)</t>
+        </is>
+      </c>
+      <c r="C39" s="7" t="inlineStr">
+        <is>
+          <t>Burocrazia delegata al PM; procura speciale inclusa nel contratto</t>
+        </is>
+      </c>
+      <c r="D39" s="6" t="inlineStr"/>
+    </row>
+    <row r="40" ht="40" customHeight="1">
+      <c r="A40" s="31" t="inlineStr">
+        <is>
+          <t>Tassa di soggiorno</t>
+        </is>
+      </c>
+      <c r="B40" s="32" t="inlineStr">
+        <is>
+          <t>Incasso e versamento gestiti dal PM (art. 2.1)</t>
+        </is>
+      </c>
+      <c r="C40" s="7" t="inlineStr">
+        <is>
+          <t>Obbligo fiscale delegato</t>
+        </is>
+      </c>
+      <c r="D40" s="32" t="inlineStr"/>
+    </row>
+    <row r="41" ht="40" customHeight="1">
+      <c r="A41" s="30" t="inlineStr">
+        <is>
+          <t>Gestione fiscale (ritenuta 21%)</t>
+        </is>
+      </c>
+      <c r="B41" s="6" t="inlineStr">
+        <is>
+          <t>PM effettua ritenuta 21% e rilascia CU annuale</t>
+        </is>
+      </c>
+      <c r="C41" s="7" t="inlineStr">
+        <is>
+          <t>Obbligo di sostituto d'imposta assolto dal PM</t>
+        </is>
+      </c>
+      <c r="D41" s="8" t="inlineStr">
+        <is>
+          <t>Il PM non offre consulenza fiscale: verifica regime cedolare secca a carico del cliente</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="40" customHeight="1">
+      <c r="A42" s="31" t="inlineStr">
+        <is>
+          <t>Pagamento saldo proprietario</t>
+        </is>
+      </c>
+      <c r="B42" s="32" t="inlineStr">
+        <is>
+          <t>Entro il 20° del mese successivo all'incasso (conteggio per data check-in)</t>
+        </is>
+      </c>
+      <c r="C42" s="7" t="inlineStr">
+        <is>
+          <t>Pagamento mensile regolare e termine chiaro</t>
+        </is>
+      </c>
+      <c r="D42" s="8" t="inlineStr">
+        <is>
+          <t>Possibile attesa fino a ~50 gg per soggiorni avvenuti a fine mese</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="40" customHeight="1">
+      <c r="A43" s="30" t="inlineStr">
+        <is>
+          <t>Manutenzione ordinaria</t>
+        </is>
+      </c>
+      <c r="B43" s="6" t="inlineStr">
+        <is>
+          <t>PM autorizzato a spendere fino a €200+IVA per intervento senza consenso preventivo del cliente</t>
+        </is>
+      </c>
+      <c r="C43" s="7" t="inlineStr">
+        <is>
+          <t>Rapidità di intervento per piccole urgenze</t>
+        </is>
+      </c>
+      <c r="D43" s="8" t="inlineStr">
+        <is>
+          <t>Soglia €200 senza consenso è alta; rischio di costi ribaltati senza preavviso</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="40" customHeight="1">
+      <c r="A44" s="31" t="inlineStr">
+        <is>
+          <t>Manutenzione straordinaria</t>
+        </is>
+      </c>
+      <c r="B44" s="32" t="inlineStr">
+        <is>
+          <t>Previa autorizzazione scritta del cliente; rimborso mediante compensazione con corrispettivo</t>
+        </is>
+      </c>
+      <c r="C44" s="32" t="inlineStr"/>
+      <c r="D44" s="32" t="inlineStr"/>
+    </row>
+    <row r="45" ht="40" customHeight="1">
+      <c r="A45" s="30" t="inlineStr">
+        <is>
+          <t>Segnalazione danni</t>
+        </is>
+      </c>
+      <c r="B45" s="6" t="inlineStr">
+        <is>
+          <t>Obbligo del PM di segnalare danni e attivare richieste di risarcimento OTA</t>
+        </is>
+      </c>
+      <c r="C45" s="7" t="inlineStr">
+        <is>
+          <t>Attivazione procedure di rimborso delegata</t>
+        </is>
+      </c>
+      <c r="D45" s="8" t="inlineStr">
+        <is>
+          <t>Nessuna garanzia di recupero effettivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="20" customHeight="1">
+      <c r="A46" s="29" t="inlineStr">
+        <is>
+          <t>🛡️ GARANZIA DANNI E ASSICURAZIONE</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="40" customHeight="1">
+      <c r="A47" s="30" t="inlineStr">
+        <is>
+          <t>Assicurazione fornita da Easylife</t>
+        </is>
+      </c>
+      <c r="B47" s="6" t="inlineStr">
+        <is>
+          <t>NESSUNA – il cliente deve stipulare a proprie spese una polizza a copertura dell'immobile e della destinazione casa vacanza (art. 10.3)</t>
+        </is>
+      </c>
+      <c r="C47" s="6" t="inlineStr"/>
+      <c r="D47" s="8" t="inlineStr">
+        <is>
+          <t>Nessuna polizza collettiva: il proprietario è completamente esposto a danni, incendio, furto, RC terzi</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="40" customHeight="1">
+      <c r="A48" s="31" t="inlineStr">
+        <is>
+          <t>Responsabilità Easylife per danni ospiti</t>
+        </is>
+      </c>
+      <c r="B48" s="32" t="inlineStr">
+        <is>
+          <t>Esonero esplicito da responsabilità contrattuale ed extracontrattuale per danni causati dagli ospiti (art. 10.1)</t>
+        </is>
+      </c>
+      <c r="C48" s="32" t="inlineStr"/>
+      <c r="D48" s="8" t="inlineStr">
+        <is>
+          <t>Massima esposizione del proprietario: nessun filtro assicurativo fornito dal PM</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="40" customHeight="1">
+      <c r="A49" s="30" t="inlineStr">
+        <is>
+          <t>Responsabilità Easylife per staff</t>
+        </is>
+      </c>
+      <c r="B49" s="6" t="inlineStr">
+        <is>
+          <t>Il PM è responsabile per danni arrecati dal proprio staff (art. 10.4)</t>
+        </is>
+      </c>
+      <c r="C49" s="7" t="inlineStr">
+        <is>
+          <t>Tutela per danni operativi causati dal personale Easylife</t>
+        </is>
+      </c>
+      <c r="D49" s="6" t="inlineStr"/>
+    </row>
+    <row r="50" ht="40" customHeight="1">
+      <c r="A50" s="31" t="inlineStr">
+        <is>
+          <t>Cauzione / deposito ospite</t>
+        </is>
+      </c>
+      <c r="B50" s="32" t="inlineStr">
+        <is>
+          <t>Non menzionata esplicitamente (dipende dalle policy OTA)</t>
+        </is>
+      </c>
+      <c r="C50" s="32" t="inlineStr"/>
+      <c r="D50" s="8" t="inlineStr">
+        <is>
+          <t>Nessuna cauzione standardizzata: protezione variabile per piattaforma</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="40" customHeight="1">
+      <c r="A51" s="30" t="inlineStr">
+        <is>
+          <t>Formula Senza Pensieri – copertura danni</t>
+        </is>
+      </c>
+      <c r="B51" s="6" t="inlineStr">
+        <is>
+          <t>Copre solo piccole manutenzioni e accessori (list. All. C); NON copre danni ospiti o eventi</t>
+        </is>
+      </c>
+      <c r="C51" s="7" t="inlineStr">
+        <is>
+          <t>Riduce costi operativi correnti</t>
+        </is>
+      </c>
+      <c r="D51" s="8" t="inlineStr">
+        <is>
+          <t>Non è un'assicurazione: non copre danni strutturali né responsabilità verso terzi</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="20" customHeight="1">
+      <c r="A52" s="29" t="inlineStr">
+        <is>
+          <t>📋 OBBLIGHI E ONERI DEL CLIENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="40" customHeight="1">
+      <c r="A53" s="30" t="inlineStr">
+        <is>
+          <t>Chiavi da consegnare</t>
+        </is>
+      </c>
+      <c r="B53" s="6" t="inlineStr">
+        <is>
+          <t>4 mazzi (oppure 1 con key box installata)</t>
+        </is>
+      </c>
+      <c r="C53" s="7" t="inlineStr">
+        <is>
+          <t>Meno mazzi rispetto a Italianway (6) e Youhosty (5)</t>
+        </is>
+      </c>
+      <c r="D53" s="6" t="inlineStr"/>
+    </row>
+    <row r="54" ht="40" customHeight="1">
+      <c r="A54" s="31" t="inlineStr">
+        <is>
+          <t>TARI, utenze, canone RAI</t>
+        </is>
+      </c>
+      <c r="B54" s="32" t="inlineStr">
+        <is>
+          <t>A carico del cliente (art. 3.2 e 3.9)</t>
+        </is>
+      </c>
+      <c r="C54" s="32" t="inlineStr"/>
+      <c r="D54" s="8" t="inlineStr">
+        <is>
+          <t>A differenza di Italianway dove alcune voci sono incluse nel canone</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="40" customHeight="1">
+      <c r="A55" s="30" t="inlineStr">
+        <is>
+          <t>Connessione Internet</t>
+        </is>
+      </c>
+      <c r="B55" s="6" t="inlineStr">
+        <is>
+          <t>A carico del cliente – min. 100 Mbps o la più veloce disponibile in zona; obbligatoria e gratuita per ospiti</t>
+        </is>
+      </c>
+      <c r="C55" s="7" t="inlineStr">
+        <is>
+          <t>Requisito standard e chiaramente indicato</t>
+        </is>
+      </c>
+      <c r="D55" s="6" t="inlineStr"/>
+    </row>
+    <row r="56" ht="40" customHeight="1">
+      <c r="A56" s="31" t="inlineStr">
+        <is>
+          <t>Stato immobile e impianti</t>
+        </is>
+      </c>
+      <c r="B56" s="32" t="inlineStr">
+        <is>
+          <t>Conformità normativa obbligatoria (abitabilità, impianti, sicurezza); manleva del PM in caso di controlli</t>
+        </is>
+      </c>
+      <c r="C56" s="32" t="inlineStr"/>
+      <c r="D56" s="8" t="inlineStr">
+        <is>
+          <t>Il cliente risponde personalmente per violazioni normative anche in assenza di colpa</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="40" customHeight="1">
+      <c r="A57" s="30" t="inlineStr">
+        <is>
+          <t>Dotazione iniziale immobile</t>
+        </is>
+      </c>
+      <c r="B57" s="6" t="inlineStr">
+        <is>
+          <t>Standard Easylife descritti nell'Allegato A (scheda alloggio)</t>
+        </is>
+      </c>
+      <c r="C57" s="7" t="inlineStr">
+        <is>
+          <t>Standard definiti dal PM per qualità commerciale</t>
+        </is>
+      </c>
+      <c r="D57" s="8" t="inlineStr">
+        <is>
+          <t>Il cliente acquista le dotazioni mancanti prima dello shooting fotografico (costo a carico)</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="40" customHeight="1">
+      <c r="A58" s="31" t="inlineStr">
+        <is>
+          <t>APE e visura catastale</t>
+        </is>
+      </c>
+      <c r="B58" s="32" t="inlineStr">
+        <is>
+          <t>A carico del cliente (obbligatorie per locazioni)</t>
+        </is>
+      </c>
+      <c r="C58" s="32" t="inlineStr"/>
+      <c r="D58" s="32" t="inlineStr"/>
+    </row>
+    <row r="59" ht="40" customHeight="1">
+      <c r="A59" s="30" t="inlineStr">
+        <is>
+          <t>Vendita immobile</t>
+        </is>
+      </c>
+      <c r="B59" s="6" t="inlineStr">
+        <is>
+          <t>Obbligo di usare agenzia partner Easylife (commissione 2%)</t>
+        </is>
+      </c>
+      <c r="C59" s="6" t="inlineStr"/>
+      <c r="D59" s="8" t="inlineStr">
+        <is>
+          <t>Il proprietario perde la libertà di scelta dell'agente immobiliare</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="40" customHeight="1">
+      <c r="A60" s="31" t="inlineStr">
+        <is>
+          <t>Spese accessorie PM non incluse</t>
+        </is>
+      </c>
+      <c r="B60" s="32" t="inlineStr">
+        <is>
+          <t>Costi extra documentati (es. autorizzazioni, licenze) trattenuti alla prima contabilità utile</t>
+        </is>
+      </c>
+      <c r="C60" s="7" t="inlineStr">
+        <is>
+          <t>Trasparenza contabile</t>
+        </is>
+      </c>
+      <c r="D60" s="8" t="inlineStr">
+        <is>
+          <t>Costi potenziali non preventivabili al momento della firma</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="20" customHeight="1">
+      <c r="A61" s="29" t="inlineStr">
+        <is>
+          <t>🔧 FORMULA 'SENZA PENSIERI' (opzionale, +2,5% sulla commissione)</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="40" customHeight="1">
+      <c r="A62" s="30" t="inlineStr">
+        <is>
+          <t>Piccole manutenzioni incluse</t>
+        </is>
+      </c>
+      <c r="B62" s="6" t="inlineStr">
+        <is>
+          <t>Lampadine, pile, maniglie, tapparelle, guarnizioni, copriasse WC, ritassellature accessori, ecc.</t>
+        </is>
+      </c>
+      <c r="C62" s="7" t="inlineStr">
+        <is>
+          <t>Eliminazione di piccoli costi inaspettati e frequenti</t>
+        </is>
+      </c>
+      <c r="D62" s="8" t="inlineStr">
+        <is>
+          <t>Solo manutenzioni di piccola entità; danni strutturali o elettrici esclusi</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="40" customHeight="1">
+      <c r="A63" s="31" t="inlineStr">
+        <is>
+          <t>Accessori inclusi</t>
+        </is>
+      </c>
+      <c r="B63" s="32" t="inlineStr">
+        <is>
+          <t>Asciugacapelli, aspirapolvere, ferro da stiro, bollitore, tostapane, kit pronto soccorso, porta ombrelli, zerbino, grucce, strumenti pulizia, cestini, WC kit, porta saponi, cuscini, copricuscini, doghe letto, copridivano, pentole, piatti, bicchieri, posate, telecomandi, scala, adattatori, pastiglia anticalcare</t>
+        </is>
+      </c>
+      <c r="C63" s="7" t="inlineStr">
+        <is>
+          <t>Lista molto dettagliata: praticamente tutti i consumabili e semi-durevoli dell'appartamento</t>
+        </is>
+      </c>
+      <c r="D63" s="8" t="inlineStr">
+        <is>
+          <t>Il costo del +2,5% si applica su ogni prenotazione: in periodi di alta occupazione può superare il valore degli interventi effettivi</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="40" customHeight="1">
+      <c r="A64" s="30" t="inlineStr">
+        <is>
+          <t>Attivazione</t>
+        </is>
+      </c>
+      <c r="B64" s="6" t="inlineStr">
+        <is>
+          <t>A partire dalla prima prenotazione</t>
+        </is>
+      </c>
+      <c r="C64" s="6" t="inlineStr"/>
+      <c r="D64" s="6" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <mergeCells count="11">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A9:D9"/>
+    <mergeCell ref="A61:D61"/>
+    <mergeCell ref="A34:D34"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="A21:D21"/>
+    <mergeCell ref="A30:D30"/>
+    <mergeCell ref="A15:D15"/>
+    <mergeCell ref="A52:D52"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A46:D46"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:D55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -3852,10 +5092,10 @@
 (A.P.P.A. Srl)</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>AZIENDA C
-(da compilare)</t>
+      <c r="D3" s="33" t="inlineStr">
+        <is>
+          <t>EASYLIFE
+(Easylife S.p.A.)</t>
         </is>
       </c>
     </row>
@@ -3887,7 +5127,13 @@
 NB: basi diverse da Italianway</t>
         </is>
       </c>
-      <c r="D5" s="14" t="inlineStr"/>
+      <c r="D5" s="36" t="inlineStr">
+        <is>
+          <t>25% + IVA sul netto (netto OTA, netto pulizie, netto biancheria)
+Opzione Senza Pensieri: 27,5% + IVA
+OTA e pulizie addebitate separatamente all'ospite</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="38" customHeight="1">
       <c r="A6" s="9" t="inlineStr">
@@ -3906,7 +5152,12 @@
 Alternativa: 0 setup + 2,5% extra su commissioni</t>
         </is>
       </c>
-      <c r="D6" s="14" t="inlineStr"/>
+      <c r="D6" s="36" t="inlineStr">
+        <is>
+          <t>€300 pratiche (1° bonifico) + €140+IVA foto + €195,57 cilindro + €185+IVA key box
+≈ €820+ IVA escl.</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="38" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
@@ -3924,7 +5175,11 @@
           <t>Non applicabile (nessun mediatore separato)</t>
         </is>
       </c>
-      <c r="D7" s="14" t="inlineStr"/>
+      <c r="D7" s="36" t="inlineStr">
+        <is>
+          <t>Non applicabile (nessun mediatore separato; OTA incluse nel flow operativo)</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="38" customHeight="1">
       <c r="A8" s="9" t="inlineStr">
@@ -3942,7 +5197,11 @@
           <t>Non separata: le commissioni Youhosty sono a carico del proprietario (trattenute dal ricavo), non dell'ospite</t>
         </is>
       </c>
-      <c r="D8" s="14" t="inlineStr"/>
+      <c r="D8" s="36" t="inlineStr">
+        <is>
+          <t>Pulizie finali e biancheria addebitate all'ospite direttamente</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="38" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
@@ -3960,7 +5219,11 @@
           <t>Non esplicitamente menzionate</t>
         </is>
       </c>
-      <c r="D9" s="14" t="inlineStr"/>
+      <c r="D9" s="36" t="inlineStr">
+        <is>
+          <t>Non menzionate esplicitamente</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="38" customHeight="1">
       <c r="A10" s="9" t="inlineStr">
@@ -3978,7 +5241,11 @@
           <t>Servizio arredo 'da definire'; non incluso in alcun pacchetto standard</t>
         </is>
       </c>
-      <c r="D10" s="14" t="inlineStr"/>
+      <c r="D10" s="36" t="inlineStr">
+        <is>
+          <t>Non inclusa; dotazioni standard definite in Allegato A (costo a carico cliente)</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="15" t="inlineStr">
@@ -4007,7 +5274,11 @@
 Online/Flexible: 8-10 mesi di prova</t>
         </is>
       </c>
-      <c r="D12" s="14" t="inlineStr"/>
+      <c r="D12" s="36" t="inlineStr">
+        <is>
+          <t>18 mesi dalla prima prenotazione ricevuta</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="38" customHeight="1">
       <c r="A13" s="9" t="inlineStr">
@@ -4025,7 +5296,11 @@
           <t>Automatico (disdetta 3 mesi prima scadenza per All-Inclusive)</t>
         </is>
       </c>
-      <c r="D13" s="14" t="inlineStr"/>
+      <c r="D13" s="36" t="inlineStr">
+        <is>
+          <t>Automatico per ulteriori 18 mesi</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="38" customHeight="1">
       <c r="A14" s="5" t="inlineStr">
@@ -4044,7 +5319,11 @@
 Online/Flexible: 120 giorni</t>
         </is>
       </c>
-      <c r="D14" s="14" t="inlineStr"/>
+      <c r="D14" s="36" t="inlineStr">
+        <is>
+          <t>90 giorni prima di ciascuna scadenza (raccomandata a/r o PEC)</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="38" customHeight="1">
       <c r="A15" s="9" t="inlineStr">
@@ -4063,7 +5342,12 @@
 Più pratiche chiusura €220-320 + disinstallazione €250-350</t>
         </is>
       </c>
-      <c r="D15" s="14" t="inlineStr"/>
+      <c r="D15" s="36" t="inlineStr">
+        <is>
+          <t>Nessuna penale esplicita di recesso anticipato per il cliente
+(PM può recedere con 30 gg preavviso senza penale)</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="38" customHeight="1">
       <c r="A16" s="5" t="inlineStr">
@@ -4081,7 +5365,11 @@
           <t>Sì – assoluta (penale = oneri maturati sui contratti paralleli)</t>
         </is>
       </c>
-      <c r="D16" s="14" t="inlineStr"/>
+      <c r="D16" s="36" t="inlineStr">
+        <is>
+          <t>Sì – mandato irrevocabile con esclusiva (art. 2.1)</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="38" customHeight="1">
       <c r="A17" s="9" t="inlineStr">
@@ -4101,7 +5389,13 @@
 Extra: €15+IVA/gg</t>
         </is>
       </c>
-      <c r="D17" s="14" t="inlineStr"/>
+      <c r="D17" s="36" t="inlineStr">
+        <is>
+          <t>Max 30 gg/anno
+Preavviso 15 gg via email
+Solo spese di pulizia a carico</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="38" customHeight="1">
       <c r="A18" s="5" t="inlineStr">
@@ -4119,7 +5413,11 @@
           <t>Non menzionato esplicitamente nel contratto</t>
         </is>
       </c>
-      <c r="D18" s="14" t="inlineStr"/>
+      <c r="D18" s="36" t="inlineStr">
+        <is>
+          <t>Non menzionato esplicitamente</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="20" customHeight="1">
       <c r="A19" s="16" t="inlineStr">
@@ -4147,7 +5445,12 @@
           <t>App/sito internet Youhosty (nome non specificato)</t>
         </is>
       </c>
-      <c r="D20" s="14" t="inlineStr"/>
+      <c r="D20" s="36" t="inlineStr">
+        <is>
+          <t>Portale web per controllo andamento e spettanze
+(caratteristiche non dettagliate)</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="38" customHeight="1">
       <c r="A21" s="9" t="inlineStr">
@@ -4165,7 +5468,12 @@
           <t>Sì – software in outsourcing (provider non nominato)</t>
         </is>
       </c>
-      <c r="D21" s="14" t="inlineStr"/>
+      <c r="D21" s="36" t="inlineStr">
+        <is>
+          <t>Sì – PM determina liberamente i prezzi (art. 2.2)
+Nessun intervento del cliente possibile</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="38" customHeight="1">
       <c r="A22" s="5" t="inlineStr">
@@ -4184,7 +5492,11 @@
 Costo OTA addebitato al cliente</t>
         </is>
       </c>
-      <c r="D22" s="14" t="inlineStr"/>
+      <c r="D22" s="36" t="inlineStr">
+        <is>
+          <t>Sì – OTA multiple + portale proprietario Easylife House</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="38" customHeight="1">
       <c r="A23" s="9" t="inlineStr">
@@ -4202,7 +5514,11 @@
           <t>Sì – self check-in automatizzato incluso (All-Inclusive)</t>
         </is>
       </c>
-      <c r="D23" s="14" t="inlineStr"/>
+      <c r="D23" s="36" t="inlineStr">
+        <is>
+          <t>Sì – remoto/automatizzato (key box €185+IVA a carico cliente)</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="38" customHeight="1">
       <c r="A24" s="5" t="inlineStr">
@@ -4220,7 +5536,11 @@
           <t>Sì – costo ribaltato sull'ospite (ove possibile sulla piattaforma)</t>
         </is>
       </c>
-      <c r="D24" s="14" t="inlineStr"/>
+      <c r="D24" s="36" t="inlineStr">
+        <is>
+          <t>Sì – addebitate all'ospite separatamente</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="38" customHeight="1">
       <c r="A25" s="9" t="inlineStr">
@@ -4238,7 +5558,11 @@
           <t>Sì – incluso in All-Inclusive</t>
         </is>
       </c>
-      <c r="D25" s="14" t="inlineStr"/>
+      <c r="D25" s="36" t="inlineStr">
+        <is>
+          <t>Sì – incluse nel mandato e nella procura speciale</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="38" customHeight="1">
       <c r="A26" s="5" t="inlineStr">
@@ -4256,7 +5580,12 @@
           <t>Non menzionato esplicitamente</t>
         </is>
       </c>
-      <c r="D26" s="14" t="inlineStr"/>
+      <c r="D26" s="36" t="inlineStr">
+        <is>
+          <t>Non menzionato esplicitamente
+Ritenuta 21% applicata; CU annuale rilasciata</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="38" customHeight="1">
       <c r="A27" s="9" t="inlineStr">
@@ -4274,7 +5603,11 @@
           <t>Sì – €99 (o €69 con pagamento anticipato), obbligatoria</t>
         </is>
       </c>
-      <c r="D27" s="14" t="inlineStr"/>
+      <c r="D27" s="36" t="inlineStr">
+        <is>
+          <t>Sì – obbligatoria, €140 + IVA a carico cliente</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="38" customHeight="1">
       <c r="A28" s="5" t="inlineStr">
@@ -4292,7 +5625,11 @@
           <t>Sì – gestione profilo multilingua inclusa</t>
         </is>
       </c>
-      <c r="D28" s="14" t="inlineStr"/>
+      <c r="D28" s="36" t="inlineStr">
+        <is>
+          <t>Non menzionate esplicitamente</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="38" customHeight="1">
       <c r="A29" s="9" t="inlineStr">
@@ -4310,7 +5647,11 @@
           <t>Sì – check-up periodico nell'abbonamento mensile</t>
         </is>
       </c>
-      <c r="D29" s="14" t="inlineStr"/>
+      <c r="D29" s="36" t="inlineStr">
+        <is>
+          <t>Sì – PM segnala danni e verifica condizioni (art. 4.4)</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="38" customHeight="1">
       <c r="A30" s="5" t="inlineStr">
@@ -4328,7 +5669,12 @@
           <t>Entro il 30° giorno del mese successivo all'incasso dalla piattaforma</t>
         </is>
       </c>
-      <c r="D30" s="14" t="inlineStr"/>
+      <c r="D30" s="36" t="inlineStr">
+        <is>
+          <t>Entro il 20° del mese successivo all'incasso
+(conteggio per data check-in)</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="20" customHeight="1">
       <c r="A31" s="17" t="inlineStr">
@@ -4356,7 +5702,11 @@
           <t>Non fornita da Youhosty – obbligatoria per legge a carico cliente</t>
         </is>
       </c>
-      <c r="D32" s="14" t="inlineStr"/>
+      <c r="D32" s="36" t="inlineStr">
+        <is>
+          <t>Non fornita da Easylife – obbligatoria per legge a carico cliente (art. 10.3)</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="38" customHeight="1">
       <c r="A33" s="9" t="inlineStr">
@@ -4374,7 +5724,11 @@
           <t>Non fornita – a carico cliente</t>
         </is>
       </c>
-      <c r="D33" s="14" t="inlineStr"/>
+      <c r="D33" s="36" t="inlineStr">
+        <is>
+          <t>Non fornita – a carico cliente</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="38" customHeight="1">
       <c r="A34" s="5" t="inlineStr">
@@ -4392,7 +5746,11 @@
           <t>Non fornita – a carico cliente</t>
         </is>
       </c>
-      <c r="D34" s="14" t="inlineStr"/>
+      <c r="D34" s="36" t="inlineStr">
+        <is>
+          <t>Non fornita – a carico cliente</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="38" customHeight="1">
       <c r="A35" s="9" t="inlineStr">
@@ -4410,7 +5768,11 @@
           <t>Non fornita – a carico cliente</t>
         </is>
       </c>
-      <c r="D35" s="14" t="inlineStr"/>
+      <c r="D35" s="36" t="inlineStr">
+        <is>
+          <t>Non fornita – a carico cliente</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="38" customHeight="1">
       <c r="A36" s="5" t="inlineStr">
@@ -4428,7 +5790,11 @@
           <t>Non fornita – a carico cliente</t>
         </is>
       </c>
-      <c r="D36" s="14" t="inlineStr"/>
+      <c r="D36" s="36" t="inlineStr">
+        <is>
+          <t>Non fornita – a carico cliente</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="38" customHeight="1">
       <c r="A37" s="9" t="inlineStr">
@@ -4446,7 +5812,11 @@
           <t>Non fornita – a carico cliente</t>
         </is>
       </c>
-      <c r="D37" s="14" t="inlineStr"/>
+      <c r="D37" s="36" t="inlineStr">
+        <is>
+          <t>Non fornita – a carico cliente</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="38" customHeight="1">
       <c r="A38" s="5" t="inlineStr">
@@ -4464,7 +5834,11 @@
           <t>Cauzione ospite (ove possibile sulla piattaforma); importo variabile</t>
         </is>
       </c>
-      <c r="D38" s="14" t="inlineStr"/>
+      <c r="D38" s="36" t="inlineStr">
+        <is>
+          <t>Dipende dalla policy OTA (non standardizzata nel contratto)</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="38" customHeight="1">
       <c r="A39" s="9" t="inlineStr">
@@ -4482,7 +5856,11 @@
           <t>Non applicabile (nessuna polizza Youhosty)</t>
         </is>
       </c>
-      <c r="D39" s="14" t="inlineStr"/>
+      <c r="D39" s="36" t="inlineStr">
+        <is>
+          <t>Non applicabile (nessuna polizza Easylife)</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="38" customHeight="1">
       <c r="A40" s="5" t="inlineStr">
@@ -4500,7 +5878,11 @@
           <t>Nessuno – cliente autonomo</t>
         </is>
       </c>
-      <c r="D40" s="14" t="inlineStr"/>
+      <c r="D40" s="36" t="inlineStr">
+        <is>
+          <t>Nessuno – cliente autonomo</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="20" customHeight="1">
       <c r="A41" s="18" t="inlineStr">
@@ -4529,7 +5911,12 @@
 Aspirapolv. incluso nella Setup Fee (facoltativo)</t>
         </is>
       </c>
-      <c r="D42" s="14" t="inlineStr"/>
+      <c r="D42" s="36" t="inlineStr">
+        <is>
+          <t>Standard definiti in Allegato A (scheda alloggio)
+Cliente acquista dotazioni mancanti prima dello shooting</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="38" customHeight="1">
       <c r="A43" s="9" t="inlineStr">
@@ -4547,7 +5934,11 @@
           <t>Non menzionato esplicitamente</t>
         </is>
       </c>
-      <c r="D43" s="14" t="inlineStr"/>
+      <c r="D43" s="36" t="inlineStr">
+        <is>
+          <t>Sì – min. 100 Mbps o la più veloce disponibile in zona (art. 3.9)</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="38" customHeight="1">
       <c r="A44" s="5" t="inlineStr">
@@ -4565,7 +5956,11 @@
           <t>Non menzionata</t>
         </is>
       </c>
-      <c r="D44" s="14" t="inlineStr"/>
+      <c r="D44" s="36" t="inlineStr">
+        <is>
+          <t>Non menzionata esplicitamente</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="38" customHeight="1">
       <c r="A45" s="9" t="inlineStr">
@@ -4584,7 +5979,12 @@
 Rinnovo incluso nell'abbonamento mensile</t>
         </is>
       </c>
-      <c r="D45" s="14" t="inlineStr"/>
+      <c r="D45" s="36" t="inlineStr">
+        <is>
+          <t>Non menzionati esplicitamente nel contratto
+(coperti dalla formula Senza Pensieri solo in parte)</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="38" customHeight="1">
       <c r="A46" s="5" t="inlineStr">
@@ -4602,7 +6002,11 @@
           <t>5 mazzi (o 1 con self check-in installato)</t>
         </is>
       </c>
-      <c r="D46" s="14" t="inlineStr"/>
+      <c r="D46" s="36" t="inlineStr">
+        <is>
+          <t>4 mazzi (oppure 1 con key box installata)</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="38" customHeight="1">
       <c r="A47" s="9" t="inlineStr">
@@ -4620,7 +6024,11 @@
           <t>Facoltativa: mono €70 / bilocale €100 / trilocale €150</t>
         </is>
       </c>
-      <c r="D47" s="14" t="inlineStr"/>
+      <c r="D47" s="36" t="inlineStr">
+        <is>
+          <t>Non menzionata esplicitamente (dotazioni devono essere pronte prima dello shooting)</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="38" customHeight="1">
       <c r="A48" s="5" t="inlineStr">
@@ -4638,7 +6046,11 @@
           <t>Non menzionato</t>
         </is>
       </c>
-      <c r="D48" s="14" t="inlineStr"/>
+      <c r="D48" s="36" t="inlineStr">
+        <is>
+          <t>Non menzionato</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="38" customHeight="1">
       <c r="A49" s="9" t="inlineStr">
@@ -4656,7 +6068,11 @@
           <t>Non specificato (nessun divieto esplicito)</t>
         </is>
       </c>
-      <c r="D49" s="14" t="inlineStr"/>
+      <c r="D49" s="36" t="inlineStr">
+        <is>
+          <t>Non specificato</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="38" customHeight="1">
       <c r="A50" s="5" t="inlineStr">
@@ -4674,7 +6090,11 @@
           <t>Nessun branding Youhosty in appartamento (non menzionato)</t>
         </is>
       </c>
-      <c r="D50" s="14" t="inlineStr"/>
+      <c r="D50" s="36" t="inlineStr">
+        <is>
+          <t>Nessun branding fisico Easylife in appartamento menzionato</t>
+        </is>
+      </c>
     </row>
     <row r="51" ht="20" customHeight="1">
       <c r="A51" s="19" t="inlineStr">
@@ -4703,7 +6123,12 @@
 A.P.P.A. Srl Milano</t>
         </is>
       </c>
-      <c r="D52" s="14" t="inlineStr"/>
+      <c r="D52" s="36" t="inlineStr">
+        <is>
+          <t>Gestione diretta con partner/collaboratori
+Easylife S.p.A. Milano</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="38" customHeight="1">
       <c r="A53" s="9" t="inlineStr">
@@ -4721,7 +6146,11 @@
           <t>Milano, via G. Pezzi 2 (cap 20135)</t>
         </is>
       </c>
-      <c r="D53" s="14" t="inlineStr"/>
+      <c r="D53" s="36" t="inlineStr">
+        <is>
+          <t>Via G.B. Pergolesi 26, 20124 Milano</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="38" customHeight="1">
       <c r="A54" s="5" t="inlineStr">
@@ -4740,7 +6169,11 @@
 Oneri dovuti anche in caso di mancato incasso</t>
         </is>
       </c>
-      <c r="D54" s="14" t="inlineStr"/>
+      <c r="D54" s="36" t="inlineStr">
+        <is>
+          <t>PM incassa per conto del cliente (mandato con rappresentanza)</t>
+        </is>
+      </c>
     </row>
     <row r="55" ht="38" customHeight="1">
       <c r="A55" s="9" t="inlineStr">
@@ -4759,7 +6192,11 @@
 Altrimenti obbligo torna al cliente</t>
         </is>
       </c>
-      <c r="D55" s="14" t="inlineStr"/>
+      <c r="D55" s="36" t="inlineStr">
+        <is>
+          <t>Non menzionata nel contratto; gestione fiscale a carico del cliente</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -4776,7 +6213,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4830,9 +6267,9 @@
           <t>YOUHOSTY</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>AZIENDA C</t>
+      <c r="D3" s="33" t="inlineStr">
+        <is>
+          <t>EASYLIFE</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
@@ -4857,11 +6294,16 @@
           <t>2</t>
         </is>
       </c>
-      <c r="D4" s="22" t="inlineStr"/>
+      <c r="D4" s="37" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
           <t>Italianway: 25% ospite + 2% provv. – verificare vs mercato
-Youhosty: 16,5% + OTA (addebitata) + abbonamento mensile €19,90-26,90 + pratiche chiusura €470 → più costoso di quanto appare</t>
+Youhosty: 16,5% + OTA (addebitata) + abbonamento mensile €19,90-26,90 + pratiche chiusura €470 → più costoso di quanto appare
+Easylife: 25%+IVA sul netto (OTA e pulizie separate, addebitate all'ospite) + costi avvio ~€820. Nessun canone mensile. Formula Senza Pensieri +2,5%.</t>
         </is>
       </c>
     </row>
@@ -4881,11 +6323,16 @@
           <t>3</t>
         </is>
       </c>
-      <c r="D5" s="22" t="inlineStr"/>
+      <c r="D5" s="37" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="E5" s="10" t="inlineStr">
         <is>
           <t>Costi abbastanza espliciti nel contratto
-Youhosty: prezzi espliciti ma molti componenti separati (OTA, mensile, chiusura) rendono difficile il calcolo del costo totale</t>
+Youhosty: prezzi espliciti ma molti componenti separati (OTA, mensile, chiusura) rendono difficile il calcolo del costo totale
+Easylife: contratto chiaro su commissioni e costi avvio, ma OTA non nominate e alcuni costi accessori 'da trattenere alla prima contabilità utile' non quantificati</t>
         </is>
       </c>
     </row>
@@ -4905,11 +6352,16 @@
           <t>1</t>
         </is>
       </c>
-      <c r="D6" s="22" t="inlineStr"/>
+      <c r="D6" s="37" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
           <t>Esclusiva + 3 mesi preavviso + rinnovo tacito = poco flessibile
-All-Inclusive 24 mesi, recesso solo forza maggiore, pratiche chiusura €470, penale accesso €50 → il meno flessibile</t>
+All-Inclusive 24 mesi, recesso solo forza maggiore, pratiche chiusura €470, penale accesso €50 → il meno flessibile
+Easylife: 18 mesi (migliore di Youhosty 24 mesi, peggiore di Italianway 12 mesi). Nessun recesso anticipato per cliente. PM può uscire con 30 gg.</t>
         </is>
       </c>
     </row>
@@ -4929,11 +6381,16 @@
           <t>4</t>
         </is>
       </c>
-      <c r="D7" s="22" t="inlineStr"/>
+      <c r="D7" s="37" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="E7" s="10" t="inlineStr">
         <is>
           <t>Check-in, pulizie, burocrazia gestiti; qualità PM locale da verificare
-Self check-in automatizzato, gestione completa, multilingual; gestione diretta (non franchising) → qualità più uniforme</t>
+Self check-in automatizzato, gestione completa, multilingual; gestione diretta (non franchising) → qualità più uniforme
+Easylife: gestione completa con partner, check-in automatizzato, portale proprietario Easylife House. Formula Senza Pensieri per manutenzioni.</t>
         </is>
       </c>
     </row>
@@ -4953,11 +6410,16 @@
           <t>3</t>
         </is>
       </c>
-      <c r="D8" s="22" t="inlineStr"/>
+      <c r="D8" s="37" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
           <t>KALISI: real-time, algoritmo Revenue Management
-App/sito proprietario con revenue management in outsourcing; meno descritto di KALISI ma funzionale</t>
+App/sito proprietario con revenue management in outsourcing; meno descritto di KALISI ma funzionale
+Easylife: portale web per controllo + Easylife House (OTA proprietaria). Funzionalità non dettagliate nel contratto.</t>
         </is>
       </c>
     </row>
@@ -4977,11 +6439,16 @@
           <t>3</t>
         </is>
       </c>
-      <c r="D9" s="22" t="inlineStr"/>
+      <c r="D9" s="37" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="E9" s="10" t="inlineStr">
         <is>
           <t>Accesso KALISI; pagamento il 28 del mese
-Reportistica per immobile disponibile; pagamento entro 30° mese; OTA addebitata separatamente aumenta complessità</t>
+Reportistica per immobile disponibile; pagamento entro 30° mese; OTA addebitata separatamente aumenta complessità
+Easylife: pagamento entro 20° del mese successivo; CU annuale; portale per controllo spettanze. Nessun dettaglio su reportistica breakdown.</t>
         </is>
       </c>
     </row>
@@ -5001,11 +6468,16 @@
           <t>1</t>
         </is>
       </c>
-      <c r="D10" s="22" t="inlineStr"/>
+      <c r="D10" s="37" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
           <t>RC €1M ottima; massimali incendio/furto nella media
-Nessuna polizza collettiva: solo cauzione piattaforma e consiglio di stipulare RC propria → rischio massimo per il proprietario</t>
+Nessuna polizza collettiva: solo cauzione piattaforma e consiglio di stipulare RC propria → rischio massimo per il proprietario
+Easylife: nessuna polizza collettiva. Il cliente deve stipulare tutto autonomamente (art. 10.3). Responsabilità danni ospiti esonerate esplicitamente.</t>
         </is>
       </c>
     </row>
@@ -5025,11 +6497,16 @@
           <t>4</t>
         </is>
       </c>
-      <c r="D11" s="22" t="inlineStr"/>
+      <c r="D11" s="37" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="E11" s="10" t="inlineStr">
         <is>
           <t>Lista dotazioni lunga; sicurezza e pulizia pre-shooting a carico proprietario
-Lista dotazioni non prescrittiva; meno obblighi iniziali; sicurezza in noleggio gestito da Youhosty</t>
+Lista dotazioni non prescrittiva; meno obblighi iniziali; sicurezza in noleggio gestito da Youhosty
+Easylife: standard Allegato A non dettagliati nel documento; 4 mazzi chiavi; costi avvio documentati ma significativi (~€820+)</t>
         </is>
       </c>
     </row>
@@ -5049,11 +6526,16 @@
           <t>3</t>
         </is>
       </c>
-      <c r="D12" s="22" t="inlineStr"/>
+      <c r="D12" s="37" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
           <t>Brand nazionale; franchising diffuso; dal 2014
-Brand riconoscibile a Milano; meno capillare di Italianway a livello nazionale</t>
+Brand riconoscibile a Milano; meno capillare di Italianway a livello nazionale
+Easylife: S.p.A. con sede a Milano, portale proprietario. Meno informazioni pubbliche rispetto a Italianway.</t>
         </is>
       </c>
     </row>
@@ -5073,11 +6555,16 @@
           <t>3</t>
         </is>
       </c>
-      <c r="D13" s="22" t="inlineStr"/>
+      <c r="D13" s="37" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="E13" s="10" t="inlineStr">
         <is>
           <t>Italianway SpA intermedia: dipendenza da solidità aziendale
-Oneri dovuti anche senza incasso; canone garantito disponibile (Allegato 3) ma non allegato</t>
+Oneri dovuti anche senza incasso; canone garantito disponibile (Allegato 3) ma non allegato
+Easylife: PM incassa per conto del cliente. Nessun canone garantito menzionato. Prenotazioni post-recesso onorate da entrambe le parti.</t>
         </is>
       </c>
     </row>
@@ -5097,11 +6584,16 @@
           <t>3</t>
         </is>
       </c>
-      <c r="D14" s="22" t="inlineStr"/>
+      <c r="D14" s="37" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="E14" s="6" t="inlineStr">
         <is>
           <t>Possibile ma con costi di ripristino non quantificati
-45 gg/anno All-Inclusive, fuori eventi principali; €15/gg extra; più gg rispetto a Italianway ma con limitazioni sui periodi</t>
+45 gg/anno All-Inclusive, fuori eventi principali; €15/gg extra; più gg rispetto a Italianway ma con limitazioni sui periodi
+Easylife: 30 gg/anno, 15 gg preavviso scritto, solo spese pulizia. Nessun costo giornaliero aggiuntivo a differenza di Youhosty.</t>
         </is>
       </c>
     </row>
@@ -5121,11 +6613,16 @@
           <t>4</t>
         </is>
       </c>
-      <c r="D15" s="22" t="inlineStr"/>
+      <c r="D15" s="37" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="E15" s="10" t="inlineStr">
         <is>
           <t>PM locale affiliato; qualità variabile per zona
-Gestione diretta non franchise → interlocutore unico e stabile; abbonamento mensile con check-up periodico</t>
+Gestione diretta non franchise → interlocutore unico e stabile; abbonamento mensile con check-up periodico
+Easylife: portale web, segnalazione danni, CU annuale. Penale accesso non autorizzato molto severa (100% incassi mese successivo).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add phone call notes and update scorecard with operational data
</commit_message>
<xml_diff>
--- a/Italianway_Analisi_Comparativa.xlsx
+++ b/Italianway_Analisi_Comparativa.xlsx
@@ -11,7 +11,8 @@
     <sheet name="RIEPILOGO YOUHOSTY" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="RIEPILOGO EASYLIFE" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="CONFRONTO 3 AZIENDE" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="SCORECARD DECISIONALE" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="NOTE TELEFONATE" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="SCORECARD DECISIONALE" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="19">
+  <fonts count="21">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -131,8 +132,20 @@
       <color rgb="001B3A5C"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="24">
+  <fills count="26">
     <fill>
       <patternFill/>
     </fill>
@@ -249,6 +262,16 @@
         <fgColor rgb="00F0F7EE"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F5A623"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EAF4FB"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="6">
     <border>
@@ -320,7 +343,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -428,6 +451,39 @@
     </xf>
     <xf numFmtId="0" fontId="18" fillId="23" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="24" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="25" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="21" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="24" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="25" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="22" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="23" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="25" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3878,6 +3934,9 @@
           <t>EASYLIFE S.p.A. – ANALISI COMPLETA</t>
         </is>
       </c>
+      <c r="B1" s="24" t="n"/>
+      <c r="C1" s="24" t="n"/>
+      <c r="D1" s="25" t="n"/>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="27" t="inlineStr">
@@ -3885,6 +3944,9 @@
           <t>Fonte: Mandato di Gestione per Affitti Brevi (Easylife S.p.A., Via G.B. Pergolesi 26, 20124 Milano, P.IVA 09640480969)</t>
         </is>
       </c>
+      <c r="B2" s="24" t="n"/>
+      <c r="C2" s="24" t="n"/>
+      <c r="D2" s="25" t="n"/>
     </row>
     <row r="3" ht="24" customHeight="1">
       <c r="A3" s="28" t="inlineStr">
@@ -3914,6 +3976,9 @@
           <t>🏢 STRUTTURA AZIENDALE</t>
         </is>
       </c>
+      <c r="B4" s="24" t="n"/>
+      <c r="C4" s="24" t="n"/>
+      <c r="D4" s="25" t="n"/>
     </row>
     <row r="5" ht="40" customHeight="1">
       <c r="A5" s="30" t="inlineStr">
@@ -4001,6 +4066,9 @@
           <t>💰 COMMISSIONI E CORRISPETTIVO</t>
         </is>
       </c>
+      <c r="B9" s="24" t="n"/>
+      <c r="C9" s="24" t="n"/>
+      <c r="D9" s="25" t="n"/>
     </row>
     <row r="10" ht="40" customHeight="1">
       <c r="A10" s="30" t="inlineStr">
@@ -4121,6 +4189,9 @@
           <t>💶 COSTI DI AVVIO (UNA TANTUM, IVA esclusa salvo indicazione)</t>
         </is>
       </c>
+      <c r="B15" s="24" t="n"/>
+      <c r="C15" s="24" t="n"/>
+      <c r="D15" s="25" t="n"/>
     </row>
     <row r="16" ht="40" customHeight="1">
       <c r="A16" s="30" t="inlineStr">
@@ -4238,6 +4309,9 @@
           <t>📄 CONTRATTO, DURATA E RECESSO</t>
         </is>
       </c>
+      <c r="B21" s="24" t="n"/>
+      <c r="C21" s="24" t="n"/>
+      <c r="D21" s="25" t="n"/>
     </row>
     <row r="22" ht="40" customHeight="1">
       <c r="A22" s="30" t="inlineStr">
@@ -4405,6 +4479,9 @@
           <t>🏠 USO PERSONALE DELL'IMMOBILE</t>
         </is>
       </c>
+      <c r="B30" s="24" t="n"/>
+      <c r="C30" s="24" t="n"/>
+      <c r="D30" s="25" t="n"/>
     </row>
     <row r="31" ht="40" customHeight="1">
       <c r="A31" s="30" t="inlineStr">
@@ -4478,6 +4555,9 @@
           <t>🛎️ SERVIZI INCLUSI NEL MANDATO</t>
         </is>
       </c>
+      <c r="B34" s="24" t="n"/>
+      <c r="C34" s="24" t="n"/>
+      <c r="D34" s="25" t="n"/>
     </row>
     <row r="35" ht="40" customHeight="1">
       <c r="A35" s="30" t="inlineStr">
@@ -4707,6 +4787,9 @@
           <t>🛡️ GARANZIA DANNI E ASSICURAZIONE</t>
         </is>
       </c>
+      <c r="B46" s="24" t="n"/>
+      <c r="C46" s="24" t="n"/>
+      <c r="D46" s="25" t="n"/>
     </row>
     <row r="47" ht="40" customHeight="1">
       <c r="A47" s="30" t="inlineStr">
@@ -4808,6 +4891,9 @@
           <t>📋 OBBLIGHI E ONERI DEL CLIENTE</t>
         </is>
       </c>
+      <c r="B52" s="24" t="n"/>
+      <c r="C52" s="24" t="n"/>
+      <c r="D52" s="25" t="n"/>
     </row>
     <row r="53" ht="40" customHeight="1">
       <c r="A53" s="30" t="inlineStr">
@@ -4963,6 +5049,9 @@
           <t>🔧 FORMULA 'SENZA PENSIERI' (opzionale, +2,5% sulla commissione)</t>
         </is>
       </c>
+      <c r="B61" s="24" t="n"/>
+      <c r="C61" s="24" t="n"/>
+      <c r="D61" s="25" t="n"/>
     </row>
     <row r="62" ht="40" customHeight="1">
       <c r="A62" s="30" t="inlineStr">
@@ -5046,7 +5135,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D55"/>
+  <dimension ref="A1:D69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5058,7 +5147,7 @@
     <row r="1" ht="36" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>CONFRONTO PROPERTY MANAGER – ITALIANWAY vs AZIENDA B vs AZIENDA C</t>
+          <t>CONFRONTO PROPERTY MANAGER – ITALIANWAY vs YOUHOSTY (A.P.P.A. Srl) vs EASYLIFE S.p.A.</t>
         </is>
       </c>
       <c r="B1" s="24" t="n"/>
@@ -6198,11 +6287,283 @@
         </is>
       </c>
     </row>
+    <row r="57" ht="22" customHeight="1">
+      <c r="A57" s="38" t="inlineStr">
+        <is>
+          <t>▶  DATI OPERATIVI DA TELEFONATE COMMERCIALI (non contrattuali)</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="45" customHeight="1">
+      <c r="A58" s="39" t="inlineStr">
+        <is>
+          <t>Appartamenti gestiti (totale)</t>
+        </is>
+      </c>
+      <c r="B58" s="40" t="inlineStr">
+        <is>
+          <t>750 attivi a Milano + network franchising</t>
+        </is>
+      </c>
+      <c r="C58" s="34" t="inlineStr">
+        <is>
+          <t>500 tra Milano e Como</t>
+        </is>
+      </c>
+      <c r="D58" s="36" t="inlineStr">
+        <is>
+          <t>500 (Milano entro 2a circonvallazione + Como, Roma, Venezia, Napoli, Lugano)</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="45" customHeight="1">
+      <c r="A59" s="41" t="inlineStr">
+        <is>
+          <t>Manutentori disponibili</t>
+        </is>
+      </c>
+      <c r="B59" s="40" t="inlineStr">
+        <is>
+          <t>~40 a Milano (1:18 per appartamento) – fino a mezzanotte</t>
+        </is>
+      </c>
+      <c r="C59" s="34" t="inlineStr">
+        <is>
+          <t>~10 a Milano (1:50) – customer care 24/7 – check-in in presenza fino alle 3</t>
+        </is>
+      </c>
+      <c r="D59" s="36" t="inlineStr">
+        <is>
+          <t>⚠️ Solo 4 per 500 appartamenti (1:125) – non H24 dopo mezzanotte</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="45" customHeight="1">
+      <c r="A60" s="39" t="inlineStr">
+        <is>
+          <t>Tasso occupazione dichiarato</t>
+        </is>
+      </c>
+      <c r="B60" s="40" t="inlineStr">
+        <is>
+          <t>72% (dati RDNA, non propri)</t>
+        </is>
+      </c>
+      <c r="C60" s="34" t="inlineStr">
+        <is>
+          <t>70-75% (zona 1, alta stagione 9/12 mesi); &gt;80% mesi strategici</t>
+        </is>
+      </c>
+      <c r="D60" s="36" t="inlineStr">
+        <is>
+          <t>~85% dichiarato. Nessun minimo garantito</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="45" customHeight="1">
+      <c r="A61" s="41" t="inlineStr">
+        <is>
+          <t>Software pricing dinamico</t>
+        </is>
+      </c>
+      <c r="B61" s="40" t="inlineStr">
+        <is>
+          <t>Team revenue settimanale. Software proprietario (nome n/d)</t>
+        </is>
+      </c>
+      <c r="C61" s="34" t="inlineStr">
+        <is>
+          <t>Algoritmo proprietario + PriceLabs (aggiornamento quotidiano)</t>
+        </is>
+      </c>
+      <c r="D61" s="36" t="inlineStr">
+        <is>
+          <t>'Be on Pricing' – aggiornamento quotidiano</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="45" customHeight="1">
+      <c r="A62" s="39" t="inlineStr">
+        <is>
+          <t>Clientela corporate / business</t>
+        </is>
+      </c>
+      <c r="B62" s="40" t="inlineStr">
+        <is>
+          <t>Presente su Booking/Airbnb for Work. Non su GDS</t>
+        </is>
+      </c>
+      <c r="C62" s="34" t="inlineStr">
+        <is>
+          <t>Sì: Bottega Veneta, Mediolanum, ecc. Confcommercio</t>
+        </is>
+      </c>
+      <c r="D62" s="36" t="inlineStr">
+        <is>
+          <t>Sì: divisione Uvet/Cisalpina/BSD; Gucci, Valentino. ⚠️ Non su GDS</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="45" customHeight="1">
+      <c r="A63" s="41" t="inlineStr">
+        <is>
+          <t>Referente per il proprietario</t>
+        </is>
+      </c>
+      <c r="B63" s="40" t="inlineStr">
+        <is>
+          <t>Property service: 2 persone (operativo + amministrativo)</t>
+        </is>
+      </c>
+      <c r="C63" s="34" t="inlineStr">
+        <is>
+          <t>House manager senior dedicato (~20 app. a testa)</t>
+        </is>
+      </c>
+      <c r="D63" s="36" t="inlineStr">
+        <is>
+          <t>Gruppo WhatsApp condiviso tra proprietari (non dedicato)</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="45" customHeight="1">
+      <c r="A64" s="39" t="inlineStr">
+        <is>
+          <t>Reperibilità emergenze notturne</t>
+        </is>
+      </c>
+      <c r="B64" s="40" t="inlineStr">
+        <is>
+          <t>1 manutentore fino a mezzanotte</t>
+        </is>
+      </c>
+      <c r="C64" s="34" t="inlineStr">
+        <is>
+          <t>Customer care 24/7 + check-in in presenza fino alle 3</t>
+        </is>
+      </c>
+      <c r="D64" s="36" t="inlineStr">
+        <is>
+          <t>⚠️ Non H24. Difficile dopo mezzanotte</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="45" customHeight="1">
+      <c r="A65" s="41" t="inlineStr">
+        <is>
+          <t>Vincolo uscita anticipata (reale)</t>
+        </is>
+      </c>
+      <c r="B65" s="40" t="inlineStr">
+        <is>
+          <t>1° anno: nessuna uscita. 2° anno+: disdetta 90 gg o €20/gg (sab+dom inclusi)</t>
+        </is>
+      </c>
+      <c r="C65" s="34" t="inlineStr">
+        <is>
+          <t>All-Incl.: solo forza maggiore o €50/gg + €470 costi chiusura</t>
+        </is>
+      </c>
+      <c r="D65" s="36" t="inlineStr">
+        <is>
+          <t>⚠️ In telefonata: 'vincolo di 1 anno' (non esplicitato chiaramente nel contratto scritto)</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="45" customHeight="1">
+      <c r="A66" s="39" t="inlineStr">
+        <is>
+          <t>Tempi avvio (firma → online)</t>
+        </is>
+      </c>
+      <c r="B66" s="40" t="inlineStr">
+        <is>
+          <t>CIN: 3-6 settimane + tempo shooting + adempimenti</t>
+        </is>
+      </c>
+      <c r="C66" s="34" t="inlineStr">
+        <is>
+          <t>20 giorni lavorativi dalla firma del contratto</t>
+        </is>
+      </c>
+      <c r="D66" s="36" t="inlineStr">
+        <is>
+          <t>Non specificato</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="45" customHeight="1">
+      <c r="A67" s="41" t="inlineStr">
+        <is>
+          <t>Gestione cedolare secca</t>
+        </is>
+      </c>
+      <c r="B67" s="40" t="inlineStr">
+        <is>
+          <t>Sì – versata da Italianway SpA per conto del proprietario</t>
+        </is>
+      </c>
+      <c r="C67" s="34" t="inlineStr">
+        <is>
+          <t>Sì – inclusa anche per medio/lungo termine</t>
+        </is>
+      </c>
+      <c r="D67" s="36" t="inlineStr">
+        <is>
+          <t>Non menzionata in telefonata. Nel contratto: ritenuta 21% applicata, CU rilasciata</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="45" customHeight="1">
+      <c r="A68" s="39" t="inlineStr">
+        <is>
+          <t>Anni di attività</t>
+        </is>
+      </c>
+      <c r="B68" s="40" t="inlineStr">
+        <is>
+          <t>14 anni</t>
+        </is>
+      </c>
+      <c r="C68" s="34" t="inlineStr">
+        <is>
+          <t>10 anni</t>
+        </is>
+      </c>
+      <c r="D68" s="36" t="inlineStr">
+        <is>
+          <t>Non dichiarato</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="45" customHeight="1">
+      <c r="A69" s="41" t="inlineStr">
+        <is>
+          <t>Assicurazione proposta</t>
+        </is>
+      </c>
+      <c r="B69" s="40" t="inlineStr">
+        <is>
+          <t>RC terzi a €30/mese (se non hai polizza propria); danni accidentali fino a €250</t>
+        </is>
+      </c>
+      <c r="C69" s="34" t="inlineStr">
+        <is>
+          <t>Nessuna. Cliente autonomo</t>
+        </is>
+      </c>
+      <c r="D69" s="36" t="inlineStr">
+        <is>
+          <t>Offrono polizza assicurativa (dettagli da richiedere per confronto con polizza esistente)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="9">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A31:D31"/>
     <mergeCell ref="A4:D4"/>
+    <mergeCell ref="A57:D57"/>
     <mergeCell ref="A41:D41"/>
     <mergeCell ref="A19:D19"/>
     <mergeCell ref="A11:D11"/>
@@ -6214,6 +6575,938 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D49"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="70" customWidth="1" min="2" max="2"/>
+    <col width="70" customWidth="1" min="3" max="3"/>
+    <col width="70" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="36" customHeight="1">
+      <c r="A1" s="26" t="inlineStr">
+        <is>
+          <t>NOTE TELEFONATE – CONFRONTO OPERATIVO (dati non contrattuali)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="27" t="inlineStr">
+        <is>
+          <t>Informazioni raccolte durante le telefonate commerciali con i tre gestori. Non sostitutive del contratto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="24" customHeight="1">
+      <c r="A3" s="28" t="inlineStr">
+        <is>
+          <t>AREA / DOMANDA</t>
+        </is>
+      </c>
+      <c r="B3" s="28" t="inlineStr">
+        <is>
+          <t>ITALIANWAY</t>
+        </is>
+      </c>
+      <c r="C3" s="28" t="inlineStr">
+        <is>
+          <t>YOUHOSTY (A.P.P.A. Srl)</t>
+        </is>
+      </c>
+      <c r="D3" s="28" t="inlineStr">
+        <is>
+          <t>EASYLIFE S.p.A.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="42" t="inlineStr">
+        <is>
+          <t>🏙️ DIMENSIONI E COPERTURA GEOGRAFICA</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="50" customHeight="1">
+      <c r="A5" s="30" t="inlineStr">
+        <is>
+          <t>Appartamenti gestiti (totale)</t>
+        </is>
+      </c>
+      <c r="B5" s="43" t="inlineStr">
+        <is>
+          <t>750 appartamenti attivi a Milano + 7.500 partner (franchising affitti brevi e vacanze estive) + ~160 dipendenti</t>
+        </is>
+      </c>
+      <c r="C5" s="44" t="inlineStr">
+        <is>
+          <t>500 immobili tra Milano e Como. Portfolio stimato €200 milioni</t>
+        </is>
+      </c>
+      <c r="D5" s="45" t="inlineStr">
+        <is>
+          <t>500 appartamenti: 160 entro 1a circonvallazione Milano (25 su Via Torino), max 2a circonvallazione. 30 Como, 15 Roma, 3 Napoli, 3 Venezia, 100 Lugano</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="50" customHeight="1">
+      <c r="A6" s="31" t="inlineStr">
+        <is>
+          <t>Copertura geografica Milano</t>
+        </is>
+      </c>
+      <c r="B6" s="43" t="inlineStr">
+        <is>
+          <t>Tutta Milano, franchising diffuso su territorio nazionale</t>
+        </is>
+      </c>
+      <c r="C6" s="44" t="inlineStr">
+        <is>
+          <t>Milano e Como (focus principale)</t>
+        </is>
+      </c>
+      <c r="D6" s="45" t="inlineStr">
+        <is>
+          <t>⚠️ SOLO entro la seconda circonvallazione di Milano. Sardegna: solo partner locali (stesso partner di Genova)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="50" customHeight="1">
+      <c r="A7" s="30" t="inlineStr">
+        <is>
+          <t>Anni di attività</t>
+        </is>
+      </c>
+      <c r="B7" s="43" t="inlineStr">
+        <is>
+          <t>14 anni di attività</t>
+        </is>
+      </c>
+      <c r="C7" s="44" t="inlineStr">
+        <is>
+          <t>10 anni operativi. Parte di Confcommercio con altri 5 player nazionali</t>
+        </is>
+      </c>
+      <c r="D7" s="45" t="inlineStr">
+        <is>
+          <t>Non dichiarato</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="50" customHeight="1">
+      <c r="A8" s="31" t="inlineStr">
+        <is>
+          <t>Modello aziendale</t>
+        </is>
+      </c>
+      <c r="B8" s="43" t="inlineStr">
+        <is>
+          <t>Franchising: Italianway SpA + affiliati locali ('partner' = venditori affitti brevi). Focus Easy e Comfort (non Luxury)</t>
+        </is>
+      </c>
+      <c r="C8" s="44" t="inlineStr">
+        <is>
+          <t>Gestione diretta (non franchising). House manager senior con ~20 appartamenti ciascuno</t>
+        </is>
+      </c>
+      <c r="D8" s="45" t="inlineStr">
+        <is>
+          <t>Gestione diretta con partner operativi. 4 manutentori per 500 appartamenti</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="42" t="inlineStr">
+        <is>
+          <t>📊 TASSO DI OCCUPAZIONE E STAGIONALITÀ</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="50" customHeight="1">
+      <c r="A10" s="30" t="inlineStr">
+        <is>
+          <t>Tasso occupazione dichiarato</t>
+        </is>
+      </c>
+      <c r="B10" s="43" t="inlineStr">
+        <is>
+          <t>72% da RDNA (dati piattaforme terze, non loro numeri diretti)</t>
+        </is>
+      </c>
+      <c r="C10" s="44" t="inlineStr">
+        <is>
+          <t>Zona 1: alta stagione 9 mesi su 12. Tasso 70-75%; 4 mesi strategici (Salone, Fashion Week, ecc.) &gt;80%</t>
+        </is>
+      </c>
+      <c r="D10" s="45" t="inlineStr">
+        <is>
+          <t>~85% (dichiarato). Nessun minimo garantito ma 'garanzia dell'esperienza'</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="50" customHeight="1">
+      <c r="A11" s="31" t="inlineStr">
+        <is>
+          <t>Stagionalità</t>
+        </is>
+      </c>
+      <c r="B11" s="43" t="inlineStr">
+        <is>
+          <t>Bassa stagione vera: fine dicembre, gennaio, agosto. Il resto dell'anno normalmente in affitto breve</t>
+        </is>
+      </c>
+      <c r="C11" s="44" t="inlineStr">
+        <is>
+          <t>Strategia stagionale suggerita: breve feb-lug; medio/lungo ago-feb (50%/50%). Effetti stagionali comunicati proattivamente</t>
+        </is>
+      </c>
+      <c r="D11" s="45" t="inlineStr">
+        <is>
+          <t>Novembre, dicembre, gennaio 'si piange'. Aprile si inizia a guadagnare bene</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="50" customHeight="1">
+      <c r="A12" s="30" t="inlineStr">
+        <is>
+          <t>Fase di start-up (nuovi immobili)</t>
+        </is>
+      </c>
+      <c r="B12" s="43" t="inlineStr">
+        <is>
+          <t>⚠️ Fase start: casa non recensita → più difficile da prenotare, tariffe più basse. Commissioni invariate anche in start-up</t>
+        </is>
+      </c>
+      <c r="C12" s="44" t="inlineStr">
+        <is>
+          <t>20 giorni lavorativi dalla firma del contratto per andare live</t>
+        </is>
+      </c>
+      <c r="D12" s="45" t="inlineStr">
+        <is>
+          <t>Non specificato</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="50" customHeight="1">
+      <c r="A13" s="31" t="inlineStr">
+        <is>
+          <t>Immobili con recensioni esistenti</t>
+        </is>
+      </c>
+      <c r="B13" s="43" t="inlineStr">
+        <is>
+          <t>Conviene mantenere le recensioni alte se già presenti (non si trasferiscono tra piattaforme)</t>
+        </is>
+      </c>
+      <c r="C13" s="44" t="inlineStr">
+        <is>
+          <t>Non discusso</t>
+        </is>
+      </c>
+      <c r="D13" s="45" t="inlineStr">
+        <is>
+          <t>Non discusso</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="42" t="inlineStr">
+        <is>
+          <t>📱 CANALI DI PRENOTAZIONE</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="50" customHeight="1">
+      <c r="A15" s="30" t="inlineStr">
+        <is>
+          <t>OTA principali</t>
+        </is>
+      </c>
+      <c r="B15" s="43" t="inlineStr">
+        <is>
+          <t>Airbnb (30% totale, 15% comm.), Booking (~18%), VRBO, Expedia + piattaforme internazionali + canale proprietario (20% totale, 18% comm.)</t>
+        </is>
+      </c>
+      <c r="C15" s="44" t="inlineStr">
+        <is>
+          <t>Airbnb + Booking + 20 canali totali + canale proprietario (20% delle prenotazioni)</t>
+        </is>
+      </c>
+      <c r="D15" s="45" t="inlineStr">
+        <is>
+          <t>Principalmente Booking e Airbnb. Portale proprietario Easylife House + Marriott (residuale ~1%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="50" customHeight="1">
+      <c r="A16" s="31" t="inlineStr">
+        <is>
+          <t>Clientela corporate / business</t>
+        </is>
+      </c>
+      <c r="B16" s="43" t="inlineStr">
+        <is>
+          <t>Business tramite Booking/Airbnb for Work e piattaforme estere. Non su GDS</t>
+        </is>
+      </c>
+      <c r="C16" s="44" t="inlineStr">
+        <is>
+          <t>Sì: aziende convenzionate (Bottega Veneta, Mediolanum, ecc.). Parte di Confcommercio</t>
+        </is>
+      </c>
+      <c r="D16" s="45" t="inlineStr">
+        <is>
+          <t>✅ Divisione corporate dedicata: Uvet, Cisalpina, BSD. Società convenzionate: Gucci, Valentino. ⚠️ Non su GDS → non integrabile con software corporate travel</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="50" customHeight="1">
+      <c r="A17" s="30" t="inlineStr">
+        <is>
+          <t>Canale diretto / proprietario</t>
+        </is>
+      </c>
+      <c r="B17" s="43" t="inlineStr">
+        <is>
+          <t>Canale Italianway (~20% totale, 18% commissione anche su questo canale)</t>
+        </is>
+      </c>
+      <c r="C17" s="44" t="inlineStr">
+        <is>
+          <t>Canale proprio: ~20% prenotazioni</t>
+        </is>
+      </c>
+      <c r="D17" s="45" t="inlineStr">
+        <is>
+          <t>Canale Easylife House + corporate. Non fornita % esatta</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="50" customHeight="1">
+      <c r="A18" s="31" t="inlineStr">
+        <is>
+          <t>Worst case commissione totale su prezzo ospite</t>
+        </is>
+      </c>
+      <c r="B18" s="43" t="inlineStr">
+        <is>
+          <t>⚠️ Worst case: 22% (promo) + 18% (piattaforma OTA) + IVA + cedolare secca = proprietario incassa ~metà del prezzo di uscita</t>
+        </is>
+      </c>
+      <c r="C18" s="44" t="inlineStr">
+        <is>
+          <t>16,5% Youhosty + commissione OTA addebitata al cliente + €26,90/mese + costi uscita</t>
+        </is>
+      </c>
+      <c r="D18" s="45" t="inlineStr">
+        <is>
+          <t>25% + IVA sul netto OTA/pulizie. OTA e pulizie pagate dall'ospite. Formula Senza Pensieri +2,5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="50" customHeight="1">
+      <c r="A19" s="30" t="inlineStr">
+        <is>
+          <t>Sincronizzazione prenotazioni</t>
+        </is>
+      </c>
+      <c r="B19" s="43" t="inlineStr">
+        <is>
+          <t>Software che parla con le piattaforme più grandi in sincrono</t>
+        </is>
+      </c>
+      <c r="C19" s="44" t="inlineStr">
+        <is>
+          <t>App aggiornata in tempo reale non appena arriva prenotazione da qualsiasi OTA</t>
+        </is>
+      </c>
+      <c r="D19" s="45" t="inlineStr">
+        <is>
+          <t>Software gestisce prenotazioni in sincrono</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="42" t="inlineStr">
+        <is>
+          <t>💲 PRICING DINAMICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="50" customHeight="1">
+      <c r="A21" s="30" t="inlineStr">
+        <is>
+          <t>Software di pricing</t>
+        </is>
+      </c>
+      <c r="B21" s="43" t="inlineStr">
+        <is>
+          <t>Team revenue dedicato. Software proprietario (nome non comunicato). Aggiornamento settimanale (lun. &lt; ven.; weekend senza prenotazioni = abbassano)</t>
+        </is>
+      </c>
+      <c r="C21" s="44" t="inlineStr">
+        <is>
+          <t>Algoritmo proprietario sviluppato in collaborazione con PriceLabs</t>
+        </is>
+      </c>
+      <c r="D21" s="45" t="inlineStr">
+        <is>
+          <t>'Be on Pricing' – software per variazioni giornaliere di prezzo</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="50" customHeight="1">
+      <c r="A22" s="31" t="inlineStr">
+        <is>
+          <t>Frequenza aggiornamento prezzi</t>
+        </is>
+      </c>
+      <c r="B22" s="43" t="inlineStr">
+        <is>
+          <t>Settimanale (aggiornamento da team revenue)</t>
+        </is>
+      </c>
+      <c r="C22" s="44" t="inlineStr">
+        <is>
+          <t>Quotidiana (algoritmo + PriceLabs)</t>
+        </is>
+      </c>
+      <c r="D22" s="45" t="inlineStr">
+        <is>
+          <t>Quotidiana ('Be on Pricing')</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="20" customHeight="1">
+      <c r="A23" s="42" t="inlineStr">
+        <is>
+          <t>🔧 MANUTENZIONE – DATI OPERATIVI</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="50" customHeight="1">
+      <c r="A24" s="30" t="inlineStr">
+        <is>
+          <t>Numero manutentori</t>
+        </is>
+      </c>
+      <c r="B24" s="43" t="inlineStr">
+        <is>
+          <t>~40 manutentori su Milano. Reperibili fino a mezzanotte</t>
+        </is>
+      </c>
+      <c r="C24" s="44" t="inlineStr">
+        <is>
+          <t>~10 manutentori su Milano. Check-in in presenza fino alle 3 di notte con supplemento. Customer care 24/7</t>
+        </is>
+      </c>
+      <c r="D24" s="45" t="inlineStr">
+        <is>
+          <t>⚠️ Solo 4 manutentori per 500 appartamenti</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="50" customHeight="1">
+      <c r="A25" s="31" t="inlineStr">
+        <is>
+          <t>Ratio manutentori / appartamenti</t>
+        </is>
+      </c>
+      <c r="B25" s="43" t="inlineStr">
+        <is>
+          <t>1:18,75 (40 per 750) → ottimo</t>
+        </is>
+      </c>
+      <c r="C25" s="44" t="inlineStr">
+        <is>
+          <t>1:50 (10 per 500) → buono</t>
+        </is>
+      </c>
+      <c r="D25" s="45" t="inlineStr">
+        <is>
+          <t>⚠️ 1:125 (4 per 500) → molto basso</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="50" customHeight="1">
+      <c r="A26" s="30" t="inlineStr">
+        <is>
+          <t>Reperibilità emergenze notturne</t>
+        </is>
+      </c>
+      <c r="B26" s="43" t="inlineStr">
+        <is>
+          <t>Fino a mezzanotte. Un manutentore di sera</t>
+        </is>
+      </c>
+      <c r="C26" s="44" t="inlineStr">
+        <is>
+          <t>Customer care 24/7. Check-in in presenza fino alle 3 (con supplemento a carico ospite). Manutentori: non specificato H24</t>
+        </is>
+      </c>
+      <c r="D26" s="45" t="inlineStr">
+        <is>
+          <t>⚠️ Non coprono H24. 'Se succede a mezzanotte ancora ancora, ma dopo è difficile'</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="50" customHeight="1">
+      <c r="A27" s="31" t="inlineStr">
+        <is>
+          <t>Costo intervento manutentore</t>
+        </is>
+      </c>
+      <c r="B27" s="43" t="inlineStr">
+        <is>
+          <t>Uscita manutentore INCLUSA nella commissione del 25%. Proprietario paga solo il materiale (notifica prima dell'intervento; autonomia fino a €250)</t>
+        </is>
+      </c>
+      <c r="C27" s="44" t="inlineStr">
+        <is>
+          <t>Nessun diritto di chiamata, nessun costo manodopera. Solo materiale di consumo. Fino a €50 copre Youhosty; €50-100 50/50; &gt;€100 obbligo notifica con preventivo (competitivo)</t>
+        </is>
+      </c>
+      <c r="D27" s="45" t="inlineStr">
+        <is>
+          <t>Autonomia fino a €200+IVA per intervento senza consenso. Costo a carico del cliente. Formula Senza Pensieri copre piccoli interventi (+2,5% commissione)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="50" customHeight="1">
+      <c r="A28" s="30" t="inlineStr">
+        <is>
+          <t>Piccole spese (recupero da ospite)</t>
+        </is>
+      </c>
+      <c r="B28" s="43" t="inlineStr">
+        <is>
+          <t>Su piccole spese difficile da recuperare (confermato dalla chiamata). Gestione principalmente interna</t>
+        </is>
+      </c>
+      <c r="C28" s="44" t="inlineStr">
+        <is>
+          <t>Strutturata: fascia €50/€50-100/€100+ con regole chiare</t>
+        </is>
+      </c>
+      <c r="D28" s="45" t="inlineStr">
+        <is>
+          <t>Su piccole spese 'difficile da recuperare'. Si fanno poco carico di questa responsabilità</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="20" customHeight="1">
+      <c r="A29" s="42" t="inlineStr">
+        <is>
+          <t>🔑 CHECK-IN / CHECK-OUT</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="50" customHeight="1">
+      <c r="A30" s="30" t="inlineStr">
+        <is>
+          <t>Modalità check-in disponibili</t>
+        </is>
+      </c>
+      <c r="B30" s="43" t="inlineStr">
+        <is>
+          <t>1) Key box con codice porta (dura quanto la prenotazione). 2) Reception fisica a Porta Ticinese (costo a carico ospite, variabile per fascia oraria/giorno)</t>
+        </is>
+      </c>
+      <c r="C30" s="44" t="inlineStr">
+        <is>
+          <t>Accoglienza e checkout IN PRESENZA inclusi. Self check-in 24h disponibile. Supplemento per arrivi notturni (fino alle 3 con supplemento)</t>
+        </is>
+      </c>
+      <c r="D30" s="45" t="inlineStr">
+        <is>
+          <t>Remoto via videochiamata (obbligatorio per legge secondo loro). Key box installata (€185+IVA a carico proprietario)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="50" customHeight="1">
+      <c r="A31" s="31" t="inlineStr">
+        <is>
+          <t>Check-out / verifica appartamento</t>
+        </is>
+      </c>
+      <c r="B31" s="43" t="inlineStr">
+        <is>
+          <t>Customer service va a controllare l'appartamento al check-out</t>
+        </is>
+      </c>
+      <c r="C31" s="44" t="inlineStr">
+        <is>
+          <t>Checkout in presenza eseguito dal loro staff</t>
+        </is>
+      </c>
+      <c r="D31" s="45" t="inlineStr">
+        <is>
+          <t>Non specificato in dettaglio</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="50" customHeight="1">
+      <c r="A32" s="30" t="inlineStr">
+        <is>
+          <t>Blocco appartamento – flessibilità</t>
+        </is>
+      </c>
+      <c r="B32" s="43" t="inlineStr">
+        <is>
+          <t>Possibile bloccare anche il giorno prima via app. Non si può aprire/chiudere costantemente: si sceglie una volta</t>
+        </is>
+      </c>
+      <c r="C32" s="44" t="inlineStr">
+        <is>
+          <t>Tramite app, anche giorno su giorno. Meglio coordinare con house manager per All-Inclusive (45 gg/anno)</t>
+        </is>
+      </c>
+      <c r="D32" s="45" t="inlineStr">
+        <is>
+          <t>Max 30 gg/anno, email 15 gg preavviso. Blocco appartamento 'anzichè mandare disdetta': clausola 30gg usata in modo discutibile da un proprietario</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="20" customHeight="1">
+      <c r="A33" s="42" t="inlineStr">
+        <is>
+          <t>🛡️ ASSICURAZIONE (dati da telefonata)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="50" customHeight="1">
+      <c r="A34" s="30" t="inlineStr">
+        <is>
+          <t>Assicurazione proposta</t>
+        </is>
+      </c>
+      <c r="B34" s="43" t="inlineStr">
+        <is>
+          <t>RC terzi obbligatoria (se non la hai, offrono la loro a €30/mese). Copre danni accidentali fino a €250. 'Non ci interessa vendere assicurazioni'</t>
+        </is>
+      </c>
+      <c r="C34" s="44" t="inlineStr">
+        <is>
+          <t>Non fornita. Cliente deve stipulare autonomamente (obbligatoria per legge). Nessuna offerta propria</t>
+        </is>
+      </c>
+      <c r="D34" s="45" t="inlineStr">
+        <is>
+          <t>Offrono assicurazione: 'da vedere se includerla comparandola con quella che già abbiamo'. Dettagli non forniti in chiamata</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="50" customHeight="1">
+      <c r="A35" s="31" t="inlineStr">
+        <is>
+          <t>Copertura danni da ospiti</t>
+        </is>
+      </c>
+      <c r="B35" s="43" t="inlineStr">
+        <is>
+          <t>RC fino a €250 accidentali. Oltre questo limite: dipendente dalla polizza propria del cliente</t>
+        </is>
+      </c>
+      <c r="C35" s="44" t="inlineStr">
+        <is>
+          <t>Nessuna copertura. Solo cauzione piattaforma OTA (variabile)</t>
+        </is>
+      </c>
+      <c r="D35" s="45" t="inlineStr">
+        <is>
+          <t>Non specificato. Responsabilità danni ospiti esonerate contrattualmente (art. 10.1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="20" customHeight="1">
+      <c r="A36" s="42" t="inlineStr">
+        <is>
+          <t>📞 REFERENTE DEDICATO E COMUNICAZIONE</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="50" customHeight="1">
+      <c r="A37" s="30" t="inlineStr">
+        <is>
+          <t>Referente per il proprietario</t>
+        </is>
+      </c>
+      <c r="B37" s="43" t="inlineStr">
+        <is>
+          <t>Property service: 2 persone dedicate (lato operativo + amministrativo). Separato: amministrativo per tasse/fiscale</t>
+        </is>
+      </c>
+      <c r="C37" s="44" t="inlineStr">
+        <is>
+          <t>House manager dedicato: ~20 appartamenti a testa, tutti senior. Interlocutore unico stabile</t>
+        </is>
+      </c>
+      <c r="D37" s="45" t="inlineStr">
+        <is>
+          <t>Gruppo WhatsApp con i proprietari (comunicazione di gruppo, non dedicata)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="50" customHeight="1">
+      <c r="A38" s="31" t="inlineStr">
+        <is>
+          <t>Canali di comunicazione</t>
+        </is>
+      </c>
+      <c r="B38" s="43" t="inlineStr">
+        <is>
+          <t>Email (poi chiamata). WhatsApp possibile. Normalmente parlano poco con il proprietario ('funzioniamo da 14 anni')</t>
+        </is>
+      </c>
+      <c r="C38" s="44" t="inlineStr">
+        <is>
+          <t>WhatsApp + email aziendale + disponibilità telefonica</t>
+        </is>
+      </c>
+      <c r="D38" s="45" t="inlineStr">
+        <is>
+          <t>Gruppo WhatsApp condiviso tra proprietari</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="50" customHeight="1">
+      <c r="A39" s="30" t="inlineStr">
+        <is>
+          <t>Qualità supporto dichiarata</t>
+        </is>
+      </c>
+      <c r="B39" s="43" t="inlineStr">
+        <is>
+          <t>'Funzioniamo da 14 anni molto bene, normalmente non parliamo spesso con il proprietario'</t>
+        </is>
+      </c>
+      <c r="C39" s="44" t="inlineStr">
+        <is>
+          <t>Customer care 24/7. Differenziatore dichiarato: velocità nel risolvere problemi + trasparenza app</t>
+        </is>
+      </c>
+      <c r="D39" s="45" t="inlineStr">
+        <is>
+          <t>Differenziatori dichiarati: vicinanza coi proprietari, velocità problemi, prenotazioni dirette corporate. In pratica: solo 4 manutentori</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="20" customHeight="1">
+      <c r="A40" s="42" t="inlineStr">
+        <is>
+          <t>⚠️ VINCOLI CONTRATTUALI – DATI REALI DA TELEFONATA</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="50" customHeight="1">
+      <c r="A41" s="30" t="inlineStr">
+        <is>
+          <t>Vincolo reale di uscita anticipata</t>
+        </is>
+      </c>
+      <c r="B41" s="43" t="inlineStr">
+        <is>
+          <t>Dal 2° anno: disdetta 90 gg prima oppure penale €20/giorno (inclusi sabato e domenica)</t>
+        </is>
+      </c>
+      <c r="C41" s="44" t="inlineStr">
+        <is>
+          <t>All-Inclusive: solo forza maggiore o penale €50/gg + €470 pratiche/disinstallazione</t>
+        </is>
+      </c>
+      <c r="D41" s="45" t="inlineStr">
+        <is>
+          <t>⚠️ ATTENZIONE: in telefonata dichiarano vincolo di 1 ANNO per rescissione. Il contratto scritto non lo esplicita chiaramente. Verificare prima della firma</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="50" customHeight="1">
+      <c r="A42" s="31" t="inlineStr">
+        <is>
+          <t>Clausola uso 30 giorni – applicazione reale</t>
+        </is>
+      </c>
+      <c r="B42" s="43" t="inlineStr">
+        <is>
+          <t>Applicazione standard: blocco via app</t>
+        </is>
+      </c>
+      <c r="C42" s="44" t="inlineStr">
+        <is>
+          <t>45 gg/anno, blocco via app coordinato con house manager</t>
+        </is>
+      </c>
+      <c r="D42" s="45" t="inlineStr">
+        <is>
+          <t>⚠️ Caso segnalato: un proprietario invece di disdire il contratto ha 'bloccato l'appartamento per 30 giorni e poi l'ha venduto' usando la clausola in modo improprio → clausola interpretata da Easylife in modo restrittivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="50" customHeight="1">
+      <c r="A43" s="30" t="inlineStr">
+        <is>
+          <t>Obblighi in caso di vendita immobile</t>
+        </is>
+      </c>
+      <c r="B43" s="43" t="inlineStr">
+        <is>
+          <t>Non menzionato in telefonata</t>
+        </is>
+      </c>
+      <c r="C43" s="44" t="inlineStr">
+        <is>
+          <t>Mandato automatico a Youhosty per pubblicazione annuncio (contratto art. 3)</t>
+        </is>
+      </c>
+      <c r="D43" s="45" t="inlineStr">
+        <is>
+          <t>2% commissione alla loro agenzia partner (obbligatorio per contratto). Loro fanno anche vendita</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="50" customHeight="1">
+      <c r="A44" s="31" t="inlineStr">
+        <is>
+          <t>Limite persone fisiche</t>
+        </is>
+      </c>
+      <c r="B44" s="43" t="inlineStr">
+        <is>
+          <t>Non menzionato</t>
+        </is>
+      </c>
+      <c r="C44" s="44" t="inlineStr">
+        <is>
+          <t>Non menzionato</t>
+        </is>
+      </c>
+      <c r="D44" s="45" t="inlineStr">
+        <is>
+          <t>Max 2 immobili a testa come persona fisica. Dal 3° (fino a 6 per persona fisica) serve società</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="50" customHeight="1">
+      <c r="A45" s="30" t="inlineStr">
+        <is>
+          <t>Doppio canale (breve + medio termine)</t>
+        </is>
+      </c>
+      <c r="B45" s="43" t="inlineStr">
+        <is>
+          <t>Entrambi i canali opzionali. Si può partire con entrambi e chiuderne uno. Canone medio termine uguale ogni mese (no stagionalità)</t>
+        </is>
+      </c>
+      <c r="C45" s="44" t="inlineStr">
+        <is>
+          <t>Suggeriscono alternanza stagionale (breve feb-lug; medio/lungo ago-feb). 0% commissione medio termine (All-Inclusive)</t>
+        </is>
+      </c>
+      <c r="D45" s="45" t="inlineStr">
+        <is>
+          <t>Non discusso in dettaglio</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="20" customHeight="1">
+      <c r="A46" s="42" t="inlineStr">
+        <is>
+          <t>🏠 REQUISITI IMMOBILE (da telefonata)</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="50" customHeight="1">
+      <c r="A47" s="30" t="inlineStr">
+        <is>
+          <t>Requisiti obbligatori</t>
+        </is>
+      </c>
+      <c r="B47" s="43" t="inlineStr">
+        <is>
+          <t>Aria condizionata obbligatoria. Lavatrice. No seminterrati. No sanit-rit. Piante: non gestite. APE richiesta. Piatti, posate, bicchieri, cuscini, estintore 6kg</t>
+        </is>
+      </c>
+      <c r="C47" s="44" t="inlineStr">
+        <is>
+          <t>Re-registrazione CAV obbligatoria. Estintori, CO detector, kit emergenza (€219-259). Pulizie iniziali/finali (o fai da te). Aspirapolvere (opzionale)</t>
+        </is>
+      </c>
+      <c r="D47" s="45" t="inlineStr">
+        <is>
+          <t>Standard Allegato A (non dettagliato in chiamata). Dotazioni base obbligatorie. Aria condizionata non menzionata esplicitamente</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="50" customHeight="1">
+      <c r="A48" s="31" t="inlineStr">
+        <is>
+          <t>Valutazione preliminare</t>
+        </is>
+      </c>
+      <c r="B48" s="43" t="inlineStr">
+        <is>
+          <t>'Prima ho bisogno di vedere l'appartamento' (le analisi reddituali si fanno con sopralluogo)</t>
+        </is>
+      </c>
+      <c r="C48" s="44" t="inlineStr">
+        <is>
+          <t>Non menzionato</t>
+        </is>
+      </c>
+      <c r="D48" s="45" t="inlineStr">
+        <is>
+          <t>Non menzionato</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="50" customHeight="1">
+      <c r="A49" s="30" t="inlineStr">
+        <is>
+          <t>Lenzuola / biancheria</t>
+        </is>
+      </c>
+      <c r="B49" s="43" t="inlineStr">
+        <is>
+          <t>NON fornite da Italianway (vengono dall'azienda di pulizie partner). Incluse nella gestione</t>
+        </is>
+      </c>
+      <c r="C49" s="44" t="inlineStr">
+        <is>
+          <t>Non menzionate</t>
+        </is>
+      </c>
+      <c r="D49" s="45" t="inlineStr">
+        <is>
+          <t>Da contratto addebitate all'ospite</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="12">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A23:D23"/>
+    <mergeCell ref="A9:D9"/>
+    <mergeCell ref="A40:D40"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="A20:D20"/>
+    <mergeCell ref="A29:D29"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A33:D33"/>
+    <mergeCell ref="A46:D46"/>
+    <mergeCell ref="A36:D36"/>
+    <mergeCell ref="A14:D14"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6313,9 +7606,9 @@
           <t>Trasparenza costi</t>
         </is>
       </c>
-      <c r="B5" s="21" t="inlineStr">
-        <is>
-          <t>4</t>
+      <c r="B5" s="46" t="inlineStr">
+        <is>
+          <t>3</t>
         </is>
       </c>
       <c r="C5" s="35" t="inlineStr">
@@ -6328,11 +7621,11 @@
           <t>3</t>
         </is>
       </c>
-      <c r="E5" s="10" t="inlineStr">
-        <is>
-          <t>Costi abbastanza espliciti nel contratto
-Youhosty: prezzi espliciti ma molti componenti separati (OTA, mensile, chiusura) rendono difficile il calcolo del costo totale
-Easylife: contratto chiaro su commissioni e costi avvio, ma OTA non nominate e alcuni costi accessori 'da trattenere alla prima contabilità utile' non quantificati</t>
+      <c r="E5" s="47" t="inlineStr">
+        <is>
+          <t>Italianway: ⚠️ worst case 22% (Italianway) + 18% (piattaforma) + IVA + cedolare secca = proprietario incassa ~metà prezzo di uscita. Base commissionale diversa da Youhosty
+Youhosty: 16,5% + OTA (a carico cliente) + €26,90/mese + €470 costi uscita. Molti componenti separati
+Easylife: 25%+IVA sul netto OTA/pulizie (OTA pagata dall'ospite). Formula Senza Pensieri +2,5%. Vincolo 1 anno non esplicitato nel contratto</t>
         </is>
       </c>
     </row>
@@ -6342,7 +7635,7 @@
           <t>Flessibilità contrattuale</t>
         </is>
       </c>
-      <c r="B6" s="21" t="inlineStr">
+      <c r="B6" s="46" t="inlineStr">
         <is>
           <t>2</t>
         </is>
@@ -6354,14 +7647,14 @@
       </c>
       <c r="D6" s="37" t="inlineStr">
         <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="E6" s="6" t="inlineStr">
-        <is>
-          <t>Esclusiva + 3 mesi preavviso + rinnovo tacito = poco flessibile
-All-Inclusive 24 mesi, recesso solo forza maggiore, pratiche chiusura €470, penale accesso €50 → il meno flessibile
-Easylife: 18 mesi (migliore di Youhosty 24 mesi, peggiore di Italianway 12 mesi). Nessun recesso anticipato per cliente. PM può uscire con 30 gg.</t>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E6" s="48" t="inlineStr">
+        <is>
+          <t>Italianway: 1° anno blindato; dal 2° anno disdetta 90 gg o €20/gg (sab+dom inclusi) → rigido ma standard
+Youhosty: 24 mesi, recesso anticipato praticamente impossibile, €470 costi uscita → il meno flessibile
+Easylife: ⚠️ in telefonata dichiarano 'vincolo di 1 anno' non esplicitato nel contratto. Penale accesso 100% incassi mese → verificare prima di firmare</t>
         </is>
       </c>
     </row>
@@ -6371,26 +7664,26 @@
           <t>Qualità servizi operativi</t>
         </is>
       </c>
-      <c r="B7" s="21" t="inlineStr">
-        <is>
-          <t>4</t>
+      <c r="B7" s="46" t="inlineStr">
+        <is>
+          <t>5</t>
         </is>
       </c>
       <c r="C7" s="35" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="D7" s="37" t="inlineStr">
         <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="E7" s="10" t="inlineStr">
-        <is>
-          <t>Check-in, pulizie, burocrazia gestiti; qualità PM locale da verificare
-Self check-in automatizzato, gestione completa, multilingual; gestione diretta (non franchising) → qualità più uniforme
-Easylife: gestione completa con partner, check-in automatizzato, portale proprietario Easylife House. Formula Senza Pensieri per manutenzioni.</t>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E7" s="47" t="inlineStr">
+        <is>
+          <t>Italianway: 40 manutentori a Milano (1:18), costo uscita incluso nella commissione, fino a mezzanotte → ottimo
+Youhosty: 10 manutentori (1:50), customer care 24/7, house manager dedicato 20 app/pers., checkout in presenza, cedolare secca gestita → eccellente
+Easylife: ⚠️ solo 4 manutentori per 500 appartamenti (1:125), non H24 dopo mezzanotte → insufficiente</t>
         </is>
       </c>
     </row>
@@ -6400,26 +7693,26 @@
           <t>Tecnologia / piattaforma</t>
         </is>
       </c>
-      <c r="B8" s="21" t="inlineStr">
+      <c r="B8" s="46" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
       <c r="C8" s="35" t="inlineStr">
         <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D8" s="37" t="inlineStr">
+        <is>
           <t>3</t>
         </is>
       </c>
-      <c r="D8" s="37" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="E8" s="6" t="inlineStr">
-        <is>
-          <t>KALISI: real-time, algoritmo Revenue Management
-App/sito proprietario con revenue management in outsourcing; meno descritto di KALISI ma funzionale
-Easylife: portale web per controllo + Easylife House (OTA proprietaria). Funzionalità non dettagliate nel contratto.</t>
+      <c r="E8" s="48" t="inlineStr">
+        <is>
+          <t>Italianway: KALISI (real-time) + app prenotazioni + team revenue settimanale. Software proprietario non nominato
+Youhosty: algoritmo pricing proprietario sviluppato con PriceLabs (aggiornamento quotidiano) + app real-time + 20 canali OTA + 20% dal canale proprio
+Easylife: 'Be on Pricing' (aggiornamento quotidiano) + portale web + Easylife House. Non su GDS (limite per clientela corporate)</t>
         </is>
       </c>
     </row>
@@ -6458,9 +7751,9 @@
           <t>Copertura assicurativa</t>
         </is>
       </c>
-      <c r="B10" s="21" t="inlineStr">
-        <is>
-          <t>3</t>
+      <c r="B10" s="46" t="inlineStr">
+        <is>
+          <t>2</t>
         </is>
       </c>
       <c r="C10" s="35" t="inlineStr">
@@ -6470,14 +7763,14 @@
       </c>
       <c r="D10" s="37" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E10" s="6" t="inlineStr">
-        <is>
-          <t>RC €1M ottima; massimali incendio/furto nella media
-Nessuna polizza collettiva: solo cauzione piattaforma e consiglio di stipulare RC propria → rischio massimo per il proprietario
-Easylife: nessuna polizza collettiva. Il cliente deve stipulare tutto autonomamente (art. 10.3). Responsabilità danni ospiti esonerate esplicitamente.</t>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E10" s="48" t="inlineStr">
+        <is>
+          <t>Italianway: RC terzi obbligatoria; se non hai polizza propria, offrono la loro a €30/mese (danni accidentali max €250 → copertura molto limitata)
+Youhosty: nessuna polizza collettiva. Cliente completamente autonomo → rischio massimo
+Easylife: offrono assicurazione propria (dettagli non forniti). Da confrontare con polizza eventualmente già in possesso</t>
         </is>
       </c>
     </row>
@@ -6516,26 +7809,26 @@
           <t>Reputazione / presenza sul mercato</t>
         </is>
       </c>
-      <c r="B12" s="21" t="inlineStr">
+      <c r="B12" s="46" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C12" s="35" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="C12" s="35" t="inlineStr">
+      <c r="D12" s="37" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="D12" s="37" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="E12" s="6" t="inlineStr">
-        <is>
-          <t>Brand nazionale; franchising diffuso; dal 2014
-Brand riconoscibile a Milano; meno capillare di Italianway a livello nazionale
-Easylife: S.p.A. con sede a Milano, portale proprietario. Meno informazioni pubbliche rispetto a Italianway.</t>
+      <c r="E12" s="48" t="inlineStr">
+        <is>
+          <t>Italianway: 750 app attivi a Milano, 7500 partner franchising, 160 dipendenti, 14 anni → leader di mercato
+Youhosty: 10 anni, Confcommercio, portfolio €200M, clientela corporate strutturata (Bottega Veneta, Mediolanum) → molto solido
+Easylife: 500 app ma solo entro 2a circonvallazione Milano; anni di attività non dichiarati → base più limitata</t>
         </is>
       </c>
     </row>
@@ -6603,26 +7896,26 @@
           <t>Supporto al proprietario</t>
         </is>
       </c>
-      <c r="B15" s="21" t="inlineStr">
-        <is>
-          <t>3</t>
+      <c r="B15" s="46" t="inlineStr">
+        <is>
+          <t>4</t>
         </is>
       </c>
       <c r="C15" s="35" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="D15" s="37" t="inlineStr">
         <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="E15" s="10" t="inlineStr">
-        <is>
-          <t>PM locale affiliato; qualità variabile per zona
-Gestione diretta non franchise → interlocutore unico e stabile; abbonamento mensile con check-up periodico
-Easylife: portale web, segnalazione danni, CU annuale. Penale accesso non autorizzato molto severa (100% incassi mese successivo).</t>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E15" s="47" t="inlineStr">
+        <is>
+          <t>Italianway: 2 persone property service (operativo + amministrativo), email + whatsapp, 14 anni di rodaggio. Non parlano spesso ma risolvono
+Youhosty: house manager senior dedicato (~20 app/persona), WhatsApp + email + telefono, 24/7 customer care → migliore supporto del gruppo
+Easylife: ⚠️ solo gruppo WhatsApp condiviso tra proprietari (non personalizzato). 4 manutentori per 500 app.</t>
         </is>
       </c>
     </row>

</xml_diff>